<commit_message>
Log this week's outreach run: 25 Apollo leads, 6 email drafts, bounce/LinkedIn cadence
- Reconstructed 25 category-A (sales/presales) prospects pulled by an earlier
  process today that were never written to the tracker, including 15 people
  who were live-emailed (not drafted) outside this automation.
- Marked 3 bounced sends (Mehdi Rabia, Adrien Gagniere, Paulina Nordgren) as
  Bounced=Y and pivoted their cadence to LinkedIn since email is dead.
- Drafted Email 1 (Gmail draft, not sent) for 6 net-new contacts with valid
  emails; queued LinkedIn connection-request text for 7 contacts (4 net-new
  without email + the 3 bounced) for manual send.
- Advanced Stage/Next Action/Next Action Date per the template cadence for
  all 13 touched rows this run.
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -660,554 +660,1798 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n"/>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Subhadeep Ghosh</t>
+        </is>
+      </c>
       <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="6" t="n"/>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/subhadeep-ghosh-221b007</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>LinkedIn Connection Requested</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="n">
+        <v>46246</v>
+      </c>
       <c r="H3" s="5">
         <f>IF(G3="","",TODAY()-G3)</f>
         <v/>
       </c>
-      <c r="I3" s="5" t="n"/>
-      <c r="J3" s="6" t="n"/>
-      <c r="K3" s="5" t="n"/>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Send LinkedIn Message 1 (if connected)</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="n">
+        <v>46248</v>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L3" s="6" t="n"/>
-      <c r="M3" s="5" t="n"/>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N3" s="6" t="n"/>
-      <c r="O3" s="5" t="n"/>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P3" s="6" t="n"/>
-      <c r="Q3" s="5" t="n"/>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>No email available via Apollo (Basic Trial plan blocks enrichment) — LinkedIn-only outreach. Hook: Saw your Presales Solutions Consultant role at Tata Consultancy Services</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="6" t="n"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Anas Aljarrah</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>anas.aljarrah@motorolasolutions.com</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/anas-aljarrah</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
       <c r="H4" s="5">
         <f>IF(G4="","",TODAY()-G4)</f>
         <v/>
       </c>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="6" t="n"/>
-      <c r="K4" s="5" t="n"/>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L4" s="6" t="n"/>
-      <c r="M4" s="5" t="n"/>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N4" s="6" t="n"/>
-      <c r="O4" s="5" t="n"/>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P4" s="6" t="n"/>
-      <c r="Q4" s="5" t="n"/>
+      <c r="Q4" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n"/>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="6" t="n"/>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Hugo Annabi</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>hugo@edko.io</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/hugo-annabi</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
       <c r="H5" s="5">
         <f>IF(G5="","",TODAY()-G5)</f>
         <v/>
       </c>
-      <c r="I5" s="5" t="n"/>
-      <c r="J5" s="6" t="n"/>
-      <c r="K5" s="5" t="n"/>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L5" s="6" t="n"/>
-      <c r="M5" s="5" t="n"/>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N5" s="6" t="n"/>
-      <c r="O5" s="5" t="n"/>
+      <c r="O5" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P5" s="6" t="n"/>
-      <c r="Q5" s="5" t="n"/>
+      <c r="Q5" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="6" t="n"/>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Bedirhan Akay</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>bedirhan.akay@apollo.eco</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/bedirhan-a-614b09105</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
       <c r="H6" s="5">
         <f>IF(G6="","",TODAY()-G6)</f>
         <v/>
       </c>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="6" t="n"/>
-      <c r="K6" s="5" t="n"/>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L6" s="6" t="n"/>
-      <c r="M6" s="5" t="n"/>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N6" s="6" t="n"/>
-      <c r="O6" s="5" t="n"/>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P6" s="6" t="n"/>
-      <c r="Q6" s="5" t="n"/>
+      <c r="Q6" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="6" t="n"/>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Sakshi Maheshwari</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>sakmahes@cisco.com</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/sakshimaheshwari19</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
       <c r="H7" s="5">
         <f>IF(G7="","",TODAY()-G7)</f>
         <v/>
       </c>
-      <c r="I7" s="5" t="n"/>
-      <c r="J7" s="6" t="n"/>
-      <c r="K7" s="5" t="n"/>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L7" s="6" t="n"/>
-      <c r="M7" s="5" t="n"/>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N7" s="6" t="n"/>
-      <c r="O7" s="5" t="n"/>
+      <c r="O7" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P7" s="6" t="n"/>
-      <c r="Q7" s="5" t="n"/>
+      <c r="Q7" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="6" t="n"/>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Mehdi Rabia</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>mehdi.rabia@flatpay.com</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/mehdi-rabia-346189389</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Bounced - LinkedIn Connection Requested</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>46246</v>
+      </c>
       <c r="H8" s="5">
         <f>IF(G8="","",TODAY()-G8)</f>
         <v/>
       </c>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="6" t="n"/>
-      <c r="K8" s="5" t="n"/>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Send LinkedIn Message 1 (if connected)</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>46248</v>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L8" s="6" t="n"/>
-      <c r="M8" s="5" t="n"/>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N8" s="6" t="n"/>
-      <c r="O8" s="5" t="n"/>
-      <c r="P8" s="6" t="n"/>
-      <c r="Q8" s="5" t="n"/>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P8" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="Q8" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 sent 2026-08-12, bounced same day (Address not found - the address couldn't be found, or is unable to receive mail.). Retroactively logged from Gmail — see run digest. Pivoting to LinkedIn since LinkedIn URL available.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="6" t="n"/>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Nael Ayadi</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>nael.ayadi@papernest.com</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/nael-ayadi-sports-business-consulting</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
       <c r="H9" s="5">
         <f>IF(G9="","",TODAY()-G9)</f>
         <v/>
       </c>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="6" t="n"/>
-      <c r="K9" s="5" t="n"/>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L9" s="6" t="n"/>
-      <c r="M9" s="5" t="n"/>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N9" s="6" t="n"/>
-      <c r="O9" s="5" t="n"/>
+      <c r="O9" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P9" s="6" t="n"/>
-      <c r="Q9" s="5" t="n"/>
+      <c r="Q9" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="6" t="n"/>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Joel Masats</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>joel.masats@driverevel.com</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/joel-masats-81a035259</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Drafted</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>46246</v>
+      </c>
       <c r="H10" s="5">
         <f>IF(G10="","",TODAY()-G10)</f>
         <v/>
       </c>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="6" t="n"/>
-      <c r="K10" s="5" t="n"/>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>46252</v>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L10" s="6" t="n"/>
-      <c r="M10" s="5" t="n"/>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N10" s="6" t="n"/>
-      <c r="O10" s="5" t="n"/>
+      <c r="O10" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P10" s="6" t="n"/>
-      <c r="Q10" s="5" t="n"/>
+      <c r="Q10" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Sales Business Development Representative role at REVEL | Renting de Coches</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="6" t="n"/>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Rohit Saha</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>rohit@ramd.am</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/rohittsaha</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
       <c r="H11" s="5">
         <f>IF(G11="","",TODAY()-G11)</f>
         <v/>
       </c>
-      <c r="I11" s="5" t="n"/>
-      <c r="J11" s="6" t="n"/>
-      <c r="K11" s="5" t="n"/>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L11" s="6" t="n"/>
-      <c r="M11" s="5" t="n"/>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N11" s="6" t="n"/>
-      <c r="O11" s="5" t="n"/>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P11" s="6" t="n"/>
-      <c r="Q11" s="5" t="n"/>
+      <c r="Q11" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="6" t="n"/>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Suvendu Sutar</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>suvendu.sutar@wipro.com</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/suvendu-sutar-1b3360178</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
       <c r="H12" s="5">
         <f>IF(G12="","",TODAY()-G12)</f>
         <v/>
       </c>
-      <c r="I12" s="5" t="n"/>
-      <c r="J12" s="6" t="n"/>
-      <c r="K12" s="5" t="n"/>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L12" s="6" t="n"/>
-      <c r="M12" s="5" t="n"/>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N12" s="6" t="n"/>
-      <c r="O12" s="5" t="n"/>
+      <c r="O12" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P12" s="6" t="n"/>
-      <c r="Q12" s="5" t="n"/>
+      <c r="Q12" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="6" t="n"/>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Adrien Gagniere</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>adrien@in-leed.com</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/adrien-gagniere-902996263</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Bounced - LinkedIn Connection Requested</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>46246</v>
+      </c>
       <c r="H13" s="5">
         <f>IF(G13="","",TODAY()-G13)</f>
         <v/>
       </c>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="6" t="n"/>
-      <c r="K13" s="5" t="n"/>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>Send LinkedIn Message 1 (if connected)</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>46248</v>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L13" s="6" t="n"/>
-      <c r="M13" s="5" t="n"/>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N13" s="6" t="n"/>
-      <c r="O13" s="5" t="n"/>
-      <c r="P13" s="6" t="n"/>
-      <c r="Q13" s="5" t="n"/>
+      <c r="O13" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P13" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 sent 2026-08-12, bounced same day (550 No Such User (address not found)). Retroactively logged from Gmail — see run digest. Pivoting to LinkedIn since LinkedIn URL available.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="n"/>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="6" t="n"/>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Boris-Mihail Todorov</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>boris.todorov@paynetics.digital</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/boris-mihail-todorov</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
       <c r="H14" s="5">
         <f>IF(G14="","",TODAY()-G14)</f>
         <v/>
       </c>
-      <c r="I14" s="5" t="n"/>
-      <c r="J14" s="6" t="n"/>
-      <c r="K14" s="5" t="n"/>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L14" s="6" t="n"/>
-      <c r="M14" s="5" t="n"/>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N14" s="6" t="n"/>
-      <c r="O14" s="5" t="n"/>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P14" s="6" t="n"/>
-      <c r="Q14" s="5" t="n"/>
+      <c r="Q14" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="6" t="n"/>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Souhaila Bouquoyoue</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>souhaila.bouquoyoue@berger-levrault.com</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/souhaila-bouquoyoue</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
       <c r="H15" s="5">
         <f>IF(G15="","",TODAY()-G15)</f>
         <v/>
       </c>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="6" t="n"/>
-      <c r="K15" s="5" t="n"/>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L15" s="6" t="n"/>
-      <c r="M15" s="5" t="n"/>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N15" s="6" t="n"/>
-      <c r="O15" s="5" t="n"/>
+      <c r="O15" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P15" s="6" t="n"/>
-      <c r="Q15" s="5" t="n"/>
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="n"/>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="6" t="n"/>
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Paulina Nordgren</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>paulina.nordgren@wolterskluwer.com</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/paulinanordgren</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Bounced - LinkedIn Connection Requested</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>46246</v>
+      </c>
       <c r="H16" s="5">
         <f>IF(G16="","",TODAY()-G16)</f>
         <v/>
       </c>
-      <c r="I16" s="5" t="n"/>
-      <c r="J16" s="6" t="n"/>
-      <c r="K16" s="5" t="n"/>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Send LinkedIn Message 1 (if connected)</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="n">
+        <v>46248</v>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L16" s="6" t="n"/>
-      <c r="M16" s="5" t="n"/>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N16" s="6" t="n"/>
-      <c r="O16" s="5" t="n"/>
-      <c r="P16" s="6" t="n"/>
-      <c r="Q16" s="5" t="n"/>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P16" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 sent 2026-08-12, bounced same day (550 5.7.1 Service unavailable / message blocked). Retroactively logged from Gmail — see run digest. Pivoting to LinkedIn since LinkedIn URL available.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="6" t="n"/>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Tanishq Munjal</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>tanishq@speargrowth.com</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/tanishq-munjal</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Drafted</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>46246</v>
+      </c>
       <c r="H17" s="5">
         <f>IF(G17="","",TODAY()-G17)</f>
         <v/>
       </c>
-      <c r="I17" s="5" t="n"/>
-      <c r="J17" s="6" t="n"/>
-      <c r="K17" s="5" t="n"/>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="n">
+        <v>46252</v>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L17" s="6" t="n"/>
-      <c r="M17" s="5" t="n"/>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N17" s="6" t="n"/>
-      <c r="O17" s="5" t="n"/>
+      <c r="O17" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P17" s="6" t="n"/>
-      <c r="Q17" s="5" t="n"/>
+      <c r="Q17" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Business Development Representative &amp; Account Executive role at Spear Growth</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n"/>
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="6" t="n"/>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Siddharth Srivastava</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>siddharth.srivastava@o9solutions.com</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/siddharth-srivastava-1b32b3202</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Drafted</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>46246</v>
+      </c>
       <c r="H18" s="5">
         <f>IF(G18="","",TODAY()-G18)</f>
         <v/>
       </c>
-      <c r="I18" s="5" t="n"/>
-      <c r="J18" s="6" t="n"/>
-      <c r="K18" s="5" t="n"/>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="n">
+        <v>46252</v>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L18" s="6" t="n"/>
-      <c r="M18" s="5" t="n"/>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N18" s="6" t="n"/>
-      <c r="O18" s="5" t="n"/>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P18" s="6" t="n"/>
-      <c r="Q18" s="5" t="n"/>
+      <c r="Q18" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Presales Solutions Consultant role at o9 Solutions, Inc.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="n"/>
-      <c r="B19" s="5" t="n"/>
-      <c r="C19" s="5" t="n"/>
-      <c r="D19" s="5" t="n"/>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5" t="n"/>
-      <c r="G19" s="6" t="n"/>
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Katie Collopy</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>katie@maverickmedia.eu</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/katie-collopy-37a0191a1</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Drafted</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>46246</v>
+      </c>
       <c r="H19" s="5">
         <f>IF(G19="","",TODAY()-G19)</f>
         <v/>
       </c>
-      <c r="I19" s="5" t="n"/>
-      <c r="J19" s="6" t="n"/>
-      <c r="K19" s="5" t="n"/>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="n">
+        <v>46252</v>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L19" s="6" t="n"/>
-      <c r="M19" s="5" t="n"/>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N19" s="6" t="n"/>
-      <c r="O19" s="5" t="n"/>
+      <c r="O19" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P19" s="6" t="n"/>
-      <c r="Q19" s="5" t="n"/>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Sales and Business Development Representative role at Maverick Media</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="n"/>
-      <c r="B20" s="5" t="n"/>
-      <c r="C20" s="5" t="n"/>
-      <c r="D20" s="5" t="n"/>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="5" t="n"/>
-      <c r="G20" s="6" t="n"/>
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Ines Diallo</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>ines.diallo@infinit.com</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/in%c3%a8s-diallo-918447172</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
       <c r="H20" s="5">
         <f>IF(G20="","",TODAY()-G20)</f>
         <v/>
       </c>
-      <c r="I20" s="5" t="n"/>
-      <c r="J20" s="6" t="n"/>
-      <c r="K20" s="5" t="n"/>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L20" s="6" t="n"/>
-      <c r="M20" s="5" t="n"/>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N20" s="6" t="n"/>
-      <c r="O20" s="5" t="n"/>
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P20" s="6" t="n"/>
-      <c r="Q20" s="5" t="n"/>
+      <c r="Q20" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="n"/>
-      <c r="B21" s="5" t="n"/>
-      <c r="C21" s="5" t="n"/>
-      <c r="D21" s="5" t="n"/>
-      <c r="E21" s="5" t="n"/>
-      <c r="F21" s="5" t="n"/>
-      <c r="G21" s="6" t="n"/>
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Lin Ye</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>lin.ye@siemens.com</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/lin-ye-171224178</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Drafted</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>46246</v>
+      </c>
       <c r="H21" s="5">
         <f>IF(G21="","",TODAY()-G21)</f>
         <v/>
       </c>
-      <c r="I21" s="5" t="n"/>
-      <c r="J21" s="6" t="n"/>
-      <c r="K21" s="5" t="n"/>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="n">
+        <v>46252</v>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L21" s="6" t="n"/>
-      <c r="M21" s="5" t="n"/>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N21" s="6" t="n"/>
-      <c r="O21" s="5" t="n"/>
+      <c r="O21" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P21" s="6" t="n"/>
-      <c r="Q21" s="5" t="n"/>
+      <c r="Q21" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Presales Solutions Consultant role at Siemens Digital Industries Software</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="n"/>
-      <c r="B22" s="5" t="n"/>
-      <c r="C22" s="5" t="n"/>
-      <c r="D22" s="5" t="n"/>
-      <c r="E22" s="5" t="n"/>
-      <c r="F22" s="5" t="n"/>
-      <c r="G22" s="6" t="n"/>
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Samuel Sebban</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>samuel.sebban@pytheascapital.com</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/samuel-sebban-1b1054231</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
       <c r="H22" s="5">
         <f>IF(G22="","",TODAY()-G22)</f>
         <v/>
       </c>
-      <c r="I22" s="5" t="n"/>
-      <c r="J22" s="6" t="n"/>
-      <c r="K22" s="5" t="n"/>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L22" s="6" t="n"/>
-      <c r="M22" s="5" t="n"/>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N22" s="6" t="n"/>
-      <c r="O22" s="5" t="n"/>
+      <c r="O22" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P22" s="6" t="n"/>
-      <c r="Q22" s="5" t="n"/>
+      <c r="Q22" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="n"/>
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Come Belmokadem</t>
+        </is>
+      </c>
       <c r="B23" s="5" t="n"/>
-      <c r="C23" s="5" t="n"/>
-      <c r="D23" s="5" t="n"/>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="5" t="n"/>
-      <c r="G23" s="6" t="n"/>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/c%c3%b4me-melis-belmokadem-390094344</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>LinkedIn Connection Requested</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>46246</v>
+      </c>
       <c r="H23" s="5">
         <f>IF(G23="","",TODAY()-G23)</f>
         <v/>
       </c>
-      <c r="I23" s="5" t="n"/>
-      <c r="J23" s="6" t="n"/>
-      <c r="K23" s="5" t="n"/>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>Send LinkedIn Message 1 (if connected)</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="n">
+        <v>46248</v>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L23" s="6" t="n"/>
-      <c r="M23" s="5" t="n"/>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N23" s="6" t="n"/>
-      <c r="O23" s="5" t="n"/>
+      <c r="O23" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P23" s="6" t="n"/>
-      <c r="Q23" s="5" t="n"/>
+      <c r="Q23" s="5" t="inlineStr">
+        <is>
+          <t>No email available via Apollo (Basic Trial plan blocks enrichment) — LinkedIn-only outreach. Hook: Saw your Sales Business Development Representative role at Luxiris</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="n"/>
-      <c r="B24" s="5" t="n"/>
-      <c r="C24" s="5" t="n"/>
-      <c r="D24" s="5" t="n"/>
-      <c r="E24" s="5" t="n"/>
-      <c r="F24" s="5" t="n"/>
-      <c r="G24" s="6" t="n"/>
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Franco Rizzi</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>franco.rizzi@siemens.com</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/frizzi</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Drafted</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>46246</v>
+      </c>
       <c r="H24" s="5">
         <f>IF(G24="","",TODAY()-G24)</f>
         <v/>
       </c>
-      <c r="I24" s="5" t="n"/>
-      <c r="J24" s="6" t="n"/>
-      <c r="K24" s="5" t="n"/>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="n">
+        <v>46252</v>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L24" s="6" t="n"/>
-      <c r="M24" s="5" t="n"/>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N24" s="6" t="n"/>
-      <c r="O24" s="5" t="n"/>
+      <c r="O24" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P24" s="6" t="n"/>
-      <c r="Q24" s="5" t="n"/>
+      <c r="Q24" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Presales Solutions Consultant role at Siemens Digital Industries Software</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="n"/>
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Dagmar Ilisson</t>
+        </is>
+      </c>
       <c r="B25" s="5" t="n"/>
-      <c r="C25" s="5" t="n"/>
-      <c r="D25" s="5" t="n"/>
-      <c r="E25" s="5" t="n"/>
-      <c r="F25" s="5" t="n"/>
-      <c r="G25" s="6" t="n"/>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/dagmar-ilisson-962358212</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>LinkedIn Connection Requested</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>46246</v>
+      </c>
       <c r="H25" s="5">
         <f>IF(G25="","",TODAY()-G25)</f>
         <v/>
       </c>
-      <c r="I25" s="5" t="n"/>
-      <c r="J25" s="6" t="n"/>
-      <c r="K25" s="5" t="n"/>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>Send LinkedIn Message 1 (if connected)</t>
+        </is>
+      </c>
+      <c r="J25" s="6" t="n">
+        <v>46248</v>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L25" s="6" t="n"/>
-      <c r="M25" s="5" t="n"/>
+      <c r="M25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N25" s="6" t="n"/>
-      <c r="O25" s="5" t="n"/>
+      <c r="O25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P25" s="6" t="n"/>
-      <c r="Q25" s="5" t="n"/>
+      <c r="Q25" s="5" t="inlineStr">
+        <is>
+          <t>No email available via Apollo (Basic Trial plan blocks enrichment) — LinkedIn-only outreach. Hook: Saw your Sales and Business Development Representative role at Eversports</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="n"/>
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Umut Ateș</t>
+        </is>
+      </c>
       <c r="B26" s="5" t="n"/>
-      <c r="C26" s="5" t="n"/>
-      <c r="D26" s="5" t="n"/>
-      <c r="E26" s="5" t="n"/>
-      <c r="F26" s="5" t="n"/>
-      <c r="G26" s="6" t="n"/>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/umut-ate%c8%99-172743164</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>LinkedIn Connection Requested</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>46246</v>
+      </c>
       <c r="H26" s="5">
         <f>IF(G26="","",TODAY()-G26)</f>
         <v/>
       </c>
-      <c r="I26" s="5" t="n"/>
-      <c r="J26" s="6" t="n"/>
-      <c r="K26" s="5" t="n"/>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Send LinkedIn Message 1 (if connected)</t>
+        </is>
+      </c>
+      <c r="J26" s="6" t="n">
+        <v>46248</v>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L26" s="6" t="n"/>
-      <c r="M26" s="5" t="n"/>
+      <c r="M26" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N26" s="6" t="n"/>
-      <c r="O26" s="5" t="n"/>
+      <c r="O26" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P26" s="6" t="n"/>
-      <c r="Q26" s="5" t="n"/>
+      <c r="Q26" s="5" t="inlineStr">
+        <is>
+          <t>No email available via Apollo (Basic Trial plan blocks enrichment) — LinkedIn-only outreach. Hook: Saw your Sales role at OPLOG</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="n"/>
-      <c r="B27" s="5" t="n"/>
-      <c r="C27" s="5" t="n"/>
-      <c r="D27" s="5" t="n"/>
-      <c r="E27" s="5" t="n"/>
-      <c r="F27" s="5" t="n"/>
-      <c r="G27" s="6" t="n"/>
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Andreea Traistaru</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>andreea.traistaru@salespartner.app</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/andreea-tr%c4%83istaru-3347a7139</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
       <c r="H27" s="5">
         <f>IF(G27="","",TODAY()-G27)</f>
         <v/>
       </c>
-      <c r="I27" s="5" t="n"/>
-      <c r="J27" s="6" t="n"/>
-      <c r="K27" s="5" t="n"/>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L27" s="6" t="n"/>
-      <c r="M27" s="5" t="n"/>
+      <c r="M27" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N27" s="6" t="n"/>
-      <c r="O27" s="5" t="n"/>
+      <c r="O27" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P27" s="6" t="n"/>
-      <c r="Q27" s="5" t="n"/>
+      <c r="Q27" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n"/>

</xml_diff>

<commit_message>
Record unsubscribe (Tanishq Munjal) and bounce (Katie Collopy)
- Tanishq Munjal replied to Email 1 asking to be removed; marked
  Opted Out = Y, permanently excluded from future contact.
- Katie Collopy's Email 1 bounced (address not found); marked
  Bounced = Y, pivoted Next Action to LinkedIn connection request.
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -1711,7 +1711,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Drafted</t>
+          <t>Opted Out</t>
         </is>
       </c>
       <c r="G17" s="6" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J17" s="6" t="n">
@@ -1737,10 +1737,12 @@
       <c r="L17" s="6" t="n"/>
       <c r="M17" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N17" s="6" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N17" s="6" t="n">
+        <v>46246</v>
+      </c>
       <c r="O17" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -1749,7 +1751,7 @@
       <c r="P17" s="6" t="n"/>
       <c r="Q17" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Business Development Representative &amp; Account Executive role at Spear Growth</t>
+          <t>Replied to Email 1 with Unsubscribe request (received 2026-08-12 12:40). Permanently excluded.</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1853,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Drafted</t>
+          <t>Bounced</t>
         </is>
       </c>
       <c r="G19" s="6" t="n">
@@ -1863,11 +1865,11 @@
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send LinkedIn Connection Request</t>
         </is>
       </c>
       <c r="J19" s="6" t="n">
-        <v>46252</v>
+        <v>46246</v>
       </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
@@ -1883,13 +1885,15 @@
       <c r="N19" s="6" t="n"/>
       <c r="O19" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="P19" s="6" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P19" s="6" t="n">
+        <v>46246</v>
+      </c>
       <c r="Q19" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales and Business Development Representative role at Maverick Media</t>
+          <t>Email bounced: address not found (mailer-daemon, 2026-08-12 12:39). Do not re-email; pivoted to LinkedIn.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Redesign outreach cadence: 5-touch email sequence on Mon/Wed/Fri schedule
- Add Follow-up 3 and Follow-up 4 to email_templates.md/.html; Email 1
  now leads into 4 follow-ups instead of 2, tied to fixed weekdays
  (Wed/Fri) rather than business-day counts.
- Add Region column to tracker.xlsx (India/Gulf/Europe/Other) for
  grouping the draft digest by approximate timezone.
- Expand Stage dropdown to include Follow-up 3/4 Sent and Sequence
  Complete.
- Migrate 16 in-flight contacts' Next Action Date from the old
  Tuesday placeholder to the new Wednesday follow-up slot.
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -93,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -115,6 +115,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -480,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q200"/>
+  <dimension ref="A1:R200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -499,7 +500,7 @@
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="11" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -585,6 +586,11 @@
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
@@ -653,7 +659,12 @@
         </is>
       </c>
       <c r="P2" s="3" t="inlineStr"/>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="Q2" s="9" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>Met at a webinar in July</t>
         </is>
@@ -721,6 +732,11 @@
       <c r="P3" s="6" t="n"/>
       <c r="Q3" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
           <t>No email available via Apollo (Basic Trial plan blocks enrichment) — LinkedIn-only outreach. Hook: Saw your Presales Solutions Consultant role at Tata Consultancy Services</t>
         </is>
       </c>
@@ -770,10 +786,8 @@
           <t>Send Follow-up 1</t>
         </is>
       </c>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
+      <c r="J4" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
@@ -795,6 +809,11 @@
       <c r="P4" s="6" t="n"/>
       <c r="Q4" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R4" s="5" t="inlineStr">
+        <is>
           <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
         </is>
       </c>
@@ -844,10 +863,8 @@
           <t>Send Follow-up 1</t>
         </is>
       </c>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
+      <c r="J5" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
@@ -869,6 +886,11 @@
       <c r="P5" s="6" t="n"/>
       <c r="Q5" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R5" s="5" t="inlineStr">
+        <is>
           <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
         </is>
       </c>
@@ -918,10 +940,8 @@
           <t>Send Follow-up 1</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
+      <c r="J6" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
@@ -943,6 +963,11 @@
       <c r="P6" s="6" t="n"/>
       <c r="Q6" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R6" s="5" t="inlineStr">
+        <is>
           <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
         </is>
       </c>
@@ -992,10 +1017,8 @@
           <t>Send Follow-up 1</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
+      <c r="J7" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
@@ -1017,6 +1040,11 @@
       <c r="P7" s="6" t="n"/>
       <c r="Q7" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R7" s="5" t="inlineStr">
+        <is>
           <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
         </is>
       </c>
@@ -1091,6 +1119,11 @@
       </c>
       <c r="Q8" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
           <t>Email 1 sent 2026-08-12, bounced same day (Address not found - the address couldn't be found, or is unable to receive mail.). Retroactively logged from Gmail — see run digest. Pivoting to LinkedIn since LinkedIn URL available.</t>
         </is>
       </c>
@@ -1140,10 +1173,8 @@
           <t>Send Follow-up 1</t>
         </is>
       </c>
-      <c r="J9" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
+      <c r="J9" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
@@ -1165,6 +1196,11 @@
       <c r="P9" s="6" t="n"/>
       <c r="Q9" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R9" s="5" t="inlineStr">
+        <is>
           <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
         </is>
       </c>
@@ -1213,7 +1249,7 @@
         </is>
       </c>
       <c r="J10" s="6" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
@@ -1235,6 +1271,11 @@
       <c r="P10" s="6" t="n"/>
       <c r="Q10" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R10" s="5" t="inlineStr">
+        <is>
           <t>Hook: Saw your Sales Business Development Representative role at REVEL | Renting de Coches</t>
         </is>
       </c>
@@ -1284,10 +1325,8 @@
           <t>Send Follow-up 1</t>
         </is>
       </c>
-      <c r="J11" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
+      <c r="J11" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
@@ -1309,6 +1348,11 @@
       <c r="P11" s="6" t="n"/>
       <c r="Q11" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R11" s="5" t="inlineStr">
+        <is>
           <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
         </is>
       </c>
@@ -1358,10 +1402,8 @@
           <t>Send Follow-up 1</t>
         </is>
       </c>
-      <c r="J12" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
+      <c r="J12" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
@@ -1383,6 +1425,11 @@
       <c r="P12" s="6" t="n"/>
       <c r="Q12" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R12" s="5" t="inlineStr">
+        <is>
           <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
         </is>
       </c>
@@ -1457,6 +1504,11 @@
       </c>
       <c r="Q13" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="inlineStr">
+        <is>
           <t>Email 1 sent 2026-08-12, bounced same day (550 No Such User (address not found)). Retroactively logged from Gmail — see run digest. Pivoting to LinkedIn since LinkedIn URL available.</t>
         </is>
       </c>
@@ -1506,10 +1558,8 @@
           <t>Send Follow-up 1</t>
         </is>
       </c>
-      <c r="J14" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
+      <c r="J14" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
@@ -1531,6 +1581,11 @@
       <c r="P14" s="6" t="n"/>
       <c r="Q14" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R14" s="5" t="inlineStr">
+        <is>
           <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
         </is>
       </c>
@@ -1580,10 +1635,8 @@
           <t>Send Follow-up 1</t>
         </is>
       </c>
-      <c r="J15" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
+      <c r="J15" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
@@ -1605,6 +1658,11 @@
       <c r="P15" s="6" t="n"/>
       <c r="Q15" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R15" s="5" t="inlineStr">
+        <is>
           <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
         </is>
       </c>
@@ -1679,6 +1737,11 @@
       </c>
       <c r="Q16" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R16" s="5" t="inlineStr">
+        <is>
           <t>Email 1 sent 2026-08-12, bounced same day (550 5.7.1 Service unavailable / message blocked). Retroactively logged from Gmail — see run digest. Pivoting to LinkedIn since LinkedIn URL available.</t>
         </is>
       </c>
@@ -1751,6 +1814,11 @@
       <c r="P17" s="6" t="n"/>
       <c r="Q17" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R17" s="5" t="inlineStr">
+        <is>
           <t>Replied to Email 1 with Unsubscribe request (received 2026-08-12 12:40). Permanently excluded.</t>
         </is>
       </c>
@@ -1799,7 +1867,7 @@
         </is>
       </c>
       <c r="J18" s="6" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
@@ -1821,6 +1889,11 @@
       <c r="P18" s="6" t="n"/>
       <c r="Q18" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R18" s="5" t="inlineStr">
+        <is>
           <t>Hook: Saw your Presales Solutions Consultant role at o9 Solutions, Inc.</t>
         </is>
       </c>
@@ -1893,6 +1966,11 @@
       </c>
       <c r="Q19" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R19" s="5" t="inlineStr">
+        <is>
           <t>Email bounced: address not found (mailer-daemon, 2026-08-12 12:39). Do not re-email; pivoted to LinkedIn.</t>
         </is>
       </c>
@@ -1942,10 +2020,8 @@
           <t>Send Follow-up 1</t>
         </is>
       </c>
-      <c r="J20" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
+      <c r="J20" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
@@ -1967,6 +2043,11 @@
       <c r="P20" s="6" t="n"/>
       <c r="Q20" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R20" s="5" t="inlineStr">
+        <is>
           <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
         </is>
       </c>
@@ -2015,7 +2096,7 @@
         </is>
       </c>
       <c r="J21" s="6" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="K21" s="5" t="inlineStr">
         <is>
@@ -2037,6 +2118,11 @@
       <c r="P21" s="6" t="n"/>
       <c r="Q21" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R21" s="5" t="inlineStr">
+        <is>
           <t>Hook: Saw your Presales Solutions Consultant role at Siemens Digital Industries Software</t>
         </is>
       </c>
@@ -2086,10 +2172,8 @@
           <t>Send Follow-up 1</t>
         </is>
       </c>
-      <c r="J22" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
+      <c r="J22" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
@@ -2111,6 +2195,11 @@
       <c r="P22" s="6" t="n"/>
       <c r="Q22" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R22" s="5" t="inlineStr">
+        <is>
           <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
         </is>
       </c>
@@ -2177,6 +2266,11 @@
       <c r="P23" s="6" t="n"/>
       <c r="Q23" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R23" s="5" t="inlineStr">
+        <is>
           <t>No email available via Apollo (Basic Trial plan blocks enrichment) — LinkedIn-only outreach. Hook: Saw your Sales Business Development Representative role at Luxiris</t>
         </is>
       </c>
@@ -2225,7 +2319,7 @@
         </is>
       </c>
       <c r="J24" s="6" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
@@ -2247,6 +2341,11 @@
       <c r="P24" s="6" t="n"/>
       <c r="Q24" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R24" s="5" t="inlineStr">
+        <is>
           <t>Hook: Saw your Presales Solutions Consultant role at Siemens Digital Industries Software</t>
         </is>
       </c>
@@ -2313,6 +2412,11 @@
       <c r="P25" s="6" t="n"/>
       <c r="Q25" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R25" s="5" t="inlineStr">
+        <is>
           <t>No email available via Apollo (Basic Trial plan blocks enrichment) — LinkedIn-only outreach. Hook: Saw your Sales and Business Development Representative role at Eversports</t>
         </is>
       </c>
@@ -2379,6 +2483,11 @@
       <c r="P26" s="6" t="n"/>
       <c r="Q26" s="5" t="inlineStr">
         <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R26" s="5" t="inlineStr">
+        <is>
           <t>No email available via Apollo (Basic Trial plan blocks enrichment) — LinkedIn-only outreach. Hook: Saw your Sales role at OPLOG</t>
         </is>
       </c>
@@ -2428,10 +2537,8 @@
           <t>Send Follow-up 1</t>
         </is>
       </c>
-      <c r="J27" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
+      <c r="J27" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
@@ -2452,6 +2559,11 @@
       </c>
       <c r="P27" s="6" t="n"/>
       <c r="Q27" s="5" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R27" s="5" t="inlineStr">
         <is>
           <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
         </is>
@@ -2478,6 +2590,7 @@
       <c r="O28" s="5" t="n"/>
       <c r="P28" s="6" t="n"/>
       <c r="Q28" s="5" t="n"/>
+      <c r="R28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n"/>
@@ -2500,6 +2613,7 @@
       <c r="O29" s="5" t="n"/>
       <c r="P29" s="6" t="n"/>
       <c r="Q29" s="5" t="n"/>
+      <c r="R29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="n"/>
@@ -2522,6 +2636,7 @@
       <c r="O30" s="5" t="n"/>
       <c r="P30" s="6" t="n"/>
       <c r="Q30" s="5" t="n"/>
+      <c r="R30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n"/>
@@ -2544,6 +2659,7 @@
       <c r="O31" s="5" t="n"/>
       <c r="P31" s="6" t="n"/>
       <c r="Q31" s="5" t="n"/>
+      <c r="R31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n"/>
@@ -2566,6 +2682,7 @@
       <c r="O32" s="5" t="n"/>
       <c r="P32" s="6" t="n"/>
       <c r="Q32" s="5" t="n"/>
+      <c r="R32" s="5" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n"/>
@@ -2588,6 +2705,7 @@
       <c r="O33" s="5" t="n"/>
       <c r="P33" s="6" t="n"/>
       <c r="Q33" s="5" t="n"/>
+      <c r="R33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n"/>
@@ -2610,6 +2728,7 @@
       <c r="O34" s="5" t="n"/>
       <c r="P34" s="6" t="n"/>
       <c r="Q34" s="5" t="n"/>
+      <c r="R34" s="5" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n"/>
@@ -2632,6 +2751,7 @@
       <c r="O35" s="5" t="n"/>
       <c r="P35" s="6" t="n"/>
       <c r="Q35" s="5" t="n"/>
+      <c r="R35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="n"/>
@@ -2654,6 +2774,7 @@
       <c r="O36" s="5" t="n"/>
       <c r="P36" s="6" t="n"/>
       <c r="Q36" s="5" t="n"/>
+      <c r="R36" s="5" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n"/>
@@ -2676,6 +2797,7 @@
       <c r="O37" s="5" t="n"/>
       <c r="P37" s="6" t="n"/>
       <c r="Q37" s="5" t="n"/>
+      <c r="R37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="n"/>
@@ -2698,6 +2820,7 @@
       <c r="O38" s="5" t="n"/>
       <c r="P38" s="6" t="n"/>
       <c r="Q38" s="5" t="n"/>
+      <c r="R38" s="5" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n"/>
@@ -2720,6 +2843,7 @@
       <c r="O39" s="5" t="n"/>
       <c r="P39" s="6" t="n"/>
       <c r="Q39" s="5" t="n"/>
+      <c r="R39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="n"/>
@@ -2742,6 +2866,7 @@
       <c r="O40" s="5" t="n"/>
       <c r="P40" s="6" t="n"/>
       <c r="Q40" s="5" t="n"/>
+      <c r="R40" s="5" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n"/>
@@ -2764,6 +2889,7 @@
       <c r="O41" s="5" t="n"/>
       <c r="P41" s="6" t="n"/>
       <c r="Q41" s="5" t="n"/>
+      <c r="R41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n"/>
@@ -2786,6 +2912,7 @@
       <c r="O42" s="5" t="n"/>
       <c r="P42" s="6" t="n"/>
       <c r="Q42" s="5" t="n"/>
+      <c r="R42" s="5" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n"/>
@@ -2808,6 +2935,7 @@
       <c r="O43" s="5" t="n"/>
       <c r="P43" s="6" t="n"/>
       <c r="Q43" s="5" t="n"/>
+      <c r="R43" s="5" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n"/>
@@ -2830,6 +2958,7 @@
       <c r="O44" s="5" t="n"/>
       <c r="P44" s="6" t="n"/>
       <c r="Q44" s="5" t="n"/>
+      <c r="R44" s="5" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n"/>
@@ -2852,6 +2981,7 @@
       <c r="O45" s="5" t="n"/>
       <c r="P45" s="6" t="n"/>
       <c r="Q45" s="5" t="n"/>
+      <c r="R45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="n"/>
@@ -2874,6 +3004,7 @@
       <c r="O46" s="5" t="n"/>
       <c r="P46" s="6" t="n"/>
       <c r="Q46" s="5" t="n"/>
+      <c r="R46" s="5" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n"/>
@@ -2896,6 +3027,7 @@
       <c r="O47" s="5" t="n"/>
       <c r="P47" s="6" t="n"/>
       <c r="Q47" s="5" t="n"/>
+      <c r="R47" s="5" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="n"/>
@@ -2918,6 +3050,7 @@
       <c r="O48" s="5" t="n"/>
       <c r="P48" s="6" t="n"/>
       <c r="Q48" s="5" t="n"/>
+      <c r="R48" s="5" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="5" t="n"/>
@@ -2940,6 +3073,7 @@
       <c r="O49" s="5" t="n"/>
       <c r="P49" s="6" t="n"/>
       <c r="Q49" s="5" t="n"/>
+      <c r="R49" s="5" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="n"/>
@@ -2962,6 +3096,7 @@
       <c r="O50" s="5" t="n"/>
       <c r="P50" s="6" t="n"/>
       <c r="Q50" s="5" t="n"/>
+      <c r="R50" s="5" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n"/>
@@ -2984,6 +3119,7 @@
       <c r="O51" s="5" t="n"/>
       <c r="P51" s="6" t="n"/>
       <c r="Q51" s="5" t="n"/>
+      <c r="R51" s="5" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="n"/>
@@ -3006,6 +3142,7 @@
       <c r="O52" s="5" t="n"/>
       <c r="P52" s="6" t="n"/>
       <c r="Q52" s="5" t="n"/>
+      <c r="R52" s="5" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n"/>
@@ -3028,6 +3165,7 @@
       <c r="O53" s="5" t="n"/>
       <c r="P53" s="6" t="n"/>
       <c r="Q53" s="5" t="n"/>
+      <c r="R53" s="5" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="n"/>
@@ -3050,6 +3188,7 @@
       <c r="O54" s="5" t="n"/>
       <c r="P54" s="6" t="n"/>
       <c r="Q54" s="5" t="n"/>
+      <c r="R54" s="5" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="5" t="n"/>
@@ -3072,6 +3211,7 @@
       <c r="O55" s="5" t="n"/>
       <c r="P55" s="6" t="n"/>
       <c r="Q55" s="5" t="n"/>
+      <c r="R55" s="5" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="5" t="n"/>
@@ -3094,6 +3234,7 @@
       <c r="O56" s="5" t="n"/>
       <c r="P56" s="6" t="n"/>
       <c r="Q56" s="5" t="n"/>
+      <c r="R56" s="5" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="5" t="n"/>
@@ -3116,6 +3257,7 @@
       <c r="O57" s="5" t="n"/>
       <c r="P57" s="6" t="n"/>
       <c r="Q57" s="5" t="n"/>
+      <c r="R57" s="5" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="5" t="n"/>
@@ -3138,6 +3280,7 @@
       <c r="O58" s="5" t="n"/>
       <c r="P58" s="6" t="n"/>
       <c r="Q58" s="5" t="n"/>
+      <c r="R58" s="5" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="5" t="n"/>
@@ -3160,6 +3303,7 @@
       <c r="O59" s="5" t="n"/>
       <c r="P59" s="6" t="n"/>
       <c r="Q59" s="5" t="n"/>
+      <c r="R59" s="5" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n"/>
@@ -3182,6 +3326,7 @@
       <c r="O60" s="5" t="n"/>
       <c r="P60" s="6" t="n"/>
       <c r="Q60" s="5" t="n"/>
+      <c r="R60" s="5" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="5" t="n"/>
@@ -3204,6 +3349,7 @@
       <c r="O61" s="5" t="n"/>
       <c r="P61" s="6" t="n"/>
       <c r="Q61" s="5" t="n"/>
+      <c r="R61" s="5" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="5" t="n"/>
@@ -3226,6 +3372,7 @@
       <c r="O62" s="5" t="n"/>
       <c r="P62" s="6" t="n"/>
       <c r="Q62" s="5" t="n"/>
+      <c r="R62" s="5" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="n"/>
@@ -3248,6 +3395,7 @@
       <c r="O63" s="5" t="n"/>
       <c r="P63" s="6" t="n"/>
       <c r="Q63" s="5" t="n"/>
+      <c r="R63" s="5" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="5" t="n"/>
@@ -3270,6 +3418,7 @@
       <c r="O64" s="5" t="n"/>
       <c r="P64" s="6" t="n"/>
       <c r="Q64" s="5" t="n"/>
+      <c r="R64" s="5" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="5" t="n"/>
@@ -3292,6 +3441,7 @@
       <c r="O65" s="5" t="n"/>
       <c r="P65" s="6" t="n"/>
       <c r="Q65" s="5" t="n"/>
+      <c r="R65" s="5" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="5" t="n"/>
@@ -3314,6 +3464,7 @@
       <c r="O66" s="5" t="n"/>
       <c r="P66" s="6" t="n"/>
       <c r="Q66" s="5" t="n"/>
+      <c r="R66" s="5" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="5" t="n"/>
@@ -3336,6 +3487,7 @@
       <c r="O67" s="5" t="n"/>
       <c r="P67" s="6" t="n"/>
       <c r="Q67" s="5" t="n"/>
+      <c r="R67" s="5" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="5" t="n"/>
@@ -3358,6 +3510,7 @@
       <c r="O68" s="5" t="n"/>
       <c r="P68" s="6" t="n"/>
       <c r="Q68" s="5" t="n"/>
+      <c r="R68" s="5" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="5" t="n"/>
@@ -3380,6 +3533,7 @@
       <c r="O69" s="5" t="n"/>
       <c r="P69" s="6" t="n"/>
       <c r="Q69" s="5" t="n"/>
+      <c r="R69" s="5" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="5" t="n"/>
@@ -3402,6 +3556,7 @@
       <c r="O70" s="5" t="n"/>
       <c r="P70" s="6" t="n"/>
       <c r="Q70" s="5" t="n"/>
+      <c r="R70" s="5" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="5" t="n"/>
@@ -3424,6 +3579,7 @@
       <c r="O71" s="5" t="n"/>
       <c r="P71" s="6" t="n"/>
       <c r="Q71" s="5" t="n"/>
+      <c r="R71" s="5" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="5" t="n"/>
@@ -3446,6 +3602,7 @@
       <c r="O72" s="5" t="n"/>
       <c r="P72" s="6" t="n"/>
       <c r="Q72" s="5" t="n"/>
+      <c r="R72" s="5" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="5" t="n"/>
@@ -3468,6 +3625,7 @@
       <c r="O73" s="5" t="n"/>
       <c r="P73" s="6" t="n"/>
       <c r="Q73" s="5" t="n"/>
+      <c r="R73" s="5" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="5" t="n"/>
@@ -3490,6 +3648,7 @@
       <c r="O74" s="5" t="n"/>
       <c r="P74" s="6" t="n"/>
       <c r="Q74" s="5" t="n"/>
+      <c r="R74" s="5" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="5" t="n"/>
@@ -3512,6 +3671,7 @@
       <c r="O75" s="5" t="n"/>
       <c r="P75" s="6" t="n"/>
       <c r="Q75" s="5" t="n"/>
+      <c r="R75" s="5" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="5" t="n"/>
@@ -3534,6 +3694,7 @@
       <c r="O76" s="5" t="n"/>
       <c r="P76" s="6" t="n"/>
       <c r="Q76" s="5" t="n"/>
+      <c r="R76" s="5" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="5" t="n"/>
@@ -3556,6 +3717,7 @@
       <c r="O77" s="5" t="n"/>
       <c r="P77" s="6" t="n"/>
       <c r="Q77" s="5" t="n"/>
+      <c r="R77" s="5" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="5" t="n"/>
@@ -3578,6 +3740,7 @@
       <c r="O78" s="5" t="n"/>
       <c r="P78" s="6" t="n"/>
       <c r="Q78" s="5" t="n"/>
+      <c r="R78" s="5" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="5" t="n"/>
@@ -3600,6 +3763,7 @@
       <c r="O79" s="5" t="n"/>
       <c r="P79" s="6" t="n"/>
       <c r="Q79" s="5" t="n"/>
+      <c r="R79" s="5" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="5" t="n"/>
@@ -3622,6 +3786,7 @@
       <c r="O80" s="5" t="n"/>
       <c r="P80" s="6" t="n"/>
       <c r="Q80" s="5" t="n"/>
+      <c r="R80" s="5" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="5" t="n"/>
@@ -3644,6 +3809,7 @@
       <c r="O81" s="5" t="n"/>
       <c r="P81" s="6" t="n"/>
       <c r="Q81" s="5" t="n"/>
+      <c r="R81" s="5" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="5" t="n"/>
@@ -3666,6 +3832,7 @@
       <c r="O82" s="5" t="n"/>
       <c r="P82" s="6" t="n"/>
       <c r="Q82" s="5" t="n"/>
+      <c r="R82" s="5" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="5" t="n"/>
@@ -3688,6 +3855,7 @@
       <c r="O83" s="5" t="n"/>
       <c r="P83" s="6" t="n"/>
       <c r="Q83" s="5" t="n"/>
+      <c r="R83" s="5" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="5" t="n"/>
@@ -3710,6 +3878,7 @@
       <c r="O84" s="5" t="n"/>
       <c r="P84" s="6" t="n"/>
       <c r="Q84" s="5" t="n"/>
+      <c r="R84" s="5" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="5" t="n"/>
@@ -3732,6 +3901,7 @@
       <c r="O85" s="5" t="n"/>
       <c r="P85" s="6" t="n"/>
       <c r="Q85" s="5" t="n"/>
+      <c r="R85" s="5" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="5" t="n"/>
@@ -3754,6 +3924,7 @@
       <c r="O86" s="5" t="n"/>
       <c r="P86" s="6" t="n"/>
       <c r="Q86" s="5" t="n"/>
+      <c r="R86" s="5" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="5" t="n"/>
@@ -3776,6 +3947,7 @@
       <c r="O87" s="5" t="n"/>
       <c r="P87" s="6" t="n"/>
       <c r="Q87" s="5" t="n"/>
+      <c r="R87" s="5" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="5" t="n"/>
@@ -3798,6 +3970,7 @@
       <c r="O88" s="5" t="n"/>
       <c r="P88" s="6" t="n"/>
       <c r="Q88" s="5" t="n"/>
+      <c r="R88" s="5" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="5" t="n"/>
@@ -3820,6 +3993,7 @@
       <c r="O89" s="5" t="n"/>
       <c r="P89" s="6" t="n"/>
       <c r="Q89" s="5" t="n"/>
+      <c r="R89" s="5" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="5" t="n"/>
@@ -3842,6 +4016,7 @@
       <c r="O90" s="5" t="n"/>
       <c r="P90" s="6" t="n"/>
       <c r="Q90" s="5" t="n"/>
+      <c r="R90" s="5" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="5" t="n"/>
@@ -3864,6 +4039,7 @@
       <c r="O91" s="5" t="n"/>
       <c r="P91" s="6" t="n"/>
       <c r="Q91" s="5" t="n"/>
+      <c r="R91" s="5" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="5" t="n"/>
@@ -3886,6 +4062,7 @@
       <c r="O92" s="5" t="n"/>
       <c r="P92" s="6" t="n"/>
       <c r="Q92" s="5" t="n"/>
+      <c r="R92" s="5" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="5" t="n"/>
@@ -3908,6 +4085,7 @@
       <c r="O93" s="5" t="n"/>
       <c r="P93" s="6" t="n"/>
       <c r="Q93" s="5" t="n"/>
+      <c r="R93" s="5" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="5" t="n"/>
@@ -3930,6 +4108,7 @@
       <c r="O94" s="5" t="n"/>
       <c r="P94" s="6" t="n"/>
       <c r="Q94" s="5" t="n"/>
+      <c r="R94" s="5" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="5" t="n"/>
@@ -3952,6 +4131,7 @@
       <c r="O95" s="5" t="n"/>
       <c r="P95" s="6" t="n"/>
       <c r="Q95" s="5" t="n"/>
+      <c r="R95" s="5" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="5" t="n"/>
@@ -3974,6 +4154,7 @@
       <c r="O96" s="5" t="n"/>
       <c r="P96" s="6" t="n"/>
       <c r="Q96" s="5" t="n"/>
+      <c r="R96" s="5" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="5" t="n"/>
@@ -3996,6 +4177,7 @@
       <c r="O97" s="5" t="n"/>
       <c r="P97" s="6" t="n"/>
       <c r="Q97" s="5" t="n"/>
+      <c r="R97" s="5" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="5" t="n"/>
@@ -4018,6 +4200,7 @@
       <c r="O98" s="5" t="n"/>
       <c r="P98" s="6" t="n"/>
       <c r="Q98" s="5" t="n"/>
+      <c r="R98" s="5" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="5" t="n"/>
@@ -4040,6 +4223,7 @@
       <c r="O99" s="5" t="n"/>
       <c r="P99" s="6" t="n"/>
       <c r="Q99" s="5" t="n"/>
+      <c r="R99" s="5" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="5" t="n"/>
@@ -4062,6 +4246,7 @@
       <c r="O100" s="5" t="n"/>
       <c r="P100" s="6" t="n"/>
       <c r="Q100" s="5" t="n"/>
+      <c r="R100" s="5" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="5" t="n"/>
@@ -4084,6 +4269,7 @@
       <c r="O101" s="5" t="n"/>
       <c r="P101" s="6" t="n"/>
       <c r="Q101" s="5" t="n"/>
+      <c r="R101" s="5" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="5" t="n"/>
@@ -4106,6 +4292,7 @@
       <c r="O102" s="5" t="n"/>
       <c r="P102" s="6" t="n"/>
       <c r="Q102" s="5" t="n"/>
+      <c r="R102" s="5" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="5" t="n"/>
@@ -4128,6 +4315,7 @@
       <c r="O103" s="5" t="n"/>
       <c r="P103" s="6" t="n"/>
       <c r="Q103" s="5" t="n"/>
+      <c r="R103" s="5" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="5" t="n"/>
@@ -4150,6 +4338,7 @@
       <c r="O104" s="5" t="n"/>
       <c r="P104" s="6" t="n"/>
       <c r="Q104" s="5" t="n"/>
+      <c r="R104" s="5" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="5" t="n"/>
@@ -4172,6 +4361,7 @@
       <c r="O105" s="5" t="n"/>
       <c r="P105" s="6" t="n"/>
       <c r="Q105" s="5" t="n"/>
+      <c r="R105" s="5" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="5" t="n"/>
@@ -4194,6 +4384,7 @@
       <c r="O106" s="5" t="n"/>
       <c r="P106" s="6" t="n"/>
       <c r="Q106" s="5" t="n"/>
+      <c r="R106" s="5" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="5" t="n"/>
@@ -4216,6 +4407,7 @@
       <c r="O107" s="5" t="n"/>
       <c r="P107" s="6" t="n"/>
       <c r="Q107" s="5" t="n"/>
+      <c r="R107" s="5" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="5" t="n"/>
@@ -4238,6 +4430,7 @@
       <c r="O108" s="5" t="n"/>
       <c r="P108" s="6" t="n"/>
       <c r="Q108" s="5" t="n"/>
+      <c r="R108" s="5" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="5" t="n"/>
@@ -4260,6 +4453,7 @@
       <c r="O109" s="5" t="n"/>
       <c r="P109" s="6" t="n"/>
       <c r="Q109" s="5" t="n"/>
+      <c r="R109" s="5" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="5" t="n"/>
@@ -4282,6 +4476,7 @@
       <c r="O110" s="5" t="n"/>
       <c r="P110" s="6" t="n"/>
       <c r="Q110" s="5" t="n"/>
+      <c r="R110" s="5" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="5" t="n"/>
@@ -4304,6 +4499,7 @@
       <c r="O111" s="5" t="n"/>
       <c r="P111" s="6" t="n"/>
       <c r="Q111" s="5" t="n"/>
+      <c r="R111" s="5" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="5" t="n"/>
@@ -4326,6 +4522,7 @@
       <c r="O112" s="5" t="n"/>
       <c r="P112" s="6" t="n"/>
       <c r="Q112" s="5" t="n"/>
+      <c r="R112" s="5" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="5" t="n"/>
@@ -4348,6 +4545,7 @@
       <c r="O113" s="5" t="n"/>
       <c r="P113" s="6" t="n"/>
       <c r="Q113" s="5" t="n"/>
+      <c r="R113" s="5" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="5" t="n"/>
@@ -4370,6 +4568,7 @@
       <c r="O114" s="5" t="n"/>
       <c r="P114" s="6" t="n"/>
       <c r="Q114" s="5" t="n"/>
+      <c r="R114" s="5" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="5" t="n"/>
@@ -4392,6 +4591,7 @@
       <c r="O115" s="5" t="n"/>
       <c r="P115" s="6" t="n"/>
       <c r="Q115" s="5" t="n"/>
+      <c r="R115" s="5" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="5" t="n"/>
@@ -4414,6 +4614,7 @@
       <c r="O116" s="5" t="n"/>
       <c r="P116" s="6" t="n"/>
       <c r="Q116" s="5" t="n"/>
+      <c r="R116" s="5" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="5" t="n"/>
@@ -4436,6 +4637,7 @@
       <c r="O117" s="5" t="n"/>
       <c r="P117" s="6" t="n"/>
       <c r="Q117" s="5" t="n"/>
+      <c r="R117" s="5" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="5" t="n"/>
@@ -4458,6 +4660,7 @@
       <c r="O118" s="5" t="n"/>
       <c r="P118" s="6" t="n"/>
       <c r="Q118" s="5" t="n"/>
+      <c r="R118" s="5" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="5" t="n"/>
@@ -4480,6 +4683,7 @@
       <c r="O119" s="5" t="n"/>
       <c r="P119" s="6" t="n"/>
       <c r="Q119" s="5" t="n"/>
+      <c r="R119" s="5" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="5" t="n"/>
@@ -4502,6 +4706,7 @@
       <c r="O120" s="5" t="n"/>
       <c r="P120" s="6" t="n"/>
       <c r="Q120" s="5" t="n"/>
+      <c r="R120" s="5" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="5" t="n"/>
@@ -4524,6 +4729,7 @@
       <c r="O121" s="5" t="n"/>
       <c r="P121" s="6" t="n"/>
       <c r="Q121" s="5" t="n"/>
+      <c r="R121" s="5" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="5" t="n"/>
@@ -4546,6 +4752,7 @@
       <c r="O122" s="5" t="n"/>
       <c r="P122" s="6" t="n"/>
       <c r="Q122" s="5" t="n"/>
+      <c r="R122" s="5" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="5" t="n"/>
@@ -4568,6 +4775,7 @@
       <c r="O123" s="5" t="n"/>
       <c r="P123" s="6" t="n"/>
       <c r="Q123" s="5" t="n"/>
+      <c r="R123" s="5" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="5" t="n"/>
@@ -4590,6 +4798,7 @@
       <c r="O124" s="5" t="n"/>
       <c r="P124" s="6" t="n"/>
       <c r="Q124" s="5" t="n"/>
+      <c r="R124" s="5" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="5" t="n"/>
@@ -4612,6 +4821,7 @@
       <c r="O125" s="5" t="n"/>
       <c r="P125" s="6" t="n"/>
       <c r="Q125" s="5" t="n"/>
+      <c r="R125" s="5" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="5" t="n"/>
@@ -4634,6 +4844,7 @@
       <c r="O126" s="5" t="n"/>
       <c r="P126" s="6" t="n"/>
       <c r="Q126" s="5" t="n"/>
+      <c r="R126" s="5" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="5" t="n"/>
@@ -4656,6 +4867,7 @@
       <c r="O127" s="5" t="n"/>
       <c r="P127" s="6" t="n"/>
       <c r="Q127" s="5" t="n"/>
+      <c r="R127" s="5" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="5" t="n"/>
@@ -4678,6 +4890,7 @@
       <c r="O128" s="5" t="n"/>
       <c r="P128" s="6" t="n"/>
       <c r="Q128" s="5" t="n"/>
+      <c r="R128" s="5" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="5" t="n"/>
@@ -4700,6 +4913,7 @@
       <c r="O129" s="5" t="n"/>
       <c r="P129" s="6" t="n"/>
       <c r="Q129" s="5" t="n"/>
+      <c r="R129" s="5" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="5" t="n"/>
@@ -4722,6 +4936,7 @@
       <c r="O130" s="5" t="n"/>
       <c r="P130" s="6" t="n"/>
       <c r="Q130" s="5" t="n"/>
+      <c r="R130" s="5" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="5" t="n"/>
@@ -4744,6 +4959,7 @@
       <c r="O131" s="5" t="n"/>
       <c r="P131" s="6" t="n"/>
       <c r="Q131" s="5" t="n"/>
+      <c r="R131" s="5" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="5" t="n"/>
@@ -4766,6 +4982,7 @@
       <c r="O132" s="5" t="n"/>
       <c r="P132" s="6" t="n"/>
       <c r="Q132" s="5" t="n"/>
+      <c r="R132" s="5" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="5" t="n"/>
@@ -4788,6 +5005,7 @@
       <c r="O133" s="5" t="n"/>
       <c r="P133" s="6" t="n"/>
       <c r="Q133" s="5" t="n"/>
+      <c r="R133" s="5" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="5" t="n"/>
@@ -4810,6 +5028,7 @@
       <c r="O134" s="5" t="n"/>
       <c r="P134" s="6" t="n"/>
       <c r="Q134" s="5" t="n"/>
+      <c r="R134" s="5" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="5" t="n"/>
@@ -4832,6 +5051,7 @@
       <c r="O135" s="5" t="n"/>
       <c r="P135" s="6" t="n"/>
       <c r="Q135" s="5" t="n"/>
+      <c r="R135" s="5" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="5" t="n"/>
@@ -4854,6 +5074,7 @@
       <c r="O136" s="5" t="n"/>
       <c r="P136" s="6" t="n"/>
       <c r="Q136" s="5" t="n"/>
+      <c r="R136" s="5" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="5" t="n"/>
@@ -4876,6 +5097,7 @@
       <c r="O137" s="5" t="n"/>
       <c r="P137" s="6" t="n"/>
       <c r="Q137" s="5" t="n"/>
+      <c r="R137" s="5" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="5" t="n"/>
@@ -4898,6 +5120,7 @@
       <c r="O138" s="5" t="n"/>
       <c r="P138" s="6" t="n"/>
       <c r="Q138" s="5" t="n"/>
+      <c r="R138" s="5" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="5" t="n"/>
@@ -4920,6 +5143,7 @@
       <c r="O139" s="5" t="n"/>
       <c r="P139" s="6" t="n"/>
       <c r="Q139" s="5" t="n"/>
+      <c r="R139" s="5" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="5" t="n"/>
@@ -4942,6 +5166,7 @@
       <c r="O140" s="5" t="n"/>
       <c r="P140" s="6" t="n"/>
       <c r="Q140" s="5" t="n"/>
+      <c r="R140" s="5" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="5" t="n"/>
@@ -4964,6 +5189,7 @@
       <c r="O141" s="5" t="n"/>
       <c r="P141" s="6" t="n"/>
       <c r="Q141" s="5" t="n"/>
+      <c r="R141" s="5" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="5" t="n"/>
@@ -4986,6 +5212,7 @@
       <c r="O142" s="5" t="n"/>
       <c r="P142" s="6" t="n"/>
       <c r="Q142" s="5" t="n"/>
+      <c r="R142" s="5" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="5" t="n"/>
@@ -5008,6 +5235,7 @@
       <c r="O143" s="5" t="n"/>
       <c r="P143" s="6" t="n"/>
       <c r="Q143" s="5" t="n"/>
+      <c r="R143" s="5" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="5" t="n"/>
@@ -5030,6 +5258,7 @@
       <c r="O144" s="5" t="n"/>
       <c r="P144" s="6" t="n"/>
       <c r="Q144" s="5" t="n"/>
+      <c r="R144" s="5" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="5" t="n"/>
@@ -5052,6 +5281,7 @@
       <c r="O145" s="5" t="n"/>
       <c r="P145" s="6" t="n"/>
       <c r="Q145" s="5" t="n"/>
+      <c r="R145" s="5" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="5" t="n"/>
@@ -5074,6 +5304,7 @@
       <c r="O146" s="5" t="n"/>
       <c r="P146" s="6" t="n"/>
       <c r="Q146" s="5" t="n"/>
+      <c r="R146" s="5" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="5" t="n"/>
@@ -5096,6 +5327,7 @@
       <c r="O147" s="5" t="n"/>
       <c r="P147" s="6" t="n"/>
       <c r="Q147" s="5" t="n"/>
+      <c r="R147" s="5" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="5" t="n"/>
@@ -5118,6 +5350,7 @@
       <c r="O148" s="5" t="n"/>
       <c r="P148" s="6" t="n"/>
       <c r="Q148" s="5" t="n"/>
+      <c r="R148" s="5" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="5" t="n"/>
@@ -5140,6 +5373,7 @@
       <c r="O149" s="5" t="n"/>
       <c r="P149" s="6" t="n"/>
       <c r="Q149" s="5" t="n"/>
+      <c r="R149" s="5" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="5" t="n"/>
@@ -5162,6 +5396,7 @@
       <c r="O150" s="5" t="n"/>
       <c r="P150" s="6" t="n"/>
       <c r="Q150" s="5" t="n"/>
+      <c r="R150" s="5" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="5" t="n"/>
@@ -5184,6 +5419,7 @@
       <c r="O151" s="5" t="n"/>
       <c r="P151" s="6" t="n"/>
       <c r="Q151" s="5" t="n"/>
+      <c r="R151" s="5" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="5" t="n"/>
@@ -5206,6 +5442,7 @@
       <c r="O152" s="5" t="n"/>
       <c r="P152" s="6" t="n"/>
       <c r="Q152" s="5" t="n"/>
+      <c r="R152" s="5" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="5" t="n"/>
@@ -5228,6 +5465,7 @@
       <c r="O153" s="5" t="n"/>
       <c r="P153" s="6" t="n"/>
       <c r="Q153" s="5" t="n"/>
+      <c r="R153" s="5" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="5" t="n"/>
@@ -5250,6 +5488,7 @@
       <c r="O154" s="5" t="n"/>
       <c r="P154" s="6" t="n"/>
       <c r="Q154" s="5" t="n"/>
+      <c r="R154" s="5" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="5" t="n"/>
@@ -5272,6 +5511,7 @@
       <c r="O155" s="5" t="n"/>
       <c r="P155" s="6" t="n"/>
       <c r="Q155" s="5" t="n"/>
+      <c r="R155" s="5" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="5" t="n"/>
@@ -5294,6 +5534,7 @@
       <c r="O156" s="5" t="n"/>
       <c r="P156" s="6" t="n"/>
       <c r="Q156" s="5" t="n"/>
+      <c r="R156" s="5" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="5" t="n"/>
@@ -5316,6 +5557,7 @@
       <c r="O157" s="5" t="n"/>
       <c r="P157" s="6" t="n"/>
       <c r="Q157" s="5" t="n"/>
+      <c r="R157" s="5" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="5" t="n"/>
@@ -5338,6 +5580,7 @@
       <c r="O158" s="5" t="n"/>
       <c r="P158" s="6" t="n"/>
       <c r="Q158" s="5" t="n"/>
+      <c r="R158" s="5" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="5" t="n"/>
@@ -5360,6 +5603,7 @@
       <c r="O159" s="5" t="n"/>
       <c r="P159" s="6" t="n"/>
       <c r="Q159" s="5" t="n"/>
+      <c r="R159" s="5" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="5" t="n"/>
@@ -5382,6 +5626,7 @@
       <c r="O160" s="5" t="n"/>
       <c r="P160" s="6" t="n"/>
       <c r="Q160" s="5" t="n"/>
+      <c r="R160" s="5" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="5" t="n"/>
@@ -5404,6 +5649,7 @@
       <c r="O161" s="5" t="n"/>
       <c r="P161" s="6" t="n"/>
       <c r="Q161" s="5" t="n"/>
+      <c r="R161" s="5" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="5" t="n"/>
@@ -5426,6 +5672,7 @@
       <c r="O162" s="5" t="n"/>
       <c r="P162" s="6" t="n"/>
       <c r="Q162" s="5" t="n"/>
+      <c r="R162" s="5" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="5" t="n"/>
@@ -5448,6 +5695,7 @@
       <c r="O163" s="5" t="n"/>
       <c r="P163" s="6" t="n"/>
       <c r="Q163" s="5" t="n"/>
+      <c r="R163" s="5" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="5" t="n"/>
@@ -5470,6 +5718,7 @@
       <c r="O164" s="5" t="n"/>
       <c r="P164" s="6" t="n"/>
       <c r="Q164" s="5" t="n"/>
+      <c r="R164" s="5" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="5" t="n"/>
@@ -5492,6 +5741,7 @@
       <c r="O165" s="5" t="n"/>
       <c r="P165" s="6" t="n"/>
       <c r="Q165" s="5" t="n"/>
+      <c r="R165" s="5" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="5" t="n"/>
@@ -5514,6 +5764,7 @@
       <c r="O166" s="5" t="n"/>
       <c r="P166" s="6" t="n"/>
       <c r="Q166" s="5" t="n"/>
+      <c r="R166" s="5" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="5" t="n"/>
@@ -5536,6 +5787,7 @@
       <c r="O167" s="5" t="n"/>
       <c r="P167" s="6" t="n"/>
       <c r="Q167" s="5" t="n"/>
+      <c r="R167" s="5" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="5" t="n"/>
@@ -5558,6 +5810,7 @@
       <c r="O168" s="5" t="n"/>
       <c r="P168" s="6" t="n"/>
       <c r="Q168" s="5" t="n"/>
+      <c r="R168" s="5" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="5" t="n"/>
@@ -5580,6 +5833,7 @@
       <c r="O169" s="5" t="n"/>
       <c r="P169" s="6" t="n"/>
       <c r="Q169" s="5" t="n"/>
+      <c r="R169" s="5" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="5" t="n"/>
@@ -5602,6 +5856,7 @@
       <c r="O170" s="5" t="n"/>
       <c r="P170" s="6" t="n"/>
       <c r="Q170" s="5" t="n"/>
+      <c r="R170" s="5" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="5" t="n"/>
@@ -5624,6 +5879,7 @@
       <c r="O171" s="5" t="n"/>
       <c r="P171" s="6" t="n"/>
       <c r="Q171" s="5" t="n"/>
+      <c r="R171" s="5" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="5" t="n"/>
@@ -5646,6 +5902,7 @@
       <c r="O172" s="5" t="n"/>
       <c r="P172" s="6" t="n"/>
       <c r="Q172" s="5" t="n"/>
+      <c r="R172" s="5" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="5" t="n"/>
@@ -5668,6 +5925,7 @@
       <c r="O173" s="5" t="n"/>
       <c r="P173" s="6" t="n"/>
       <c r="Q173" s="5" t="n"/>
+      <c r="R173" s="5" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="5" t="n"/>
@@ -5690,6 +5948,7 @@
       <c r="O174" s="5" t="n"/>
       <c r="P174" s="6" t="n"/>
       <c r="Q174" s="5" t="n"/>
+      <c r="R174" s="5" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="5" t="n"/>
@@ -5712,6 +5971,7 @@
       <c r="O175" s="5" t="n"/>
       <c r="P175" s="6" t="n"/>
       <c r="Q175" s="5" t="n"/>
+      <c r="R175" s="5" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="5" t="n"/>
@@ -5734,6 +5994,7 @@
       <c r="O176" s="5" t="n"/>
       <c r="P176" s="6" t="n"/>
       <c r="Q176" s="5" t="n"/>
+      <c r="R176" s="5" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="5" t="n"/>
@@ -5756,6 +6017,7 @@
       <c r="O177" s="5" t="n"/>
       <c r="P177" s="6" t="n"/>
       <c r="Q177" s="5" t="n"/>
+      <c r="R177" s="5" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="5" t="n"/>
@@ -5778,6 +6040,7 @@
       <c r="O178" s="5" t="n"/>
       <c r="P178" s="6" t="n"/>
       <c r="Q178" s="5" t="n"/>
+      <c r="R178" s="5" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="5" t="n"/>
@@ -5800,6 +6063,7 @@
       <c r="O179" s="5" t="n"/>
       <c r="P179" s="6" t="n"/>
       <c r="Q179" s="5" t="n"/>
+      <c r="R179" s="5" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="5" t="n"/>
@@ -5822,6 +6086,7 @@
       <c r="O180" s="5" t="n"/>
       <c r="P180" s="6" t="n"/>
       <c r="Q180" s="5" t="n"/>
+      <c r="R180" s="5" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="5" t="n"/>
@@ -5844,6 +6109,7 @@
       <c r="O181" s="5" t="n"/>
       <c r="P181" s="6" t="n"/>
       <c r="Q181" s="5" t="n"/>
+      <c r="R181" s="5" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="5" t="n"/>
@@ -5866,6 +6132,7 @@
       <c r="O182" s="5" t="n"/>
       <c r="P182" s="6" t="n"/>
       <c r="Q182" s="5" t="n"/>
+      <c r="R182" s="5" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="5" t="n"/>
@@ -5888,6 +6155,7 @@
       <c r="O183" s="5" t="n"/>
       <c r="P183" s="6" t="n"/>
       <c r="Q183" s="5" t="n"/>
+      <c r="R183" s="5" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="5" t="n"/>
@@ -5910,6 +6178,7 @@
       <c r="O184" s="5" t="n"/>
       <c r="P184" s="6" t="n"/>
       <c r="Q184" s="5" t="n"/>
+      <c r="R184" s="5" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="5" t="n"/>
@@ -5932,6 +6201,7 @@
       <c r="O185" s="5" t="n"/>
       <c r="P185" s="6" t="n"/>
       <c r="Q185" s="5" t="n"/>
+      <c r="R185" s="5" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="5" t="n"/>
@@ -5954,6 +6224,7 @@
       <c r="O186" s="5" t="n"/>
       <c r="P186" s="6" t="n"/>
       <c r="Q186" s="5" t="n"/>
+      <c r="R186" s="5" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="5" t="n"/>
@@ -5976,6 +6247,7 @@
       <c r="O187" s="5" t="n"/>
       <c r="P187" s="6" t="n"/>
       <c r="Q187" s="5" t="n"/>
+      <c r="R187" s="5" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="5" t="n"/>
@@ -5998,6 +6270,7 @@
       <c r="O188" s="5" t="n"/>
       <c r="P188" s="6" t="n"/>
       <c r="Q188" s="5" t="n"/>
+      <c r="R188" s="5" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="5" t="n"/>
@@ -6020,6 +6293,7 @@
       <c r="O189" s="5" t="n"/>
       <c r="P189" s="6" t="n"/>
       <c r="Q189" s="5" t="n"/>
+      <c r="R189" s="5" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="5" t="n"/>
@@ -6042,6 +6316,7 @@
       <c r="O190" s="5" t="n"/>
       <c r="P190" s="6" t="n"/>
       <c r="Q190" s="5" t="n"/>
+      <c r="R190" s="5" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="5" t="n"/>
@@ -6064,6 +6339,7 @@
       <c r="O191" s="5" t="n"/>
       <c r="P191" s="6" t="n"/>
       <c r="Q191" s="5" t="n"/>
+      <c r="R191" s="5" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="5" t="n"/>
@@ -6086,6 +6362,7 @@
       <c r="O192" s="5" t="n"/>
       <c r="P192" s="6" t="n"/>
       <c r="Q192" s="5" t="n"/>
+      <c r="R192" s="5" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="5" t="n"/>
@@ -6108,6 +6385,7 @@
       <c r="O193" s="5" t="n"/>
       <c r="P193" s="6" t="n"/>
       <c r="Q193" s="5" t="n"/>
+      <c r="R193" s="5" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="5" t="n"/>
@@ -6130,6 +6408,7 @@
       <c r="O194" s="5" t="n"/>
       <c r="P194" s="6" t="n"/>
       <c r="Q194" s="5" t="n"/>
+      <c r="R194" s="5" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="5" t="n"/>
@@ -6152,6 +6431,7 @@
       <c r="O195" s="5" t="n"/>
       <c r="P195" s="6" t="n"/>
       <c r="Q195" s="5" t="n"/>
+      <c r="R195" s="5" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="5" t="n"/>
@@ -6174,6 +6454,7 @@
       <c r="O196" s="5" t="n"/>
       <c r="P196" s="6" t="n"/>
       <c r="Q196" s="5" t="n"/>
+      <c r="R196" s="5" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="5" t="n"/>
@@ -6196,6 +6477,7 @@
       <c r="O197" s="5" t="n"/>
       <c r="P197" s="6" t="n"/>
       <c r="Q197" s="5" t="n"/>
+      <c r="R197" s="5" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="5" t="n"/>
@@ -6218,6 +6500,7 @@
       <c r="O198" s="5" t="n"/>
       <c r="P198" s="6" t="n"/>
       <c r="Q198" s="5" t="n"/>
+      <c r="R198" s="5" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="5" t="n"/>
@@ -6240,6 +6523,7 @@
       <c r="O199" s="5" t="n"/>
       <c r="P199" s="6" t="n"/>
       <c r="Q199" s="5" t="n"/>
+      <c r="R199" s="5" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="5" t="n"/>
@@ -6262,11 +6546,12 @@
       <c r="O200" s="5" t="n"/>
       <c r="P200" s="6" t="n"/>
       <c r="Q200" s="5" t="n"/>
+      <c r="R200" s="5" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="5">
+  <dataValidations count="6">
     <dataValidation sqref="F2:F201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"New,Email 1 Sent,Follow-up 1 Sent,Follow-up 2 Sent,Replied,LinkedIn Connected,LinkedIn Msg Sent,Booked,Not Interested,Opted Out,Bounced,Cold"</formula1>
+      <formula1>"New,Email 1 Sent,Follow-up 1 Sent,Follow-up 2 Sent,Follow-up 3 Sent,Follow-up 4 Sent,Sequence Complete,Replied,LinkedIn Connected,LinkedIn Msg Sent,Booked,Not Interested,Opted Out,Bounced,Cold"</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Send Initial Email,Send Follow-up Email,Send LinkedIn Connection Note,Send LinkedIn Follow-up,Wait,Mark Booked,None"</formula1>
@@ -6280,6 +6565,9 @@
     <dataValidation sqref="O2:O201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
+    <dataValidation sqref="Q2:Q201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"India,Gulf (UAE),Europe,Other,Unknown"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6291,7 +6579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -6317,56 +6605,77 @@
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2. Stage tracks where each contact is in the sequence: New -&gt; Email 1 Sent -&gt; Follow-up 1 Sent -&gt; Follow-up 2 Sent -&gt; Replied / Booked / Not Interested.</t>
+          <t>2. Stage tracks where each contact is in the sequence: New -&gt; Email 1 Sent -&gt; Follow-up 1 Sent -&gt; Follow-up 2 Sent -&gt; Follow-up 3 Sent -&gt; Follow-up 4 Sent -&gt; Sequence Complete (or Replied / Booked / Not Interested / Opted Out / Bounced at any point).</t>
         </is>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>3. Next Action + Next Action Date tell you (or the automated weekly run) what to do and when.</t>
+          <t>3. Email cadence runs on a fixed Mon/Wed/Fri schedule, not day-counts: Email 1 (Monday, new leads only) -&gt; Follow-up 1 (Wednesday, same week) -&gt; Follow-up 2 (Friday, same week) -&gt; Follow-up 3 (Wednesday, following week) -&gt; Follow-up 4 (Friday, following week, final). Three separate scheduled routines drive this: Monday pulls fresh leads and sends Email 1 only; Wednesday and Friday only draft due follow-ups for existing contacts, no new leads.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>4. Days Since Contact calculates automatically from Last Contact Date — use it to spot who's overdue for a follow-up.</t>
+          <t>4. Next Action + Next Action Date tell you (or the automated routines) what to do and when.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>5. LinkedIn messages are drafted for you but NOT sent automatically — LinkedIn's terms prohibit automated messaging, so you paste and send them yourself, then update Stage.</t>
+          <t>5. Days Since Contact calculates automatically from Last Contact Date — use it to spot who's overdue for a follow-up.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>6. Mark Booked = Y and fill Booking Date as soon as a booking confirmation arrives (email/SMS/WhatsApp) — booked contacts are excluded from further follow-ups.</t>
+          <t>6. Region groups each contact by rough timezone (India / Gulf (UAE) / Europe / Other) so the automation can order its draft digest to roughly match business hours in each region when you do your manual send pass. This does not control actual send time — nothing sends automatically, see note below.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>7. Mark Opted Out = Y and fill Opt-Out Date if someone asks to stop hearing from you (via the email unsubscribe link, a reply, or manually) — opted-out contacts are permanently excluded from all future emails, LinkedIn messages, and even from being re-added if Apollo surfaces them again later.</t>
+          <t>7. LinkedIn messages are drafted for you but NOT sent automatically — LinkedIn's terms prohibit automated messaging, so you paste and send them yourself, then update Stage.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>8. Mark Bounced = Y and fill Bounce Date if you get a "Delivery Status Notification (Failure)" from Gmail for that contact — stop emailing that address, but it's fine to still try LinkedIn if you have their profile URL. The automation checks for these automatically each run.</t>
+          <t>8. IMPORTANT: emails are drafted, never auto-sent. The Gmail integration has no send capability, so nothing leaves your account until you personally open Gmail's Drafts folder and hit Send. Exact per-recipient local-time delivery isn't possible for this reason.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="34" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>9. See email_templates.md / email_templates.html and linkedin_templates.md in this folder for the message sequence.</t>
+          <t>9. Mark Booked = Y and fill Booking Date as soon as a booking confirmation arrives (email/SMS/WhatsApp) — booked contacts are excluded from further follow-ups.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>10. Mark Opted Out = Y and fill Opt-Out Date if someone asks to stop hearing from you (via the email unsubscribe link, a reply, or manually) — opted-out contacts are permanently excluded from all future emails, LinkedIn messages, and even from being re-added if Apollo surfaces them again later.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>11. Mark Bounced = Y and fill Bounce Date if you get a "Delivery Status Notification (Failure)" from Gmail for that contact — stop emailing that address, but it's fine to still try LinkedIn if you have their profile URL. The automation checks for these automatically each run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>12. See email_templates.md / email_templates.html and linkedin_templates.md in this folder for the message sequence.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Process missed Lin Ye unsubscribe; no Follow-up 2/4 due this run
Friday follow-up routine: no rows are yet in Follow-up 1 Sent/Follow-up
3 Sent stage, so no follow-up drafts this cycle. Caught one unsubscribe
(Lin Ye, lin.ye@siemens.com) that a prior run missed - marked Opted Out.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014j96Sd2KyyK4jz2oFYxQhk
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -2080,7 +2080,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Drafted</t>
+          <t>Opted Out</t>
         </is>
       </c>
       <c r="G21" s="6" t="n">
@@ -2092,7 +2092,7 @@
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J21" s="6" t="n">
@@ -2106,10 +2106,12 @@
       <c r="L21" s="6" t="n"/>
       <c r="M21" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N21" s="6" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N21" s="6" t="n">
+        <v>46248</v>
+      </c>
       <c r="O21" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -2123,7 +2125,7 @@
       </c>
       <c r="R21" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales Solutions Consultant role at Siemens Digital Industries Software</t>
+          <t>Hook: Saw your Presales Solutions Consultant role at Siemens Digital Industries Software | Unsubscribe request received 2026-08-12 13:16 (missed in prior run, processed 2026-08-14). Permanently excluded.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monday fresh-list run: Segment A leads (week 34, 32 new Apollo contacts)
Sourced 32 net-new Presales & Sales Professionals across India/UAE/Europe
via Apollo (0 from saved contacts, 32 newly enriched, 32 lead credits
spent, 27 remaining). Drafted Email 1 for 31 with valid emails plus one
overdue pre-existing row (Jane Doe); 1 LinkedIn-only lead queued for
manual connection request. No bounces/opt-outs/bookings since last run.
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -623,23 +623,23 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr"/>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>46251</v>
+      </c>
       <c r="H2" s="4">
         <f>IF(G2="","",TODAY()-G2)</f>
         <v/>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Send Initial Email</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>46253</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -666,7 +666,7 @@
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Met at a webinar in July</t>
+          <t>Met at a webinar in July | Service Interest predates current 4-service taxonomy; treated as closest match (Career Guidance) for Email 1 wording. Overdue row from prior run, swept up by Monday routine 2026-08-17.</t>
         </is>
       </c>
     </row>
@@ -2572,740 +2572,2398 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="n"/>
-      <c r="B28" s="5" t="n"/>
-      <c r="C28" s="5" t="n"/>
-      <c r="D28" s="5" t="n"/>
-      <c r="E28" s="5" t="n"/>
-      <c r="F28" s="5" t="n"/>
-      <c r="G28" s="6" t="n"/>
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Sami Moukhalalati</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>sami.moukhalalati@earnix.com</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/moukhalalati</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H28" s="5">
         <f>IF(G28="","",TODAY()-G28)</f>
         <v/>
       </c>
-      <c r="I28" s="5" t="n"/>
-      <c r="J28" s="6" t="n"/>
-      <c r="K28" s="5" t="n"/>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J28" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K28" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L28" s="6" t="n"/>
-      <c r="M28" s="5" t="n"/>
+      <c r="M28" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N28" s="6" t="n"/>
-      <c r="O28" s="5" t="n"/>
+      <c r="O28" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P28" s="6" t="n"/>
-      <c r="Q28" s="5" t="n"/>
-      <c r="R28" s="5" t="n"/>
+      <c r="Q28" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R28" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Presales - Solutions Consultant role at Earnix</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="n"/>
-      <c r="B29" s="5" t="n"/>
-      <c r="C29" s="5" t="n"/>
-      <c r="D29" s="5" t="n"/>
-      <c r="E29" s="5" t="n"/>
-      <c r="F29" s="5" t="n"/>
-      <c r="G29" s="6" t="n"/>
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Krishna Sudheer</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>krishna.sudheer@orolabs.ai</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/krishna-sudheer-9234aa124</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H29" s="5">
         <f>IF(G29="","",TODAY()-G29)</f>
         <v/>
       </c>
-      <c r="I29" s="5" t="n"/>
-      <c r="J29" s="6" t="n"/>
-      <c r="K29" s="5" t="n"/>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J29" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L29" s="6" t="n"/>
-      <c r="M29" s="5" t="n"/>
+      <c r="M29" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N29" s="6" t="n"/>
-      <c r="O29" s="5" t="n"/>
+      <c r="O29" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P29" s="6" t="n"/>
-      <c r="Q29" s="5" t="n"/>
-      <c r="R29" s="5" t="n"/>
+      <c r="Q29" s="5" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="R29" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Solutions Consultant role at ORO Labs</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="n"/>
-      <c r="B30" s="5" t="n"/>
-      <c r="C30" s="5" t="n"/>
-      <c r="D30" s="5" t="n"/>
-      <c r="E30" s="5" t="n"/>
-      <c r="F30" s="5" t="n"/>
-      <c r="G30" s="6" t="n"/>
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Arun Venkadasubbu</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>arun.venkadasubbu@aspiresys.com</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/arunvenkadasubbu</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H30" s="5">
         <f>IF(G30="","",TODAY()-G30)</f>
         <v/>
       </c>
-      <c r="I30" s="5" t="n"/>
-      <c r="J30" s="6" t="n"/>
-      <c r="K30" s="5" t="n"/>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J30" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K30" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L30" s="6" t="n"/>
-      <c r="M30" s="5" t="n"/>
+      <c r="M30" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N30" s="6" t="n"/>
-      <c r="O30" s="5" t="n"/>
+      <c r="O30" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P30" s="6" t="n"/>
-      <c r="Q30" s="5" t="n"/>
-      <c r="R30" s="5" t="n"/>
+      <c r="Q30" s="5" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="R30" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Presales and Solutions Consultant role at Aspire Systems</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="n"/>
-      <c r="B31" s="5" t="n"/>
-      <c r="C31" s="5" t="n"/>
-      <c r="D31" s="5" t="n"/>
-      <c r="E31" s="5" t="n"/>
-      <c r="F31" s="5" t="n"/>
-      <c r="G31" s="6" t="n"/>
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Louise Scheibner</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>louise.scheibner@columbusglobal.com</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/louisescheibner</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H31" s="5">
         <f>IF(G31="","",TODAY()-G31)</f>
         <v/>
       </c>
-      <c r="I31" s="5" t="n"/>
-      <c r="J31" s="6" t="n"/>
-      <c r="K31" s="5" t="n"/>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J31" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L31" s="6" t="n"/>
-      <c r="M31" s="5" t="n"/>
+      <c r="M31" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N31" s="6" t="n"/>
-      <c r="O31" s="5" t="n"/>
+      <c r="O31" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P31" s="6" t="n"/>
-      <c r="Q31" s="5" t="n"/>
-      <c r="R31" s="5" t="n"/>
+      <c r="Q31" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R31" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Presales &amp; Solutions Consultant role at Columbus</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="n"/>
-      <c r="B32" s="5" t="n"/>
-      <c r="C32" s="5" t="n"/>
-      <c r="D32" s="5" t="n"/>
-      <c r="E32" s="5" t="n"/>
-      <c r="F32" s="5" t="n"/>
-      <c r="G32" s="6" t="n"/>
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Keerthana Subramanian</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>keerthana.s@entomo.co</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/keerthana93</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H32" s="5">
         <f>IF(G32="","",TODAY()-G32)</f>
         <v/>
       </c>
-      <c r="I32" s="5" t="n"/>
-      <c r="J32" s="6" t="n"/>
-      <c r="K32" s="5" t="n"/>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K32" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L32" s="6" t="n"/>
-      <c r="M32" s="5" t="n"/>
+      <c r="M32" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N32" s="6" t="n"/>
-      <c r="O32" s="5" t="n"/>
+      <c r="O32" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P32" s="6" t="n"/>
-      <c r="Q32" s="5" t="n"/>
-      <c r="R32" s="5" t="n"/>
+      <c r="Q32" s="5" t="inlineStr">
+        <is>
+          <t>Gulf (UAE)</t>
+        </is>
+      </c>
+      <c r="R32" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Presales and Solutions Consultant role at entomo</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="n"/>
-      <c r="B33" s="5" t="n"/>
-      <c r="C33" s="5" t="n"/>
-      <c r="D33" s="5" t="n"/>
-      <c r="E33" s="5" t="n"/>
-      <c r="F33" s="5" t="n"/>
-      <c r="G33" s="6" t="n"/>
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Subhabrata Bhattacharya</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>subhabrata.bhattacharya@tcs.com</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/subhabratabhattacharya</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H33" s="5">
         <f>IF(G33="","",TODAY()-G33)</f>
         <v/>
       </c>
-      <c r="I33" s="5" t="n"/>
-      <c r="J33" s="6" t="n"/>
-      <c r="K33" s="5" t="n"/>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L33" s="6" t="n"/>
-      <c r="M33" s="5" t="n"/>
+      <c r="M33" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N33" s="6" t="n"/>
-      <c r="O33" s="5" t="n"/>
+      <c r="O33" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P33" s="6" t="n"/>
-      <c r="Q33" s="5" t="n"/>
-      <c r="R33" s="5" t="n"/>
+      <c r="Q33" s="5" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="R33" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Presales &amp; Solutions Consultant role at Tata Consultancy Services</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="n"/>
-      <c r="B34" s="5" t="n"/>
-      <c r="C34" s="5" t="n"/>
-      <c r="D34" s="5" t="n"/>
-      <c r="E34" s="5" t="n"/>
-      <c r="F34" s="5" t="n"/>
-      <c r="G34" s="6" t="n"/>
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Yuxuan Wang</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>yuxuan1.wang@orangecyberdefense.com</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/yuxuan-wang-2429a9177</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H34" s="5">
         <f>IF(G34="","",TODAY()-G34)</f>
         <v/>
       </c>
-      <c r="I34" s="5" t="n"/>
-      <c r="J34" s="6" t="n"/>
-      <c r="K34" s="5" t="n"/>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J34" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K34" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L34" s="6" t="n"/>
-      <c r="M34" s="5" t="n"/>
+      <c r="M34" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N34" s="6" t="n"/>
-      <c r="O34" s="5" t="n"/>
+      <c r="O34" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P34" s="6" t="n"/>
-      <c r="Q34" s="5" t="n"/>
-      <c r="R34" s="5" t="n"/>
+      <c r="Q34" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R34" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Presales Solutions Consultant, Bid Manager role at Orange Cyberdefense</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="n"/>
-      <c r="B35" s="5" t="n"/>
-      <c r="C35" s="5" t="n"/>
-      <c r="D35" s="5" t="n"/>
-      <c r="E35" s="5" t="n"/>
-      <c r="F35" s="5" t="n"/>
-      <c r="G35" s="6" t="n"/>
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Antoine Demaille</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>antoine.demaille@haiilo.com</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/antoine-demaille-0b7882241</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H35" s="5">
         <f>IF(G35="","",TODAY()-G35)</f>
         <v/>
       </c>
-      <c r="I35" s="5" t="n"/>
-      <c r="J35" s="6" t="n"/>
-      <c r="K35" s="5" t="n"/>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J35" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K35" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L35" s="6" t="n"/>
-      <c r="M35" s="5" t="n"/>
+      <c r="M35" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N35" s="6" t="n"/>
-      <c r="O35" s="5" t="n"/>
+      <c r="O35" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P35" s="6" t="n"/>
-      <c r="Q35" s="5" t="n"/>
-      <c r="R35" s="5" t="n"/>
+      <c r="Q35" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R35" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Account Executive Sales Manager role at Haiilo</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="n"/>
-      <c r="B36" s="5" t="n"/>
-      <c r="C36" s="5" t="n"/>
-      <c r="D36" s="5" t="n"/>
-      <c r="E36" s="5" t="n"/>
-      <c r="F36" s="5" t="n"/>
-      <c r="G36" s="6" t="n"/>
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Buse Sen</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>buse@storyly.io</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/buse-%c5%9fen-aa894417b</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H36" s="5">
         <f>IF(G36="","",TODAY()-G36)</f>
         <v/>
       </c>
-      <c r="I36" s="5" t="n"/>
-      <c r="J36" s="6" t="n"/>
-      <c r="K36" s="5" t="n"/>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J36" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L36" s="6" t="n"/>
-      <c r="M36" s="5" t="n"/>
+      <c r="M36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N36" s="6" t="n"/>
-      <c r="O36" s="5" t="n"/>
+      <c r="O36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P36" s="6" t="n"/>
-      <c r="Q36" s="5" t="n"/>
-      <c r="R36" s="5" t="n"/>
+      <c r="Q36" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="R36" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Account Executive / Sales Manager role at Storyly</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="n"/>
-      <c r="B37" s="5" t="n"/>
-      <c r="C37" s="5" t="n"/>
-      <c r="D37" s="5" t="n"/>
-      <c r="E37" s="5" t="n"/>
-      <c r="F37" s="5" t="n"/>
-      <c r="G37" s="6" t="n"/>
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Stanislav Minikaev</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>stanislav.minikaev@truelab.games</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/stanislav-minikaev-a92912282</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H37" s="5">
         <f>IF(G37="","",TODAY()-G37)</f>
         <v/>
       </c>
-      <c r="I37" s="5" t="n"/>
-      <c r="J37" s="6" t="n"/>
-      <c r="K37" s="5" t="n"/>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J37" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L37" s="6" t="n"/>
-      <c r="M37" s="5" t="n"/>
+      <c r="M37" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N37" s="6" t="n"/>
-      <c r="O37" s="5" t="n"/>
+      <c r="O37" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P37" s="6" t="n"/>
-      <c r="Q37" s="5" t="n"/>
-      <c r="R37" s="5" t="n"/>
+      <c r="Q37" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R37" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Account Executive Sales Manager role at TRUE LABS</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="n"/>
-      <c r="B38" s="5" t="n"/>
-      <c r="C38" s="5" t="n"/>
-      <c r="D38" s="5" t="n"/>
-      <c r="E38" s="5" t="n"/>
-      <c r="F38" s="5" t="n"/>
-      <c r="G38" s="6" t="n"/>
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Shaun Pearson</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>shaun@insure-smart.co.uk</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/shaun-pearson-24294743</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H38" s="5">
         <f>IF(G38="","",TODAY()-G38)</f>
         <v/>
       </c>
-      <c r="I38" s="5" t="n"/>
-      <c r="J38" s="6" t="n"/>
-      <c r="K38" s="5" t="n"/>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J38" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K38" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L38" s="6" t="n"/>
-      <c r="M38" s="5" t="n"/>
+      <c r="M38" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N38" s="6" t="n"/>
-      <c r="O38" s="5" t="n"/>
+      <c r="O38" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P38" s="6" t="n"/>
-      <c r="Q38" s="5" t="n"/>
-      <c r="R38" s="5" t="n"/>
+      <c r="Q38" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R38" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Account Executive &amp; Sales Manager role at Insure Smart Limited</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="n"/>
-      <c r="B39" s="5" t="n"/>
-      <c r="C39" s="5" t="n"/>
-      <c r="D39" s="5" t="n"/>
-      <c r="E39" s="5" t="n"/>
-      <c r="F39" s="5" t="n"/>
-      <c r="G39" s="6" t="n"/>
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Taavi Ruudi</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>taavi.ruudi@cybexer.com</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/taaviruudi</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H39" s="5">
         <f>IF(G39="","",TODAY()-G39)</f>
         <v/>
       </c>
-      <c r="I39" s="5" t="n"/>
-      <c r="J39" s="6" t="n"/>
-      <c r="K39" s="5" t="n"/>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J39" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L39" s="6" t="n"/>
-      <c r="M39" s="5" t="n"/>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N39" s="6" t="n"/>
-      <c r="O39" s="5" t="n"/>
+      <c r="O39" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P39" s="6" t="n"/>
-      <c r="Q39" s="5" t="n"/>
-      <c r="R39" s="5" t="n"/>
+      <c r="Q39" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R39" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Sales Manager / Account Executive role at CybExer Technologies</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="n"/>
-      <c r="B40" s="5" t="n"/>
-      <c r="C40" s="5" t="n"/>
-      <c r="D40" s="5" t="n"/>
-      <c r="E40" s="5" t="n"/>
-      <c r="F40" s="5" t="n"/>
-      <c r="G40" s="6" t="n"/>
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Stefano Carsenzuola</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>stefano.carsenzuola@v-valley.com</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/carse</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H40" s="5">
         <f>IF(G40="","",TODAY()-G40)</f>
         <v/>
       </c>
-      <c r="I40" s="5" t="n"/>
-      <c r="J40" s="6" t="n"/>
-      <c r="K40" s="5" t="n"/>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J40" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K40" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L40" s="6" t="n"/>
-      <c r="M40" s="5" t="n"/>
+      <c r="M40" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N40" s="6" t="n"/>
-      <c r="O40" s="5" t="n"/>
+      <c r="O40" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P40" s="6" t="n"/>
-      <c r="Q40" s="5" t="n"/>
-      <c r="R40" s="5" t="n"/>
+      <c r="Q40" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R40" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Presales Consultant Manager role at V-Valley</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="n"/>
-      <c r="B41" s="5" t="n"/>
-      <c r="C41" s="5" t="n"/>
-      <c r="D41" s="5" t="n"/>
-      <c r="E41" s="5" t="n"/>
-      <c r="F41" s="5" t="n"/>
-      <c r="G41" s="6" t="n"/>
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Nastassia Baravik</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>nb@alconost.com</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/nastassia-baravik</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H41" s="5">
         <f>IF(G41="","",TODAY()-G41)</f>
         <v/>
       </c>
-      <c r="I41" s="5" t="n"/>
-      <c r="J41" s="6" t="n"/>
-      <c r="K41" s="5" t="n"/>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J41" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K41" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L41" s="6" t="n"/>
-      <c r="M41" s="5" t="n"/>
+      <c r="M41" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N41" s="6" t="n"/>
-      <c r="O41" s="5" t="n"/>
+      <c r="O41" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P41" s="6" t="n"/>
-      <c r="Q41" s="5" t="n"/>
-      <c r="R41" s="5" t="n"/>
+      <c r="Q41" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R41" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Sales Manager, Account Executive role at Alconost</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="n"/>
-      <c r="B42" s="5" t="n"/>
-      <c r="C42" s="5" t="n"/>
-      <c r="D42" s="5" t="n"/>
-      <c r="E42" s="5" t="n"/>
-      <c r="F42" s="5" t="n"/>
-      <c r="G42" s="6" t="n"/>
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Romain Le Gousse</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>romain.le@supermetrics.com</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/romain-le-gousse-2a47b31a1</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H42" s="5">
         <f>IF(G42="","",TODAY()-G42)</f>
         <v/>
       </c>
-      <c r="I42" s="5" t="n"/>
-      <c r="J42" s="6" t="n"/>
-      <c r="K42" s="5" t="n"/>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J42" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K42" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L42" s="6" t="n"/>
-      <c r="M42" s="5" t="n"/>
+      <c r="M42" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N42" s="6" t="n"/>
-      <c r="O42" s="5" t="n"/>
+      <c r="O42" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P42" s="6" t="n"/>
-      <c r="Q42" s="5" t="n"/>
-      <c r="R42" s="5" t="n"/>
+      <c r="Q42" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R42" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Account Executive (Sales Executive) role at Supermetrics</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="n"/>
-      <c r="B43" s="5" t="n"/>
-      <c r="C43" s="5" t="n"/>
-      <c r="D43" s="5" t="n"/>
-      <c r="E43" s="5" t="n"/>
-      <c r="F43" s="5" t="n"/>
-      <c r="G43" s="6" t="n"/>
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Krutika Shukla</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>krutika.shukla@hexadroit.com</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/krutika-shukla</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H43" s="5">
         <f>IF(G43="","",TODAY()-G43)</f>
         <v/>
       </c>
-      <c r="I43" s="5" t="n"/>
-      <c r="J43" s="6" t="n"/>
-      <c r="K43" s="5" t="n"/>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J43" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K43" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L43" s="6" t="n"/>
-      <c r="M43" s="5" t="n"/>
+      <c r="M43" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N43" s="6" t="n"/>
-      <c r="O43" s="5" t="n"/>
+      <c r="O43" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P43" s="6" t="n"/>
-      <c r="Q43" s="5" t="n"/>
-      <c r="R43" s="5" t="n"/>
+      <c r="Q43" s="5" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="R43" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Senior Presales Consultant &amp; Solutions Consultant role at Hexadroit Pvt. Ltd.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="n"/>
-      <c r="B44" s="5" t="n"/>
-      <c r="C44" s="5" t="n"/>
-      <c r="D44" s="5" t="n"/>
-      <c r="E44" s="5" t="n"/>
-      <c r="F44" s="5" t="n"/>
-      <c r="G44" s="6" t="n"/>
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Filippo Fazio</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>filippo.fazio@moduline.it</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/filippo-fazio-moduline</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H44" s="5">
         <f>IF(G44="","",TODAY()-G44)</f>
         <v/>
       </c>
-      <c r="I44" s="5" t="n"/>
-      <c r="J44" s="6" t="n"/>
-      <c r="K44" s="5" t="n"/>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J44" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K44" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L44" s="6" t="n"/>
-      <c r="M44" s="5" t="n"/>
+      <c r="M44" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N44" s="6" t="n"/>
-      <c r="O44" s="5" t="n"/>
+      <c r="O44" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P44" s="6" t="n"/>
-      <c r="Q44" s="5" t="n"/>
-      <c r="R44" s="5" t="n"/>
+      <c r="Q44" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R44" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Account Executive Sales Manager role at Moduline s.r.l.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="5" t="n"/>
-      <c r="B45" s="5" t="n"/>
-      <c r="C45" s="5" t="n"/>
-      <c r="D45" s="5" t="n"/>
-      <c r="E45" s="5" t="n"/>
-      <c r="F45" s="5" t="n"/>
-      <c r="G45" s="6" t="n"/>
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Philipp Stoll Franco</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>philipp.stollfranco@boomi.com</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/philipp-stoll-franco-97a348195</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H45" s="5">
         <f>IF(G45="","",TODAY()-G45)</f>
         <v/>
       </c>
-      <c r="I45" s="5" t="n"/>
-      <c r="J45" s="6" t="n"/>
-      <c r="K45" s="5" t="n"/>
+      <c r="I45" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J45" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K45" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L45" s="6" t="n"/>
-      <c r="M45" s="5" t="n"/>
+      <c r="M45" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N45" s="6" t="n"/>
-      <c r="O45" s="5" t="n"/>
+      <c r="O45" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P45" s="6" t="n"/>
-      <c r="Q45" s="5" t="n"/>
-      <c r="R45" s="5" t="n"/>
+      <c r="Q45" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R45" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Commercial Account Manager role at Boomi</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="n"/>
-      <c r="B46" s="5" t="n"/>
-      <c r="C46" s="5" t="n"/>
-      <c r="D46" s="5" t="n"/>
-      <c r="E46" s="5" t="n"/>
-      <c r="F46" s="5" t="n"/>
-      <c r="G46" s="6" t="n"/>
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Benedict Ortmeier</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>benedict.ortmeier@yoummday.com</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/benedict-ortmeier</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H46" s="5">
         <f>IF(G46="","",TODAY()-G46)</f>
         <v/>
       </c>
-      <c r="I46" s="5" t="n"/>
-      <c r="J46" s="6" t="n"/>
-      <c r="K46" s="5" t="n"/>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J46" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K46" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L46" s="6" t="n"/>
-      <c r="M46" s="5" t="n"/>
+      <c r="M46" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N46" s="6" t="n"/>
-      <c r="O46" s="5" t="n"/>
+      <c r="O46" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P46" s="6" t="n"/>
-      <c r="Q46" s="5" t="n"/>
-      <c r="R46" s="5" t="n"/>
+      <c r="Q46" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R46" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Sales Manager / Account Executive role at yoummday</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="n"/>
-      <c r="B47" s="5" t="n"/>
-      <c r="C47" s="5" t="n"/>
-      <c r="D47" s="5" t="n"/>
-      <c r="E47" s="5" t="n"/>
-      <c r="F47" s="5" t="n"/>
-      <c r="G47" s="6" t="n"/>
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Tanishq Saini</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>tanishq.saini@neeyamo.com</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/tanishq-saini24</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H47" s="5">
         <f>IF(G47="","",TODAY()-G47)</f>
         <v/>
       </c>
-      <c r="I47" s="5" t="n"/>
-      <c r="J47" s="6" t="n"/>
-      <c r="K47" s="5" t="n"/>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J47" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K47" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L47" s="6" t="n"/>
-      <c r="M47" s="5" t="n"/>
+      <c r="M47" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N47" s="6" t="n"/>
-      <c r="O47" s="5" t="n"/>
+      <c r="O47" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P47" s="6" t="n"/>
-      <c r="Q47" s="5" t="n"/>
-      <c r="R47" s="5" t="n"/>
+      <c r="Q47" s="5" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="R47" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Account Executive / Enterprise Sales role at Neeyamo</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="5" t="n"/>
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Vinoth Kumar</t>
+        </is>
+      </c>
       <c r="B48" s="5" t="n"/>
-      <c r="C48" s="5" t="n"/>
-      <c r="D48" s="5" t="n"/>
-      <c r="E48" s="5" t="n"/>
-      <c r="F48" s="5" t="n"/>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/vinoth-kumar-332a31114</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="G48" s="6" t="n"/>
       <c r="H48" s="5">
         <f>IF(G48="","",TODAY()-G48)</f>
         <v/>
       </c>
-      <c r="I48" s="5" t="n"/>
-      <c r="J48" s="6" t="n"/>
-      <c r="K48" s="5" t="n"/>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>Send LinkedIn Connection Request</t>
+        </is>
+      </c>
+      <c r="J48" s="6" t="n">
+        <v>46251</v>
+      </c>
+      <c r="K48" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L48" s="6" t="n"/>
-      <c r="M48" s="5" t="n"/>
+      <c r="M48" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N48" s="6" t="n"/>
-      <c r="O48" s="5" t="n"/>
+      <c r="O48" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P48" s="6" t="n"/>
-      <c r="Q48" s="5" t="n"/>
-      <c r="R48" s="5" t="n"/>
+      <c r="Q48" s="5" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="R48" s="5" t="inlineStr">
+        <is>
+          <t>No email available via Apollo enrichment — LinkedIn-only outreach. Hook: Saw your Account Executive Sales Manager role at adidas</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="n"/>
-      <c r="B49" s="5" t="n"/>
-      <c r="C49" s="5" t="n"/>
-      <c r="D49" s="5" t="n"/>
-      <c r="E49" s="5" t="n"/>
-      <c r="F49" s="5" t="n"/>
-      <c r="G49" s="6" t="n"/>
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Magnus Garpedal</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>magnus.garpedal@spandex.se</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/magnus-garpedal-2530a584</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H49" s="5">
         <f>IF(G49="","",TODAY()-G49)</f>
         <v/>
       </c>
-      <c r="I49" s="5" t="n"/>
-      <c r="J49" s="6" t="n"/>
-      <c r="K49" s="5" t="n"/>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J49" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K49" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L49" s="6" t="n"/>
-      <c r="M49" s="5" t="n"/>
+      <c r="M49" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N49" s="6" t="n"/>
-      <c r="O49" s="5" t="n"/>
+      <c r="O49" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P49" s="6" t="n"/>
-      <c r="Q49" s="5" t="n"/>
-      <c r="R49" s="5" t="n"/>
+      <c r="Q49" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R49" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Account Executive Sales Manager role at Spandex Sverige AB</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="n"/>
-      <c r="B50" s="5" t="n"/>
-      <c r="C50" s="5" t="n"/>
-      <c r="D50" s="5" t="n"/>
-      <c r="E50" s="5" t="n"/>
-      <c r="F50" s="5" t="n"/>
-      <c r="G50" s="6" t="n"/>
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Matilda Schwarz</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>matilda.schwarz@kununu.com</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/matilda-schwarz-powerus</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H50" s="5">
         <f>IF(G50="","",TODAY()-G50)</f>
         <v/>
       </c>
-      <c r="I50" s="5" t="n"/>
-      <c r="J50" s="6" t="n"/>
-      <c r="K50" s="5" t="n"/>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J50" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K50" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L50" s="6" t="n"/>
-      <c r="M50" s="5" t="n"/>
+      <c r="M50" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N50" s="6" t="n"/>
-      <c r="O50" s="5" t="n"/>
+      <c r="O50" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P50" s="6" t="n"/>
-      <c r="Q50" s="5" t="n"/>
-      <c r="R50" s="5" t="n"/>
+      <c r="Q50" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R50" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Sales Manager | Account Executive role at kununu</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="n"/>
-      <c r="B51" s="5" t="n"/>
-      <c r="C51" s="5" t="n"/>
-      <c r="D51" s="5" t="n"/>
-      <c r="E51" s="5" t="n"/>
-      <c r="F51" s="5" t="n"/>
-      <c r="G51" s="6" t="n"/>
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Dawid Vosloo</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>dawid.vosloo@dyad.net</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/dawid-vosloo-695396235</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H51" s="5">
         <f>IF(G51="","",TODAY()-G51)</f>
         <v/>
       </c>
-      <c r="I51" s="5" t="n"/>
-      <c r="J51" s="6" t="n"/>
-      <c r="K51" s="5" t="n"/>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J51" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K51" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L51" s="6" t="n"/>
-      <c r="M51" s="5" t="n"/>
+      <c r="M51" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N51" s="6" t="n"/>
-      <c r="O51" s="5" t="n"/>
+      <c r="O51" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P51" s="6" t="n"/>
-      <c r="Q51" s="5" t="n"/>
-      <c r="R51" s="5" t="n"/>
+      <c r="Q51" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R51" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Sales Manager role at Dyad</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="5" t="n"/>
-      <c r="B52" s="5" t="n"/>
-      <c r="C52" s="5" t="n"/>
-      <c r="D52" s="5" t="n"/>
-      <c r="E52" s="5" t="n"/>
-      <c r="F52" s="5" t="n"/>
-      <c r="G52" s="6" t="n"/>
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Steve Herd</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>steven.herd@muckrack.com</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/steven-herd-</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H52" s="5">
         <f>IF(G52="","",TODAY()-G52)</f>
         <v/>
       </c>
-      <c r="I52" s="5" t="n"/>
-      <c r="J52" s="6" t="n"/>
-      <c r="K52" s="5" t="n"/>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J52" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L52" s="6" t="n"/>
-      <c r="M52" s="5" t="n"/>
+      <c r="M52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N52" s="6" t="n"/>
-      <c r="O52" s="5" t="n"/>
+      <c r="O52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P52" s="6" t="n"/>
-      <c r="Q52" s="5" t="n"/>
-      <c r="R52" s="5" t="n"/>
+      <c r="Q52" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R52" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Account Executive | Sales Manager role at Muck Rack</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="5" t="n"/>
-      <c r="B53" s="5" t="n"/>
-      <c r="C53" s="5" t="n"/>
-      <c r="D53" s="5" t="n"/>
-      <c r="E53" s="5" t="n"/>
-      <c r="F53" s="5" t="n"/>
-      <c r="G53" s="6" t="n"/>
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Niklas Kugler</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>n.kugler@arivo.co</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/niklas-kugler-1b6a65224</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G53" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H53" s="5">
         <f>IF(G53="","",TODAY()-G53)</f>
         <v/>
       </c>
-      <c r="I53" s="5" t="n"/>
-      <c r="J53" s="6" t="n"/>
-      <c r="K53" s="5" t="n"/>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J53" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K53" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L53" s="6" t="n"/>
-      <c r="M53" s="5" t="n"/>
+      <c r="M53" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N53" s="6" t="n"/>
-      <c r="O53" s="5" t="n"/>
+      <c r="O53" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P53" s="6" t="n"/>
-      <c r="Q53" s="5" t="n"/>
-      <c r="R53" s="5" t="n"/>
+      <c r="Q53" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R53" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Sales Manager - Account Executive role at Arivo</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="5" t="n"/>
-      <c r="B54" s="5" t="n"/>
-      <c r="C54" s="5" t="n"/>
-      <c r="D54" s="5" t="n"/>
-      <c r="E54" s="5" t="n"/>
-      <c r="F54" s="5" t="n"/>
-      <c r="G54" s="6" t="n"/>
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Arthur Tilleul</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>atilleul@uptoo.fr</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/arthur-tilleul-recrutement-business-uptoo</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H54" s="5">
         <f>IF(G54="","",TODAY()-G54)</f>
         <v/>
       </c>
-      <c r="I54" s="5" t="n"/>
-      <c r="J54" s="6" t="n"/>
-      <c r="K54" s="5" t="n"/>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J54" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K54" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L54" s="6" t="n"/>
-      <c r="M54" s="5" t="n"/>
+      <c r="M54" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N54" s="6" t="n"/>
-      <c r="O54" s="5" t="n"/>
+      <c r="O54" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P54" s="6" t="n"/>
-      <c r="Q54" s="5" t="n"/>
-      <c r="R54" s="5" t="n"/>
+      <c r="Q54" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R54" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Sales Manager - Account Executive role at UPTOO</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="5" t="n"/>
-      <c r="B55" s="5" t="n"/>
-      <c r="C55" s="5" t="n"/>
-      <c r="D55" s="5" t="n"/>
-      <c r="E55" s="5" t="n"/>
-      <c r="F55" s="5" t="n"/>
-      <c r="G55" s="6" t="n"/>
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Andrew Sin</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>andrew.sin@epiuselabs.com</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/andrew-sin</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G55" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H55" s="5">
         <f>IF(G55="","",TODAY()-G55)</f>
         <v/>
       </c>
-      <c r="I55" s="5" t="n"/>
-      <c r="J55" s="6" t="n"/>
-      <c r="K55" s="5" t="n"/>
+      <c r="I55" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J55" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K55" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L55" s="6" t="n"/>
-      <c r="M55" s="5" t="n"/>
+      <c r="M55" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N55" s="6" t="n"/>
-      <c r="O55" s="5" t="n"/>
+      <c r="O55" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P55" s="6" t="n"/>
-      <c r="Q55" s="5" t="n"/>
-      <c r="R55" s="5" t="n"/>
+      <c r="Q55" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R55" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your SAP Partner Sales Manager &amp; Enterprise Account Executive role at EPI-USE Labs</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="5" t="n"/>
-      <c r="B56" s="5" t="n"/>
-      <c r="C56" s="5" t="n"/>
-      <c r="D56" s="5" t="n"/>
-      <c r="E56" s="5" t="n"/>
-      <c r="F56" s="5" t="n"/>
-      <c r="G56" s="6" t="n"/>
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Sam Dinsi</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>sam.dinsi@dyad.net</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/samdinsi</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H56" s="5">
         <f>IF(G56="","",TODAY()-G56)</f>
         <v/>
       </c>
-      <c r="I56" s="5" t="n"/>
-      <c r="J56" s="6" t="n"/>
-      <c r="K56" s="5" t="n"/>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J56" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L56" s="6" t="n"/>
-      <c r="M56" s="5" t="n"/>
+      <c r="M56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N56" s="6" t="n"/>
-      <c r="O56" s="5" t="n"/>
+      <c r="O56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P56" s="6" t="n"/>
-      <c r="Q56" s="5" t="n"/>
-      <c r="R56" s="5" t="n"/>
+      <c r="Q56" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R56" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Sales Manager &amp; Account Executive role at Dyad</t>
+        </is>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" s="5" t="n"/>
-      <c r="B57" s="5" t="n"/>
-      <c r="C57" s="5" t="n"/>
-      <c r="D57" s="5" t="n"/>
-      <c r="E57" s="5" t="n"/>
-      <c r="F57" s="5" t="n"/>
-      <c r="G57" s="6" t="n"/>
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>Jack Pearson</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>jack.pearson@tellimer.com</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/jack-pearson-9a7589221</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G57" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H57" s="5">
         <f>IF(G57="","",TODAY()-G57)</f>
         <v/>
       </c>
-      <c r="I57" s="5" t="n"/>
-      <c r="J57" s="6" t="n"/>
-      <c r="K57" s="5" t="n"/>
+      <c r="I57" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J57" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K57" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L57" s="6" t="n"/>
-      <c r="M57" s="5" t="n"/>
+      <c r="M57" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N57" s="6" t="n"/>
-      <c r="O57" s="5" t="n"/>
+      <c r="O57" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P57" s="6" t="n"/>
-      <c r="Q57" s="5" t="n"/>
-      <c r="R57" s="5" t="n"/>
+      <c r="Q57" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R57" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Sales Manager / Account Executive role at Tellimer</t>
+        </is>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" s="5" t="n"/>
-      <c r="B58" s="5" t="n"/>
-      <c r="C58" s="5" t="n"/>
-      <c r="D58" s="5" t="n"/>
-      <c r="E58" s="5" t="n"/>
-      <c r="F58" s="5" t="n"/>
-      <c r="G58" s="6" t="n"/>
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Stephen Lyons</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>stephen.lyons@42gears.com</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/stephen-lyons-b497a1126</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H58" s="5">
         <f>IF(G58="","",TODAY()-G58)</f>
         <v/>
       </c>
-      <c r="I58" s="5" t="n"/>
-      <c r="J58" s="6" t="n"/>
-      <c r="K58" s="5" t="n"/>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J58" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K58" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L58" s="6" t="n"/>
-      <c r="M58" s="5" t="n"/>
+      <c r="M58" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N58" s="6" t="n"/>
-      <c r="O58" s="5" t="n"/>
+      <c r="O58" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P58" s="6" t="n"/>
-      <c r="Q58" s="5" t="n"/>
-      <c r="R58" s="5" t="n"/>
+      <c r="Q58" s="5" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="R58" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Enterprise Account Manager &amp; Sales Manager role at 42Gears</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="5" t="n"/>
-      <c r="B59" s="5" t="n"/>
-      <c r="C59" s="5" t="n"/>
-      <c r="D59" s="5" t="n"/>
-      <c r="E59" s="5" t="n"/>
-      <c r="F59" s="5" t="n"/>
-      <c r="G59" s="6" t="n"/>
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>Rajeev M</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>rajeev@anakinhq.com</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/rajeevem</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Apollo.io</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Sales &amp; Presales Career Progression</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>Email 1 Sent</t>
+        </is>
+      </c>
+      <c r="G59" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="H59" s="5">
         <f>IF(G59="","",TODAY()-G59)</f>
         <v/>
       </c>
-      <c r="I59" s="5" t="n"/>
-      <c r="J59" s="6" t="n"/>
-      <c r="K59" s="5" t="n"/>
+      <c r="I59" s="5" t="inlineStr">
+        <is>
+          <t>Send Follow-up 1</t>
+        </is>
+      </c>
+      <c r="J59" s="6" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K59" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="L59" s="6" t="n"/>
-      <c r="M59" s="5" t="n"/>
+      <c r="M59" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N59" s="6" t="n"/>
-      <c r="O59" s="5" t="n"/>
+      <c r="O59" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="P59" s="6" t="n"/>
-      <c r="Q59" s="5" t="n"/>
-      <c r="R59" s="5" t="n"/>
+      <c r="Q59" s="5" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="R59" s="5" t="inlineStr">
+        <is>
+          <t>Hook: Saw your Enterprise Sales Manager / Account Executive role at Anakin (YC S21)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n"/>

</xml_diff>

<commit_message>
Record 3 bounces + 1 unsubscribe from this week's Segment A send; neutralize erroneous example-row send
- Magnus Garpedal, Keerthana Subramanian: bounced (address not
  found / recipient unknown), pivoted to LinkedIn.
- Romain Le Gousse: functional bounce (auto-reply "not found in
  our system"), pivoted to LinkedIn.
- Filippo Fazio: unsubscribed, permanently excluded.
- Jane Doe (row 2, the instructional example row) was mistakenly
  emailed live and bounced (jane@example.com, fake domain).
  Neutralized (Next Action = None) and documented so it's never
  picked up again. Root cause fixed in all 3 routine prompts:
  explicit skip rule for row 2, plus broader bounce-detection
  (recognize non-mailer-daemon bounce/rejection formats).
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -635,7 +635,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J2" s="3" t="n">
@@ -655,10 +655,12 @@
       <c r="N2" s="3" t="inlineStr"/>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="P2" s="3" t="inlineStr"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="n">
+        <v>46251</v>
+      </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
           <t>India</t>
@@ -666,7 +668,7 @@
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Met at a webinar in July | Service Interest predates current 4-service taxonomy; treated as closest match (Career Guidance) for Email 1 wording. Overdue row from prior run, swept up by Monday routine 2026-08-17.</t>
+          <t>EXAMPLE ROW, NOT A REAL CONTACT -- accidentally emailed by the automation on 2026-08-17 (jane@example.com bounced, domain not found). Neutralized (Next Action=None) so this never fires again. Root cause fixed in the routine prompt.</t>
         </is>
       </c>
     </row>
@@ -2899,7 +2901,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Bounced</t>
         </is>
       </c>
       <c r="G32" s="6" t="n">
@@ -2911,11 +2913,11 @@
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send LinkedIn Connection Request</t>
         </is>
       </c>
       <c r="J32" s="6" t="n">
-        <v>46253</v>
+        <v>46251</v>
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
@@ -2931,10 +2933,12 @@
       <c r="N32" s="6" t="n"/>
       <c r="O32" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="P32" s="6" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P32" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="Q32" s="5" t="inlineStr">
         <is>
           <t>Gulf (UAE)</t>
@@ -2942,7 +2946,7 @@
       </c>
       <c r="R32" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales and Solutions Consultant role at entomo</t>
+          <t>Hook: Saw your Presales and Solutions Consultant role at entomo | Email bounced 2026-08-17: Recipient Unknown (postmaster@entomo.co). Do not re-email; pivoted to LinkedIn.</t>
         </is>
       </c>
     </row>
@@ -3649,7 +3653,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Bounced</t>
         </is>
       </c>
       <c r="G42" s="6" t="n">
@@ -3661,11 +3665,11 @@
       </c>
       <c r="I42" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send LinkedIn Connection Request</t>
         </is>
       </c>
       <c r="J42" s="6" t="n">
-        <v>46253</v>
+        <v>46251</v>
       </c>
       <c r="K42" s="5" t="inlineStr">
         <is>
@@ -3681,10 +3685,12 @@
       <c r="N42" s="6" t="n"/>
       <c r="O42" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="P42" s="6" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P42" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="Q42" s="5" t="inlineStr">
         <is>
           <t>Europe</t>
@@ -3692,7 +3698,7 @@
       </c>
       <c r="R42" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Account Executive (Sales Executive) role at Supermetrics</t>
+          <t>Hook: Saw your Account Executive (Sales Executive) role at Supermetrics | Email bounced 2026-08-17: auto-reply "email was not found in our system" (supermetrics.com). Do not re-email; pivoted to LinkedIn.</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3805,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Opted Out</t>
         </is>
       </c>
       <c r="G44" s="6" t="n">
@@ -3811,7 +3817,7 @@
       </c>
       <c r="I44" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>None</t>
         </is>
       </c>
       <c r="J44" s="6" t="n">
@@ -3825,10 +3831,12 @@
       <c r="L44" s="6" t="n"/>
       <c r="M44" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N44" s="6" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N44" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="O44" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -3842,7 +3850,7 @@
       </c>
       <c r="R44" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Account Executive Sales Manager role at Moduline s.r.l.</t>
+          <t>Hook: Saw your Account Executive Sales Manager role at Moduline s.r.l. | Replied to Email 1 with Unsubscribe request (received 2026-08-17). Permanently excluded.</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4176,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Bounced</t>
         </is>
       </c>
       <c r="G49" s="6" t="n">
@@ -4180,11 +4188,11 @@
       </c>
       <c r="I49" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send LinkedIn Connection Request</t>
         </is>
       </c>
       <c r="J49" s="6" t="n">
-        <v>46253</v>
+        <v>46251</v>
       </c>
       <c r="K49" s="5" t="inlineStr">
         <is>
@@ -4200,10 +4208,12 @@
       <c r="N49" s="6" t="n"/>
       <c r="O49" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="P49" s="6" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P49" s="6" t="n">
+        <v>46251</v>
+      </c>
       <c r="Q49" s="5" t="inlineStr">
         <is>
           <t>Europe</t>
@@ -4211,7 +4221,7 @@
       </c>
       <c r="R49" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Account Executive Sales Manager role at Spandex Sverige AB</t>
+          <t>Hook: Saw your Account Executive Sales Manager role at Spandex Sverige AB | Email bounced 2026-08-17: address not found (mailer-daemon). Do not re-email; pivoted to LinkedIn.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wednesday follow-up run: send Follow-up 1 to 39 due contacts
No new bounces, opt-outs, or bookings since Monday's run (all previously
recorded). Sent Follow-up 1 (threaded reply) to every contact with
Stage=Email 1 Sent and Next Action Date <= today; advanced each to
Follow-up 1 Sent with Next Action Date set to Friday. No Follow-up 2/4
rows existed yet, so nothing was due for Follow-up 3. Jane Doe example
row and all Bounced/Opted Out/Booked rows were skipped per the
permanent exclusion rules.

Note: LibreOffice recalculation is broken in this environment (even
trivial file conversions fail to load), so the Days Since Contact
formula column was not recalculated in-place; it will recompute
normally the next time the file is opened in Excel or Sheets.
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -772,13 +772,11 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
+          <t>Follow-up 1 Sent</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="H4" s="5">
         <f>IF(G4="","",TODAY()-G4)</f>
@@ -786,11 +784,11 @@
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J4" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
@@ -849,13 +847,11 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
+          <t>Follow-up 1 Sent</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="H5" s="5">
         <f>IF(G5="","",TODAY()-G5)</f>
@@ -863,11 +859,11 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J5" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
@@ -926,13 +922,11 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
+          <t>Follow-up 1 Sent</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="H6" s="5">
         <f>IF(G6="","",TODAY()-G6)</f>
@@ -940,11 +934,11 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J6" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
@@ -1003,13 +997,11 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
+          <t>Follow-up 1 Sent</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="H7" s="5">
         <f>IF(G7="","",TODAY()-G7)</f>
@@ -1017,11 +1009,11 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J7" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
@@ -1159,13 +1151,11 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
+          <t>Follow-up 1 Sent</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="H9" s="5">
         <f>IF(G9="","",TODAY()-G9)</f>
@@ -1173,11 +1163,11 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J9" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
@@ -1311,13 +1301,11 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
+          <t>Follow-up 1 Sent</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="H11" s="5">
         <f>IF(G11="","",TODAY()-G11)</f>
@@ -1325,11 +1313,11 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J11" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
@@ -1388,13 +1376,11 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
+          <t>Follow-up 1 Sent</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="H12" s="5">
         <f>IF(G12="","",TODAY()-G12)</f>
@@ -1402,11 +1388,11 @@
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J12" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
@@ -1544,13 +1530,11 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
+          <t>Follow-up 1 Sent</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="H14" s="5">
         <f>IF(G14="","",TODAY()-G14)</f>
@@ -1558,11 +1542,11 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J14" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
@@ -1621,13 +1605,11 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
+          <t>Follow-up 1 Sent</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="H15" s="5">
         <f>IF(G15="","",TODAY()-G15)</f>
@@ -1635,11 +1617,11 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J15" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
@@ -2006,13 +1988,11 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
+          <t>Follow-up 1 Sent</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="H20" s="5">
         <f>IF(G20="","",TODAY()-G20)</f>
@@ -2020,11 +2000,11 @@
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J20" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
@@ -2160,13 +2140,11 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
+          <t>Follow-up 1 Sent</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="H22" s="5">
         <f>IF(G22="","",TODAY()-G22)</f>
@@ -2174,11 +2152,11 @@
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J22" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
@@ -2525,13 +2503,11 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
+          <t>Follow-up 1 Sent</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="n">
+        <v>46253</v>
       </c>
       <c r="H27" s="5">
         <f>IF(G27="","",TODAY()-G27)</f>
@@ -2539,11 +2515,11 @@
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J27" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
@@ -2602,11 +2578,11 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G28" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H28" s="5">
         <f>IF(G28="","",TODAY()-G28)</f>
@@ -2614,11 +2590,11 @@
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J28" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
@@ -2677,11 +2653,11 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G29" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H29" s="5">
         <f>IF(G29="","",TODAY()-G29)</f>
@@ -2689,11 +2665,11 @@
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J29" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K29" s="5" t="inlineStr">
         <is>
@@ -2752,11 +2728,11 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G30" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H30" s="5">
         <f>IF(G30="","",TODAY()-G30)</f>
@@ -2764,11 +2740,11 @@
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J30" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
@@ -2827,11 +2803,11 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G31" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H31" s="5">
         <f>IF(G31="","",TODAY()-G31)</f>
@@ -2839,11 +2815,11 @@
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J31" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K31" s="5" t="inlineStr">
         <is>
@@ -2979,11 +2955,11 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G33" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H33" s="5">
         <f>IF(G33="","",TODAY()-G33)</f>
@@ -2991,11 +2967,11 @@
       </c>
       <c r="I33" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J33" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K33" s="5" t="inlineStr">
         <is>
@@ -3054,11 +3030,11 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G34" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H34" s="5">
         <f>IF(G34="","",TODAY()-G34)</f>
@@ -3066,11 +3042,11 @@
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J34" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
@@ -3129,11 +3105,11 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G35" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H35" s="5">
         <f>IF(G35="","",TODAY()-G35)</f>
@@ -3141,11 +3117,11 @@
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J35" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K35" s="5" t="inlineStr">
         <is>
@@ -3204,11 +3180,11 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G36" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H36" s="5">
         <f>IF(G36="","",TODAY()-G36)</f>
@@ -3216,11 +3192,11 @@
       </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J36" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K36" s="5" t="inlineStr">
         <is>
@@ -3279,11 +3255,11 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G37" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H37" s="5">
         <f>IF(G37="","",TODAY()-G37)</f>
@@ -3291,11 +3267,11 @@
       </c>
       <c r="I37" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J37" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K37" s="5" t="inlineStr">
         <is>
@@ -3354,11 +3330,11 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G38" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H38" s="5">
         <f>IF(G38="","",TODAY()-G38)</f>
@@ -3366,11 +3342,11 @@
       </c>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J38" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K38" s="5" t="inlineStr">
         <is>
@@ -3429,11 +3405,11 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G39" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H39" s="5">
         <f>IF(G39="","",TODAY()-G39)</f>
@@ -3441,11 +3417,11 @@
       </c>
       <c r="I39" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J39" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K39" s="5" t="inlineStr">
         <is>
@@ -3504,11 +3480,11 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G40" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H40" s="5">
         <f>IF(G40="","",TODAY()-G40)</f>
@@ -3516,11 +3492,11 @@
       </c>
       <c r="I40" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J40" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K40" s="5" t="inlineStr">
         <is>
@@ -3579,11 +3555,11 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G41" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H41" s="5">
         <f>IF(G41="","",TODAY()-G41)</f>
@@ -3591,11 +3567,11 @@
       </c>
       <c r="I41" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J41" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K41" s="5" t="inlineStr">
         <is>
@@ -3731,11 +3707,11 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G43" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H43" s="5">
         <f>IF(G43="","",TODAY()-G43)</f>
@@ -3743,11 +3719,11 @@
       </c>
       <c r="I43" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J43" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K43" s="5" t="inlineStr">
         <is>
@@ -3883,11 +3859,11 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G45" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H45" s="5">
         <f>IF(G45="","",TODAY()-G45)</f>
@@ -3895,11 +3871,11 @@
       </c>
       <c r="I45" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J45" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K45" s="5" t="inlineStr">
         <is>
@@ -3958,11 +3934,11 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G46" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H46" s="5">
         <f>IF(G46="","",TODAY()-G46)</f>
@@ -3970,11 +3946,11 @@
       </c>
       <c r="I46" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J46" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K46" s="5" t="inlineStr">
         <is>
@@ -4033,11 +4009,11 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G47" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H47" s="5">
         <f>IF(G47="","",TODAY()-G47)</f>
@@ -4045,11 +4021,11 @@
       </c>
       <c r="I47" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J47" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K47" s="5" t="inlineStr">
         <is>
@@ -4254,11 +4230,11 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G50" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H50" s="5">
         <f>IF(G50="","",TODAY()-G50)</f>
@@ -4266,11 +4242,11 @@
       </c>
       <c r="I50" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J50" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K50" s="5" t="inlineStr">
         <is>
@@ -4329,11 +4305,11 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G51" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H51" s="5">
         <f>IF(G51="","",TODAY()-G51)</f>
@@ -4341,11 +4317,11 @@
       </c>
       <c r="I51" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J51" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K51" s="5" t="inlineStr">
         <is>
@@ -4404,11 +4380,11 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G52" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H52" s="5">
         <f>IF(G52="","",TODAY()-G52)</f>
@@ -4416,11 +4392,11 @@
       </c>
       <c r="I52" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J52" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K52" s="5" t="inlineStr">
         <is>
@@ -4479,11 +4455,11 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G53" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H53" s="5">
         <f>IF(G53="","",TODAY()-G53)</f>
@@ -4491,11 +4467,11 @@
       </c>
       <c r="I53" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J53" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K53" s="5" t="inlineStr">
         <is>
@@ -4554,11 +4530,11 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G54" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H54" s="5">
         <f>IF(G54="","",TODAY()-G54)</f>
@@ -4566,11 +4542,11 @@
       </c>
       <c r="I54" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J54" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K54" s="5" t="inlineStr">
         <is>
@@ -4629,11 +4605,11 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G55" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H55" s="5">
         <f>IF(G55="","",TODAY()-G55)</f>
@@ -4641,11 +4617,11 @@
       </c>
       <c r="I55" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J55" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K55" s="5" t="inlineStr">
         <is>
@@ -4704,11 +4680,11 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G56" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H56" s="5">
         <f>IF(G56="","",TODAY()-G56)</f>
@@ -4716,11 +4692,11 @@
       </c>
       <c r="I56" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J56" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K56" s="5" t="inlineStr">
         <is>
@@ -4779,11 +4755,11 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G57" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H57" s="5">
         <f>IF(G57="","",TODAY()-G57)</f>
@@ -4791,11 +4767,11 @@
       </c>
       <c r="I57" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J57" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K57" s="5" t="inlineStr">
         <is>
@@ -4854,11 +4830,11 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G58" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H58" s="5">
         <f>IF(G58="","",TODAY()-G58)</f>
@@ -4866,11 +4842,11 @@
       </c>
       <c r="I58" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J58" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K58" s="5" t="inlineStr">
         <is>
@@ -4929,11 +4905,11 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G59" s="6" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="H59" s="5">
         <f>IF(G59="","",TODAY()-G59)</f>
@@ -4941,11 +4917,11 @@
       </c>
       <c r="I59" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J59" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="K59" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Friday follow-up run: send Follow-up 2 to 39 due contacts
Sent Follow-up 2 (different-angle email) to all contacts whose Stage was
"Follow-up 1 Sent" and Next Action Date <= 2026-08-21, threaded as replies
to their Wednesday Follow-up 1 message. No bounces, opt-outs, or bookings
detected in Gmail since Wednesday's run. No Follow-up 3 Sent rows existed
yet, so no Follow-up 4 sends this run.
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -772,11 +772,11 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G4" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H4" s="5">
         <f>IF(G4="","",TODAY()-G4)</f>
@@ -784,11 +784,11 @@
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J4" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
@@ -847,11 +847,11 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G5" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H5" s="5">
         <f>IF(G5="","",TODAY()-G5)</f>
@@ -859,11 +859,11 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J5" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
@@ -922,11 +922,11 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G6" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H6" s="5">
         <f>IF(G6="","",TODAY()-G6)</f>
@@ -934,11 +934,11 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J6" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
@@ -997,11 +997,11 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G7" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H7" s="5">
         <f>IF(G7="","",TODAY()-G7)</f>
@@ -1009,11 +1009,11 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J7" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
@@ -1151,11 +1151,11 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H9" s="5">
         <f>IF(G9="","",TODAY()-G9)</f>
@@ -1163,11 +1163,11 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J9" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
@@ -1301,11 +1301,11 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G11" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H11" s="5">
         <f>IF(G11="","",TODAY()-G11)</f>
@@ -1313,11 +1313,11 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J11" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
@@ -1376,11 +1376,11 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G12" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H12" s="5">
         <f>IF(G12="","",TODAY()-G12)</f>
@@ -1388,11 +1388,11 @@
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J12" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
@@ -1530,11 +1530,11 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G14" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H14" s="5">
         <f>IF(G14="","",TODAY()-G14)</f>
@@ -1542,11 +1542,11 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J14" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
@@ -1605,11 +1605,11 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G15" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H15" s="5">
         <f>IF(G15="","",TODAY()-G15)</f>
@@ -1617,11 +1617,11 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J15" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
@@ -1988,11 +1988,11 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G20" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H20" s="5">
         <f>IF(G20="","",TODAY()-G20)</f>
@@ -2000,11 +2000,11 @@
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J20" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
@@ -2140,11 +2140,11 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G22" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H22" s="5">
         <f>IF(G22="","",TODAY()-G22)</f>
@@ -2152,11 +2152,11 @@
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J22" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
@@ -2503,11 +2503,11 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G27" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H27" s="5">
         <f>IF(G27="","",TODAY()-G27)</f>
@@ -2515,11 +2515,11 @@
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J27" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
@@ -2578,11 +2578,11 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G28" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H28" s="5">
         <f>IF(G28="","",TODAY()-G28)</f>
@@ -2590,11 +2590,11 @@
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J28" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
@@ -2653,11 +2653,11 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G29" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H29" s="5">
         <f>IF(G29="","",TODAY()-G29)</f>
@@ -2665,11 +2665,11 @@
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J29" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K29" s="5" t="inlineStr">
         <is>
@@ -2728,11 +2728,11 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G30" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H30" s="5">
         <f>IF(G30="","",TODAY()-G30)</f>
@@ -2740,11 +2740,11 @@
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J30" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
@@ -2803,11 +2803,11 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G31" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H31" s="5">
         <f>IF(G31="","",TODAY()-G31)</f>
@@ -2815,11 +2815,11 @@
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J31" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K31" s="5" t="inlineStr">
         <is>
@@ -2955,11 +2955,11 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G33" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H33" s="5">
         <f>IF(G33="","",TODAY()-G33)</f>
@@ -2967,11 +2967,11 @@
       </c>
       <c r="I33" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J33" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K33" s="5" t="inlineStr">
         <is>
@@ -3030,11 +3030,11 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G34" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H34" s="5">
         <f>IF(G34="","",TODAY()-G34)</f>
@@ -3042,11 +3042,11 @@
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J34" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
@@ -3105,11 +3105,11 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G35" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H35" s="5">
         <f>IF(G35="","",TODAY()-G35)</f>
@@ -3117,11 +3117,11 @@
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J35" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K35" s="5" t="inlineStr">
         <is>
@@ -3180,11 +3180,11 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G36" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H36" s="5">
         <f>IF(G36="","",TODAY()-G36)</f>
@@ -3192,11 +3192,11 @@
       </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J36" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K36" s="5" t="inlineStr">
         <is>
@@ -3255,11 +3255,11 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G37" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H37" s="5">
         <f>IF(G37="","",TODAY()-G37)</f>
@@ -3267,11 +3267,11 @@
       </c>
       <c r="I37" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J37" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K37" s="5" t="inlineStr">
         <is>
@@ -3330,11 +3330,11 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G38" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H38" s="5">
         <f>IF(G38="","",TODAY()-G38)</f>
@@ -3342,11 +3342,11 @@
       </c>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J38" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K38" s="5" t="inlineStr">
         <is>
@@ -3405,11 +3405,11 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G39" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H39" s="5">
         <f>IF(G39="","",TODAY()-G39)</f>
@@ -3417,11 +3417,11 @@
       </c>
       <c r="I39" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J39" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K39" s="5" t="inlineStr">
         <is>
@@ -3480,11 +3480,11 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G40" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H40" s="5">
         <f>IF(G40="","",TODAY()-G40)</f>
@@ -3492,11 +3492,11 @@
       </c>
       <c r="I40" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J40" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K40" s="5" t="inlineStr">
         <is>
@@ -3555,11 +3555,11 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G41" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H41" s="5">
         <f>IF(G41="","",TODAY()-G41)</f>
@@ -3567,11 +3567,11 @@
       </c>
       <c r="I41" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J41" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K41" s="5" t="inlineStr">
         <is>
@@ -3707,11 +3707,11 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G43" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H43" s="5">
         <f>IF(G43="","",TODAY()-G43)</f>
@@ -3719,11 +3719,11 @@
       </c>
       <c r="I43" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J43" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K43" s="5" t="inlineStr">
         <is>
@@ -3859,11 +3859,11 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G45" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H45" s="5">
         <f>IF(G45="","",TODAY()-G45)</f>
@@ -3871,11 +3871,11 @@
       </c>
       <c r="I45" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J45" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K45" s="5" t="inlineStr">
         <is>
@@ -3934,11 +3934,11 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G46" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H46" s="5">
         <f>IF(G46="","",TODAY()-G46)</f>
@@ -3946,11 +3946,11 @@
       </c>
       <c r="I46" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J46" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K46" s="5" t="inlineStr">
         <is>
@@ -4009,11 +4009,11 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G47" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H47" s="5">
         <f>IF(G47="","",TODAY()-G47)</f>
@@ -4021,11 +4021,11 @@
       </c>
       <c r="I47" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J47" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K47" s="5" t="inlineStr">
         <is>
@@ -4230,11 +4230,11 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G50" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H50" s="5">
         <f>IF(G50="","",TODAY()-G50)</f>
@@ -4242,11 +4242,11 @@
       </c>
       <c r="I50" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J50" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K50" s="5" t="inlineStr">
         <is>
@@ -4305,11 +4305,11 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G51" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H51" s="5">
         <f>IF(G51="","",TODAY()-G51)</f>
@@ -4317,11 +4317,11 @@
       </c>
       <c r="I51" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J51" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K51" s="5" t="inlineStr">
         <is>
@@ -4380,11 +4380,11 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G52" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H52" s="5">
         <f>IF(G52="","",TODAY()-G52)</f>
@@ -4392,11 +4392,11 @@
       </c>
       <c r="I52" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J52" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K52" s="5" t="inlineStr">
         <is>
@@ -4455,11 +4455,11 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G53" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H53" s="5">
         <f>IF(G53="","",TODAY()-G53)</f>
@@ -4467,11 +4467,11 @@
       </c>
       <c r="I53" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J53" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K53" s="5" t="inlineStr">
         <is>
@@ -4530,11 +4530,11 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G54" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H54" s="5">
         <f>IF(G54="","",TODAY()-G54)</f>
@@ -4542,11 +4542,11 @@
       </c>
       <c r="I54" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J54" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K54" s="5" t="inlineStr">
         <is>
@@ -4605,11 +4605,11 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G55" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H55" s="5">
         <f>IF(G55="","",TODAY()-G55)</f>
@@ -4617,11 +4617,11 @@
       </c>
       <c r="I55" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J55" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K55" s="5" t="inlineStr">
         <is>
@@ -4680,11 +4680,11 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G56" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H56" s="5">
         <f>IF(G56="","",TODAY()-G56)</f>
@@ -4692,11 +4692,11 @@
       </c>
       <c r="I56" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J56" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K56" s="5" t="inlineStr">
         <is>
@@ -4755,11 +4755,11 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G57" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H57" s="5">
         <f>IF(G57="","",TODAY()-G57)</f>
@@ -4767,11 +4767,11 @@
       </c>
       <c r="I57" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J57" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K57" s="5" t="inlineStr">
         <is>
@@ -4830,11 +4830,11 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G58" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H58" s="5">
         <f>IF(G58="","",TODAY()-G58)</f>
@@ -4842,11 +4842,11 @@
       </c>
       <c r="I58" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J58" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K58" s="5" t="inlineStr">
         <is>
@@ -4905,11 +4905,11 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G59" s="6" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="H59" s="5">
         <f>IF(G59="","",TODAY()-G59)</f>
@@ -4917,11 +4917,11 @@
       </c>
       <c r="I59" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J59" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="K59" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Wednesday follow-up run: send Follow-up 3 to 39 due contacts
Sent Follow-up 3 (short check-in) to all contacts whose Stage was
"Follow-up 2 Sent" and Next Action Date <= 2026-08-26, threaded as replies
into their existing Gmail conversations. No bounces, opt-outs, or bookings
detected in Gmail since Monday's run. No Email 1 Sent rows were due for
Follow-up 1 this run.
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -772,11 +772,11 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G4" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H4" s="5">
         <f>IF(G4="","",TODAY()-G4)</f>
@@ -784,11 +784,11 @@
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J4" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
@@ -847,11 +847,11 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G5" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H5" s="5">
         <f>IF(G5="","",TODAY()-G5)</f>
@@ -859,11 +859,11 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J5" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
@@ -922,11 +922,11 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G6" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H6" s="5">
         <f>IF(G6="","",TODAY()-G6)</f>
@@ -934,11 +934,11 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J6" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
@@ -997,11 +997,11 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G7" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H7" s="5">
         <f>IF(G7="","",TODAY()-G7)</f>
@@ -1009,11 +1009,11 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J7" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
@@ -1151,11 +1151,11 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H9" s="5">
         <f>IF(G9="","",TODAY()-G9)</f>
@@ -1163,11 +1163,11 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J9" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
@@ -1301,11 +1301,11 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G11" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H11" s="5">
         <f>IF(G11="","",TODAY()-G11)</f>
@@ -1313,11 +1313,11 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J11" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
@@ -1376,11 +1376,11 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G12" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H12" s="5">
         <f>IF(G12="","",TODAY()-G12)</f>
@@ -1388,11 +1388,11 @@
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J12" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
@@ -1530,11 +1530,11 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G14" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H14" s="5">
         <f>IF(G14="","",TODAY()-G14)</f>
@@ -1542,11 +1542,11 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J14" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
@@ -1605,11 +1605,11 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G15" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H15" s="5">
         <f>IF(G15="","",TODAY()-G15)</f>
@@ -1617,11 +1617,11 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J15" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
@@ -1988,11 +1988,11 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G20" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H20" s="5">
         <f>IF(G20="","",TODAY()-G20)</f>
@@ -2000,11 +2000,11 @@
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J20" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
@@ -2140,11 +2140,11 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G22" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H22" s="5">
         <f>IF(G22="","",TODAY()-G22)</f>
@@ -2152,11 +2152,11 @@
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J22" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
@@ -2503,11 +2503,11 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G27" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H27" s="5">
         <f>IF(G27="","",TODAY()-G27)</f>
@@ -2515,11 +2515,11 @@
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J27" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
@@ -2578,11 +2578,11 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G28" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H28" s="5">
         <f>IF(G28="","",TODAY()-G28)</f>
@@ -2590,11 +2590,11 @@
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J28" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
@@ -2653,11 +2653,11 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G29" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H29" s="5">
         <f>IF(G29="","",TODAY()-G29)</f>
@@ -2665,11 +2665,11 @@
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J29" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K29" s="5" t="inlineStr">
         <is>
@@ -2728,11 +2728,11 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G30" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H30" s="5">
         <f>IF(G30="","",TODAY()-G30)</f>
@@ -2740,11 +2740,11 @@
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J30" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
@@ -2803,11 +2803,11 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G31" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H31" s="5">
         <f>IF(G31="","",TODAY()-G31)</f>
@@ -2815,11 +2815,11 @@
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J31" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K31" s="5" t="inlineStr">
         <is>
@@ -2955,11 +2955,11 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G33" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H33" s="5">
         <f>IF(G33="","",TODAY()-G33)</f>
@@ -2967,11 +2967,11 @@
       </c>
       <c r="I33" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J33" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K33" s="5" t="inlineStr">
         <is>
@@ -3030,11 +3030,11 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G34" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H34" s="5">
         <f>IF(G34="","",TODAY()-G34)</f>
@@ -3042,11 +3042,11 @@
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J34" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
@@ -3105,11 +3105,11 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G35" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H35" s="5">
         <f>IF(G35="","",TODAY()-G35)</f>
@@ -3117,11 +3117,11 @@
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J35" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K35" s="5" t="inlineStr">
         <is>
@@ -3180,11 +3180,11 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G36" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H36" s="5">
         <f>IF(G36="","",TODAY()-G36)</f>
@@ -3192,11 +3192,11 @@
       </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J36" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K36" s="5" t="inlineStr">
         <is>
@@ -3255,11 +3255,11 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G37" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H37" s="5">
         <f>IF(G37="","",TODAY()-G37)</f>
@@ -3267,11 +3267,11 @@
       </c>
       <c r="I37" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J37" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K37" s="5" t="inlineStr">
         <is>
@@ -3330,11 +3330,11 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G38" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H38" s="5">
         <f>IF(G38="","",TODAY()-G38)</f>
@@ -3342,11 +3342,11 @@
       </c>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J38" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K38" s="5" t="inlineStr">
         <is>
@@ -3405,11 +3405,11 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G39" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H39" s="5">
         <f>IF(G39="","",TODAY()-G39)</f>
@@ -3417,11 +3417,11 @@
       </c>
       <c r="I39" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J39" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K39" s="5" t="inlineStr">
         <is>
@@ -3480,11 +3480,11 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G40" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H40" s="5">
         <f>IF(G40="","",TODAY()-G40)</f>
@@ -3492,11 +3492,11 @@
       </c>
       <c r="I40" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J40" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K40" s="5" t="inlineStr">
         <is>
@@ -3555,11 +3555,11 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G41" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H41" s="5">
         <f>IF(G41="","",TODAY()-G41)</f>
@@ -3567,11 +3567,11 @@
       </c>
       <c r="I41" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J41" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K41" s="5" t="inlineStr">
         <is>
@@ -3707,11 +3707,11 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G43" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H43" s="5">
         <f>IF(G43="","",TODAY()-G43)</f>
@@ -3719,11 +3719,11 @@
       </c>
       <c r="I43" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J43" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K43" s="5" t="inlineStr">
         <is>
@@ -3859,11 +3859,11 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G45" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H45" s="5">
         <f>IF(G45="","",TODAY()-G45)</f>
@@ -3871,11 +3871,11 @@
       </c>
       <c r="I45" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J45" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K45" s="5" t="inlineStr">
         <is>
@@ -3934,11 +3934,11 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G46" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H46" s="5">
         <f>IF(G46="","",TODAY()-G46)</f>
@@ -3946,11 +3946,11 @@
       </c>
       <c r="I46" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J46" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K46" s="5" t="inlineStr">
         <is>
@@ -4009,11 +4009,11 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G47" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H47" s="5">
         <f>IF(G47="","",TODAY()-G47)</f>
@@ -4021,11 +4021,11 @@
       </c>
       <c r="I47" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J47" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K47" s="5" t="inlineStr">
         <is>
@@ -4230,11 +4230,11 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G50" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H50" s="5">
         <f>IF(G50="","",TODAY()-G50)</f>
@@ -4242,11 +4242,11 @@
       </c>
       <c r="I50" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J50" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K50" s="5" t="inlineStr">
         <is>
@@ -4305,11 +4305,11 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G51" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H51" s="5">
         <f>IF(G51="","",TODAY()-G51)</f>
@@ -4317,11 +4317,11 @@
       </c>
       <c r="I51" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J51" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K51" s="5" t="inlineStr">
         <is>
@@ -4380,11 +4380,11 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G52" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H52" s="5">
         <f>IF(G52="","",TODAY()-G52)</f>
@@ -4392,11 +4392,11 @@
       </c>
       <c r="I52" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J52" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K52" s="5" t="inlineStr">
         <is>
@@ -4455,11 +4455,11 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G53" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H53" s="5">
         <f>IF(G53="","",TODAY()-G53)</f>
@@ -4467,11 +4467,11 @@
       </c>
       <c r="I53" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J53" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K53" s="5" t="inlineStr">
         <is>
@@ -4530,11 +4530,11 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G54" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H54" s="5">
         <f>IF(G54="","",TODAY()-G54)</f>
@@ -4542,11 +4542,11 @@
       </c>
       <c r="I54" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J54" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K54" s="5" t="inlineStr">
         <is>
@@ -4605,11 +4605,11 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G55" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H55" s="5">
         <f>IF(G55="","",TODAY()-G55)</f>
@@ -4617,11 +4617,11 @@
       </c>
       <c r="I55" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J55" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K55" s="5" t="inlineStr">
         <is>
@@ -4680,11 +4680,11 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G56" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H56" s="5">
         <f>IF(G56="","",TODAY()-G56)</f>
@@ -4692,11 +4692,11 @@
       </c>
       <c r="I56" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J56" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K56" s="5" t="inlineStr">
         <is>
@@ -4755,11 +4755,11 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G57" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H57" s="5">
         <f>IF(G57="","",TODAY()-G57)</f>
@@ -4767,11 +4767,11 @@
       </c>
       <c r="I57" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J57" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K57" s="5" t="inlineStr">
         <is>
@@ -4830,11 +4830,11 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G58" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H58" s="5">
         <f>IF(G58="","",TODAY()-G58)</f>
@@ -4842,11 +4842,11 @@
       </c>
       <c r="I58" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J58" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K58" s="5" t="inlineStr">
         <is>
@@ -4905,11 +4905,11 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 2 Sent</t>
+          <t>Follow-up 3 Sent</t>
         </is>
       </c>
       <c r="G59" s="6" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="H59" s="5">
         <f>IF(G59="","",TODAY()-G59)</f>
@@ -4917,11 +4917,11 @@
       </c>
       <c r="I59" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 3</t>
+          <t>Send Follow-up 4</t>
         </is>
       </c>
       <c r="J59" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K59" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Friday follow-up run: send Follow-up 4 to 39 due contacts
Final touch in the 5-email sequence, sent to the cohort that received
Follow-up 3 on Wednesday. No bounces, opt-outs, or bookings detected
this run.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014PfKLEXLnmtU1RM423u5pq
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -772,11 +772,11 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G4" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H4" s="5">
         <f>IF(G4="","",TODAY()-G4)</f>
@@ -784,12 +784,10 @@
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J4" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="n"/>
       <c r="K4" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -815,7 +813,7 @@
       </c>
       <c r="R4" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -847,11 +845,11 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G5" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H5" s="5">
         <f>IF(G5="","",TODAY()-G5)</f>
@@ -859,12 +857,10 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="n"/>
       <c r="K5" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -890,7 +886,7 @@
       </c>
       <c r="R5" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -922,11 +918,11 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G6" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H6" s="5">
         <f>IF(G6="","",TODAY()-G6)</f>
@@ -934,12 +930,10 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J6" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="n"/>
       <c r="K6" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -965,7 +959,7 @@
       </c>
       <c r="R6" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -997,11 +991,11 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G7" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H7" s="5">
         <f>IF(G7="","",TODAY()-G7)</f>
@@ -1009,12 +1003,10 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="n"/>
       <c r="K7" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -1040,7 +1032,7 @@
       </c>
       <c r="R7" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -1151,11 +1143,11 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H9" s="5">
         <f>IF(G9="","",TODAY()-G9)</f>
@@ -1163,12 +1155,10 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J9" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="n"/>
       <c r="K9" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -1194,7 +1184,7 @@
       </c>
       <c r="R9" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -1301,11 +1291,11 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G11" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H11" s="5">
         <f>IF(G11="","",TODAY()-G11)</f>
@@ -1313,12 +1303,10 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J11" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="n"/>
       <c r="K11" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -1344,7 +1332,7 @@
       </c>
       <c r="R11" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -1376,11 +1364,11 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G12" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H12" s="5">
         <f>IF(G12="","",TODAY()-G12)</f>
@@ -1388,12 +1376,10 @@
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J12" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="n"/>
       <c r="K12" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -1419,7 +1405,7 @@
       </c>
       <c r="R12" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -1530,11 +1516,11 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G14" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H14" s="5">
         <f>IF(G14="","",TODAY()-G14)</f>
@@ -1542,12 +1528,10 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J14" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="n"/>
       <c r="K14" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -1573,7 +1557,7 @@
       </c>
       <c r="R14" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -1605,11 +1589,11 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G15" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H15" s="5">
         <f>IF(G15="","",TODAY()-G15)</f>
@@ -1617,12 +1601,10 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J15" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="n"/>
       <c r="K15" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -1648,7 +1630,7 @@
       </c>
       <c r="R15" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -1988,11 +1970,11 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G20" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H20" s="5">
         <f>IF(G20="","",TODAY()-G20)</f>
@@ -2000,12 +1982,10 @@
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J20" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="n"/>
       <c r="K20" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -2031,7 +2011,7 @@
       </c>
       <c r="R20" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -2140,11 +2120,11 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G22" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H22" s="5">
         <f>IF(G22="","",TODAY()-G22)</f>
@@ -2152,12 +2132,10 @@
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J22" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="n"/>
       <c r="K22" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -2183,7 +2161,7 @@
       </c>
       <c r="R22" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -2503,11 +2481,11 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G27" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H27" s="5">
         <f>IF(G27="","",TODAY()-G27)</f>
@@ -2515,12 +2493,10 @@
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J27" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J27" s="6" t="n"/>
       <c r="K27" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -2546,7 +2522,7 @@
       </c>
       <c r="R27" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context).</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -2578,11 +2554,11 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G28" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H28" s="5">
         <f>IF(G28="","",TODAY()-G28)</f>
@@ -2590,12 +2566,10 @@
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J28" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J28" s="6" t="n"/>
       <c r="K28" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -2621,7 +2595,7 @@
       </c>
       <c r="R28" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales - Solutions Consultant role at Earnix</t>
+          <t>Hook: Saw your Presales - Solutions Consultant role at Earnix 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -2653,11 +2627,11 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G29" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H29" s="5">
         <f>IF(G29="","",TODAY()-G29)</f>
@@ -2665,12 +2639,10 @@
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J29" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J29" s="6" t="n"/>
       <c r="K29" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -2696,7 +2668,7 @@
       </c>
       <c r="R29" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Solutions Consultant role at ORO Labs</t>
+          <t>Hook: Saw your Solutions Consultant role at ORO Labs 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -2728,11 +2700,11 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G30" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H30" s="5">
         <f>IF(G30="","",TODAY()-G30)</f>
@@ -2740,12 +2712,10 @@
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J30" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J30" s="6" t="n"/>
       <c r="K30" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -2771,7 +2741,7 @@
       </c>
       <c r="R30" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales and Solutions Consultant role at Aspire Systems</t>
+          <t>Hook: Saw your Presales and Solutions Consultant role at Aspire Systems 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -2803,11 +2773,11 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G31" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H31" s="5">
         <f>IF(G31="","",TODAY()-G31)</f>
@@ -2815,12 +2785,10 @@
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J31" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J31" s="6" t="n"/>
       <c r="K31" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -2846,7 +2814,7 @@
       </c>
       <c r="R31" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales &amp; Solutions Consultant role at Columbus</t>
+          <t>Hook: Saw your Presales &amp; Solutions Consultant role at Columbus 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -2955,11 +2923,11 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G33" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H33" s="5">
         <f>IF(G33="","",TODAY()-G33)</f>
@@ -2967,12 +2935,10 @@
       </c>
       <c r="I33" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J33" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="n"/>
       <c r="K33" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -2998,7 +2964,7 @@
       </c>
       <c r="R33" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales &amp; Solutions Consultant role at Tata Consultancy Services</t>
+          <t>Hook: Saw your Presales &amp; Solutions Consultant role at Tata Consultancy Services 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -3030,11 +2996,11 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G34" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H34" s="5">
         <f>IF(G34="","",TODAY()-G34)</f>
@@ -3042,12 +3008,10 @@
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J34" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J34" s="6" t="n"/>
       <c r="K34" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -3073,7 +3037,7 @@
       </c>
       <c r="R34" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales Solutions Consultant, Bid Manager role at Orange Cyberdefense</t>
+          <t>Hook: Saw your Presales Solutions Consultant, Bid Manager role at Orange Cyberdefense 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -3105,11 +3069,11 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G35" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H35" s="5">
         <f>IF(G35="","",TODAY()-G35)</f>
@@ -3117,12 +3081,10 @@
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J35" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J35" s="6" t="n"/>
       <c r="K35" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -3148,7 +3110,7 @@
       </c>
       <c r="R35" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Account Executive Sales Manager role at Haiilo</t>
+          <t>Hook: Saw your Account Executive Sales Manager role at Haiilo 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -3180,11 +3142,11 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G36" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H36" s="5">
         <f>IF(G36="","",TODAY()-G36)</f>
@@ -3192,12 +3154,10 @@
       </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J36" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J36" s="6" t="n"/>
       <c r="K36" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -3223,7 +3183,7 @@
       </c>
       <c r="R36" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Account Executive / Sales Manager role at Storyly</t>
+          <t>Hook: Saw your Account Executive / Sales Manager role at Storyly 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -3255,11 +3215,11 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G37" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H37" s="5">
         <f>IF(G37="","",TODAY()-G37)</f>
@@ -3267,12 +3227,10 @@
       </c>
       <c r="I37" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J37" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J37" s="6" t="n"/>
       <c r="K37" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -3298,7 +3256,7 @@
       </c>
       <c r="R37" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Account Executive Sales Manager role at TRUE LABS</t>
+          <t>Hook: Saw your Account Executive Sales Manager role at TRUE LABS 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -3330,11 +3288,11 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G38" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H38" s="5">
         <f>IF(G38="","",TODAY()-G38)</f>
@@ -3342,12 +3300,10 @@
       </c>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J38" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J38" s="6" t="n"/>
       <c r="K38" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -3373,7 +3329,7 @@
       </c>
       <c r="R38" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Account Executive &amp; Sales Manager role at Insure Smart Limited</t>
+          <t>Hook: Saw your Account Executive &amp; Sales Manager role at Insure Smart Limited 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -3405,11 +3361,11 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G39" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H39" s="5">
         <f>IF(G39="","",TODAY()-G39)</f>
@@ -3417,12 +3373,10 @@
       </c>
       <c r="I39" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J39" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J39" s="6" t="n"/>
       <c r="K39" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -3448,7 +3402,7 @@
       </c>
       <c r="R39" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager / Account Executive role at CybExer Technologies</t>
+          <t>Hook: Saw your Sales Manager / Account Executive role at CybExer Technologies 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -3480,11 +3434,11 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G40" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H40" s="5">
         <f>IF(G40="","",TODAY()-G40)</f>
@@ -3492,12 +3446,10 @@
       </c>
       <c r="I40" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J40" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J40" s="6" t="n"/>
       <c r="K40" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -3523,7 +3475,7 @@
       </c>
       <c r="R40" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales Consultant Manager role at V-Valley</t>
+          <t>Hook: Saw your Presales Consultant Manager role at V-Valley 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -3555,11 +3507,11 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G41" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H41" s="5">
         <f>IF(G41="","",TODAY()-G41)</f>
@@ -3567,12 +3519,10 @@
       </c>
       <c r="I41" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J41" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J41" s="6" t="n"/>
       <c r="K41" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -3598,7 +3548,7 @@
       </c>
       <c r="R41" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager, Account Executive role at Alconost</t>
+          <t>Hook: Saw your Sales Manager, Account Executive role at Alconost 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -3707,11 +3657,11 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G43" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H43" s="5">
         <f>IF(G43="","",TODAY()-G43)</f>
@@ -3719,12 +3669,10 @@
       </c>
       <c r="I43" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J43" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J43" s="6" t="n"/>
       <c r="K43" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -3750,7 +3698,7 @@
       </c>
       <c r="R43" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Senior Presales Consultant &amp; Solutions Consultant role at Hexadroit Pvt. Ltd.</t>
+          <t>Hook: Saw your Senior Presales Consultant &amp; Solutions Consultant role at Hexadroit Pvt. Ltd. 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -3859,11 +3807,11 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G45" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H45" s="5">
         <f>IF(G45="","",TODAY()-G45)</f>
@@ -3871,12 +3819,10 @@
       </c>
       <c r="I45" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J45" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J45" s="6" t="n"/>
       <c r="K45" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -3902,7 +3848,7 @@
       </c>
       <c r="R45" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Commercial Account Manager role at Boomi</t>
+          <t>Hook: Saw your Commercial Account Manager role at Boomi 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -3934,11 +3880,11 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G46" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H46" s="5">
         <f>IF(G46="","",TODAY()-G46)</f>
@@ -3946,12 +3892,10 @@
       </c>
       <c r="I46" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J46" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J46" s="6" t="n"/>
       <c r="K46" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -3977,7 +3921,7 @@
       </c>
       <c r="R46" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager / Account Executive role at yoummday</t>
+          <t>Hook: Saw your Sales Manager / Account Executive role at yoummday 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -4009,11 +3953,11 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G47" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H47" s="5">
         <f>IF(G47="","",TODAY()-G47)</f>
@@ -4021,12 +3965,10 @@
       </c>
       <c r="I47" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J47" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J47" s="6" t="n"/>
       <c r="K47" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -4052,7 +3994,7 @@
       </c>
       <c r="R47" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Account Executive / Enterprise Sales role at Neeyamo</t>
+          <t>Hook: Saw your Account Executive / Enterprise Sales role at Neeyamo 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -4230,11 +4172,11 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G50" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H50" s="5">
         <f>IF(G50="","",TODAY()-G50)</f>
@@ -4242,12 +4184,10 @@
       </c>
       <c r="I50" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J50" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J50" s="6" t="n"/>
       <c r="K50" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -4273,7 +4213,7 @@
       </c>
       <c r="R50" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager | Account Executive role at kununu</t>
+          <t>Hook: Saw your Sales Manager | Account Executive role at kununu 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -4305,11 +4245,11 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G51" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H51" s="5">
         <f>IF(G51="","",TODAY()-G51)</f>
@@ -4317,12 +4257,10 @@
       </c>
       <c r="I51" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J51" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J51" s="6" t="n"/>
       <c r="K51" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -4348,7 +4286,7 @@
       </c>
       <c r="R51" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager role at Dyad</t>
+          <t>Hook: Saw your Sales Manager role at Dyad 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -4380,11 +4318,11 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G52" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H52" s="5">
         <f>IF(G52="","",TODAY()-G52)</f>
@@ -4392,12 +4330,10 @@
       </c>
       <c r="I52" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J52" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J52" s="6" t="n"/>
       <c r="K52" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -4423,7 +4359,7 @@
       </c>
       <c r="R52" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Account Executive | Sales Manager role at Muck Rack</t>
+          <t>Hook: Saw your Account Executive | Sales Manager role at Muck Rack 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -4455,11 +4391,11 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G53" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H53" s="5">
         <f>IF(G53="","",TODAY()-G53)</f>
@@ -4467,12 +4403,10 @@
       </c>
       <c r="I53" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J53" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J53" s="6" t="n"/>
       <c r="K53" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -4498,7 +4432,7 @@
       </c>
       <c r="R53" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager - Account Executive role at Arivo</t>
+          <t>Hook: Saw your Sales Manager - Account Executive role at Arivo 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -4530,11 +4464,11 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G54" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H54" s="5">
         <f>IF(G54="","",TODAY()-G54)</f>
@@ -4542,12 +4476,10 @@
       </c>
       <c r="I54" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J54" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J54" s="6" t="n"/>
       <c r="K54" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -4573,7 +4505,7 @@
       </c>
       <c r="R54" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager - Account Executive role at UPTOO</t>
+          <t>Hook: Saw your Sales Manager - Account Executive role at UPTOO 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -4605,11 +4537,11 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G55" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H55" s="5">
         <f>IF(G55="","",TODAY()-G55)</f>
@@ -4617,12 +4549,10 @@
       </c>
       <c r="I55" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J55" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J55" s="6" t="n"/>
       <c r="K55" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -4648,7 +4578,7 @@
       </c>
       <c r="R55" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your SAP Partner Sales Manager &amp; Enterprise Account Executive role at EPI-USE Labs</t>
+          <t>Hook: Saw your SAP Partner Sales Manager &amp; Enterprise Account Executive role at EPI-USE Labs 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -4680,11 +4610,11 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G56" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H56" s="5">
         <f>IF(G56="","",TODAY()-G56)</f>
@@ -4692,12 +4622,10 @@
       </c>
       <c r="I56" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J56" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J56" s="6" t="n"/>
       <c r="K56" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -4723,7 +4651,7 @@
       </c>
       <c r="R56" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager &amp; Account Executive role at Dyad</t>
+          <t>Hook: Saw your Sales Manager &amp; Account Executive role at Dyad 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -4755,11 +4683,11 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G57" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H57" s="5">
         <f>IF(G57="","",TODAY()-G57)</f>
@@ -4767,12 +4695,10 @@
       </c>
       <c r="I57" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J57" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J57" s="6" t="n"/>
       <c r="K57" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -4798,7 +4724,7 @@
       </c>
       <c r="R57" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager / Account Executive role at Tellimer</t>
+          <t>Hook: Saw your Sales Manager / Account Executive role at Tellimer 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -4830,11 +4756,11 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G58" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H58" s="5">
         <f>IF(G58="","",TODAY()-G58)</f>
@@ -4842,12 +4768,10 @@
       </c>
       <c r="I58" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J58" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J58" s="6" t="n"/>
       <c r="K58" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -4873,7 +4797,7 @@
       </c>
       <c r="R58" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Enterprise Account Manager &amp; Sales Manager role at 42Gears</t>
+          <t>Hook: Saw your Enterprise Account Manager &amp; Sales Manager role at 42Gears 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -4905,11 +4829,11 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G59" s="6" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="H59" s="5">
         <f>IF(G59="","",TODAY()-G59)</f>
@@ -4917,12 +4841,10 @@
       </c>
       <c r="I59" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J59" s="6" t="n">
-        <v>46262</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J59" s="6" t="n"/>
       <c r="K59" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -4948,7 +4870,7 @@
       </c>
       <c r="R59" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Enterprise Sales Manager / Account Executive role at Anakin (YC S21)</t>
+          <t>Hook: Saw your Enterprise Sales Manager / Account Executive role at Anakin (YC S21) 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document multi-Apollo-account rotation and fix stale geography docs
Add a How To Use item explaining the two rotating free-tier Apollo.io
accounts (75 credits/month each) -- safe by design since dedup/exclusion
always reads from this Tracker sheet, never from either account's own
saved-contacts state. Also fixes item 5's stale 6-country list (still
said UAE/Malaysia/Thailand after the 8/22 narrowing) and the Region
item's outdated value list, and records the new 90/10 India-weighted
sourcing target agreed 2026-08-30 (the routine's own schedule config
still needs a matching manual edit -- not something this repo controls).
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -94,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -117,6 +117,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -8148,7 +8149,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -8195,70 +8196,77 @@
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>5. Lead sourcing (Monday only) targets 6 countries: India, United Arab Emirates (Dubai), Malaysia, Singapore, Thailand, and the United Kingdom. It also rotates through 3 audience segments on a 3-week cycle — Segment A: Presales &amp; Sales Professionals, Segment B: Freshers &amp; Early Career (0-2 yrs, any field), Segment C: SDR/BDR &amp; Delivery people breaking in — one segment per Monday, cycling automatically forever based on the ISO week number.</t>
+          <t>5. Lead sourcing (Monday only) targets 3 English-speaking countries as of 2026-08-22: India, Singapore, and the United Kingdom. As of 2026-08-30, sourcing is additionally weighted 90% India / 10% combined Singapore + United Kingdom (e.g. of a ~30-person target, aim for ~27 India and ~3 Singapore+UK; for Segment A, apply this 90/10 split within each sub-group's ~15 target too). It also rotates through 3 audience segments on a 3-week cycle — Segment A: Presales &amp; Sales Professionals, Segment B: Freshers &amp; Early Career (0-2 yrs, any field), Segment C: SDR/BDR &amp; Delivery people breaking in — one segment per Monday, cycling automatically forever based on the ISO week number.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>6. Next Action + Next Action Date tell you (or the automated routines) what to do and when.</t>
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>6. This team rotates between multiple free-tier Apollo.io accounts (each renews 75 free lead credits/month) since a paid plan hasn't been purchased yet -- whichever account currently has credits gets connected for that run. This is safe by design: duplicate/bounced/opted-out exclusion is always driven by this Tracker sheet (Email + LinkedIn URL match), never by any single Apollo account's own saved-contacts list, so switching accounts never risks a repeat send or a re-added exclusion regardless of which Apollo account sourced or enriched a lead.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>7. Days Since Contact calculates automatically from Last Contact Date — use it to spot who's overdue for a follow-up.</t>
+          <t>7. Next Action + Next Action Date tell you (or the automated routines) what to do and when.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>8. Region groups each contact by rough timezone (India / Gulf (UAE) / Southeast Asia / United Kingdom / Other / Unknown; "Europe" is a legacy value from before geography was narrowed, no longer assigned to new rows) — kept for your own visibility into what went out where. It does not control send timing.</t>
+          <t>8. Days Since Contact calculates automatically from Last Contact Date — use it to spot who's overdue for a follow-up.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="34" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>9. LinkedIn messages are generated as text for you but NOT sent automatically — there is no LinkedIn connector and LinkedIn's terms prohibit automated messaging, so you paste and send them yourself, then update Stage.</t>
+          <t>9. Region groups each contact by country (India / Singapore / United Kingdom / Other / Unknown; "Gulf (UAE)" and "Europe" are legacy values from before geography was narrowed, no longer assigned to new rows) -- kept for your own visibility into what went out where. It does not control send timing.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="34" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>10. Mark Booked = Y and fill Booking Date as soon as a booking confirmation arrives (email/SMS/WhatsApp) — booked contacts are excluded from further follow-ups.</t>
+          <t>10. LinkedIn messages are generated as text for you but NOT sent automatically — there is no LinkedIn connector and LinkedIn's terms prohibit automated messaging, so you paste and send them yourself, then update Stage.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="34" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>11. Mark Opted Out = Y and fill Opt-Out Date if someone asks to stop hearing from you (via the email unsubscribe link, a reply, or manually) — opted-out contacts are permanently excluded from all future emails, LinkedIn messages, and even from being re-added if Apollo surfaces them again later.</t>
+          <t>11. Mark Booked = Y and fill Booking Date as soon as a booking confirmation arrives (email/SMS/WhatsApp) — booked contacts are excluded from further follow-ups.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="34" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>12. Mark Bounced = Y and fill Bounce Date if you get a "Delivery Status Notification (Failure)" from Gmail for that contact — stop emailing that address, but it's fine to still try LinkedIn if you have their profile URL. The automation checks for these automatically each run.</t>
+          <t>12. Mark Opted Out = Y and fill Opt-Out Date if someone asks to stop hearing from you (via the email unsubscribe link, a reply, or manually) — opted-out contacts are permanently excluded from all future emails, LinkedIn messages, and even from being re-added if Apollo surfaces them again later.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="34" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>13. See email_templates.md / email_templates.html and linkedin_templates.md in this folder for the message sequence.</t>
+          <t>13. Mark Bounced = Y and fill Bounce Date if you get a "Delivery Status Notification (Failure)" from Gmail for that contact — stop emailing that address, but it's fine to still try LinkedIn if you have their profile URL. The automation checks for these automatically each run.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="34" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>14. "Apollo Archive" (third sheet) is a permanent historical log of every candidate Apollo has ever returned to the Monday routine — including duplicates and rejects that never made it into the active Tracker — with richer raw data (title, company, country) for your own future reference. It's a passive record only; it never drives outreach decisions or exclusions on its own.</t>
+          <t>14. See email_templates.md / email_templates.html and linkedin_templates.md in this folder for the message sequence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>15. "Apollo Archive" (third sheet) is a permanent historical log of every candidate Apollo has ever returned to the Monday routine — including duplicates and rejects that never made it into the active Tracker — with richer raw data (title, company, country) for your own future reference. It's a passive record only; it never drives outreach decisions or exclusions on its own.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document 0-7 years experience filter for Segment A1 Presales sourcing
Standing rule as of 2026-08-31: sub-group A1 (Presales) titles are now
additionally filtered to 0-7 years total professional experience. Applies
to A1 only, not A2 (Sales) or the other segments.
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -10811,7 +10811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -10865,77 +10865,84 @@
     <row r="8" ht="34" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>6. This team rotates between multiple free-tier Apollo.io accounts (each renews 75 free lead credits/month) since a paid plan hasn't been purchased yet -- whichever account currently has credits gets connected for that run. This is safe by design: duplicate/bounced/opted-out exclusion is always driven by this Tracker sheet (Email + LinkedIn URL match), never by any single Apollo account's own saved-contacts list, so switching accounts never risks a repeat send or a re-added exclusion regardless of which Apollo account sourced or enriched a lead.</t>
+          <t>6. As of 2026-08-31, Segment A sub-group A1 "Presales" is additionally filtered to 0-7 years of total professional experience -- this applies to Presales titles specifically, not sub-group A2 "Sales", and not the other segments (B, C) which have their own separate experience/tenure criteria already.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>7. If the connected Apollo.io account's prospecting/search API is plan-gated (a free trial can show available lead credits while still blocking apollo_agent_find_prospects with an API_INACCESSIBLE error -- this happened 2026-08-31), the fallback is manual sourcing: search Apollo's own web app by hand (its UI search still works on a trial plan even when the API doesn't), export results to a simple Name/Email/LinkedIn URL/Title/Company/Country spreadsheet, and hand it to the assistant to dedup, log to Apollo Archive, add to Tracker, and send from -- same exclusion rules apply regardless of how a candidate was sourced.</t>
+          <t>7. This team rotates between multiple free-tier Apollo.io accounts (each renews 75 free lead credits/month) since a paid plan hasn't been purchased yet -- whichever account currently has credits gets connected for that run. This is safe by design: duplicate/bounced/opted-out exclusion is always driven by this Tracker sheet (Email + LinkedIn URL match), never by any single Apollo account's own saved-contacts list, so switching accounts never risks a repeat send or a re-added exclusion regardless of which Apollo account sourced or enriched a lead.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>8. Next Action + Next Action Date tell you (or the automated routines) what to do and when.</t>
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>8. If the connected Apollo.io account's prospecting/search API is plan-gated (a free trial can show available lead credits while still blocking apollo_agent_find_prospects with an API_INACCESSIBLE error -- this happened 2026-08-31), the fallback is manual sourcing: search Apollo's own web app by hand (its UI search still works on a trial plan even when the API doesn't), export results to a simple Name/Email/LinkedIn URL/Title/Company/Country spreadsheet, and hand it to the assistant to dedup, log to Apollo Archive, add to Tracker, and send from -- same exclusion rules apply regardless of how a candidate was sourced.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="34" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>9. Days Since Contact calculates automatically from Last Contact Date — use it to spot who's overdue for a follow-up.</t>
+          <t>9. Next Action + Next Action Date tell you (or the automated routines) what to do and when.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="34" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>10. Region groups each contact by country (India / Singapore / United Kingdom / Other / Unknown; "Gulf (UAE)" and "Europe" are legacy values from before geography was narrowed, no longer assigned to new rows) -- kept for your own visibility into what went out where. It does not control send timing.</t>
+          <t>10. Days Since Contact calculates automatically from Last Contact Date — use it to spot who's overdue for a follow-up.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="34" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>11. LinkedIn messages are generated as text for you but NOT sent automatically — there is no LinkedIn connector and LinkedIn's terms prohibit automated messaging, so you paste and send them yourself, then update Stage.</t>
+          <t>11. Region groups each contact by country (India / Singapore / United Kingdom / Other / Unknown; "Gulf (UAE)" and "Europe" are legacy values from before geography was narrowed, no longer assigned to new rows) -- kept for your own visibility into what went out where. It does not control send timing.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="34" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>12. Mark Booked = Y and fill Booking Date as soon as a booking confirmation arrives (email/SMS/WhatsApp) — booked contacts are excluded from further follow-ups.</t>
+          <t>12. LinkedIn messages are generated as text for you but NOT sent automatically — there is no LinkedIn connector and LinkedIn's terms prohibit automated messaging, so you paste and send them yourself, then update Stage.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="34" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>13. Mark Opted Out = Y and fill Opt-Out Date if someone asks to stop hearing from you (via the email unsubscribe link, a reply, or manually) — opted-out contacts are permanently excluded from all future emails, LinkedIn messages, and even from being re-added if Apollo surfaces them again later.</t>
+          <t>13. Mark Booked = Y and fill Booking Date as soon as a booking confirmation arrives (email/SMS/WhatsApp) — booked contacts are excluded from further follow-ups.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="34" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>14. Mark Bounced = Y and fill Bounce Date if you get a "Delivery Status Notification (Failure)" from Gmail for that contact — stop emailing that address, but it's fine to still try LinkedIn if you have their profile URL. The automation checks for these automatically each run.</t>
+          <t>14. Mark Opted Out = Y and fill Opt-Out Date if someone asks to stop hearing from you (via the email unsubscribe link, a reply, or manually) — opted-out contacts are permanently excluded from all future emails, LinkedIn messages, and even from being re-added if Apollo surfaces them again later.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>15. See email_templates.md / email_templates.html and linkedin_templates.md in this folder for the message sequence.</t>
+          <t>15. Mark Bounced = Y and fill Bounce Date if you get a "Delivery Status Notification (Failure)" from Gmail for that contact — stop emailing that address, but it's fine to still try LinkedIn if you have their profile URL. The automation checks for these automatically each run.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>16. "Apollo Archive" (third sheet) is a permanent historical log of every candidate Apollo has ever returned to the Monday routine — including duplicates and rejects that never made it into the active Tracker — with richer raw data (title, company, country) for your own future reference. It's a passive record only; it never drives outreach decisions or exclusions on its own.</t>
+          <t>16. See email_templates.md / email_templates.html and linkedin_templates.md in this folder for the message sequence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>17. "Apollo Archive" (third sheet) is a permanent historical log of every candidate Apollo has ever returned to the Monday routine — including duplicates and rejects that never made it into the active Tracker — with richer raw data (title, company, country) for your own future reference. It's a passive record only; it never drives outreach decisions or exclusions on its own.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wednesday follow-up run: send Follow-up 1 to 37 due contacts
Sent Follow-up 1 to 37 contacts on the Email 1 -> Follow-up 1 cadence
(Stage=Email 1 Sent, Next Action Date<=2026-09-02), threaded via Gmail
reply into their original Email 1 sent 2026-08-31. Excluded the
permanent Jane Doe example row per standing rule.

Also processed 8 bounces detected via mailer-daemon Delivery Status
Notifications since Monday's manual catch-up send (all Accenture/
SplashBI addresses, "Address not found") - marked Bounced=Y with
today's date and reason noted; left Stage/Next Action untouched since
all 8 have a LinkedIn URL on file for manual fallback outreach.

No opt-outs or bookings matched tracker contacts this run.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GKWSm7onrKK1J1o7oc7Sjb
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -4903,11 +4903,11 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G60" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H60" s="5">
         <f>IF(G60="","",TODAY()-G60)</f>
@@ -4915,11 +4915,11 @@
       </c>
       <c r="I60" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J60" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K60" s="5" t="inlineStr">
         <is>
@@ -4978,11 +4978,11 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G61" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H61" s="5">
         <f>IF(G61="","",TODAY()-G61)</f>
@@ -4990,11 +4990,11 @@
       </c>
       <c r="I61" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J61" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K61" s="5" t="inlineStr">
         <is>
@@ -5053,11 +5053,11 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G62" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H62" s="5">
         <f>IF(G62="","",TODAY()-G62)</f>
@@ -5065,11 +5065,11 @@
       </c>
       <c r="I62" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J62" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K62" s="5" t="inlineStr">
         <is>
@@ -5128,11 +5128,11 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G63" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H63" s="5">
         <f>IF(G63="","",TODAY()-G63)</f>
@@ -5140,11 +5140,11 @@
       </c>
       <c r="I63" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J63" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K63" s="5" t="inlineStr">
         <is>
@@ -5203,11 +5203,11 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G64" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H64" s="5">
         <f>IF(G64="","",TODAY()-G64)</f>
@@ -5215,11 +5215,11 @@
       </c>
       <c r="I64" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J64" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K64" s="5" t="inlineStr">
         <is>
@@ -5278,11 +5278,11 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G65" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H65" s="5">
         <f>IF(G65="","",TODAY()-G65)</f>
@@ -5290,11 +5290,11 @@
       </c>
       <c r="I65" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J65" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K65" s="5" t="inlineStr">
         <is>
@@ -5422,11 +5422,11 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G67" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H67" s="5">
         <f>IF(G67="","",TODAY()-G67)</f>
@@ -5434,11 +5434,11 @@
       </c>
       <c r="I67" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J67" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K67" s="5" t="inlineStr">
         <is>
@@ -5497,11 +5497,11 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G68" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H68" s="5">
         <f>IF(G68="","",TODAY()-G68)</f>
@@ -5509,11 +5509,11 @@
       </c>
       <c r="I68" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J68" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K68" s="5" t="inlineStr">
         <is>
@@ -5572,11 +5572,11 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G69" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H69" s="5">
         <f>IF(G69="","",TODAY()-G69)</f>
@@ -5584,11 +5584,11 @@
       </c>
       <c r="I69" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J69" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K69" s="5" t="inlineStr">
         <is>
@@ -5647,11 +5647,11 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G70" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H70" s="5">
         <f>IF(G70="","",TODAY()-G70)</f>
@@ -5659,11 +5659,11 @@
       </c>
       <c r="I70" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J70" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K70" s="5" t="inlineStr">
         <is>
@@ -5722,11 +5722,11 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G71" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H71" s="5">
         <f>IF(G71="","",TODAY()-G71)</f>
@@ -5734,11 +5734,11 @@
       </c>
       <c r="I71" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J71" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K71" s="5" t="inlineStr">
         <is>
@@ -5797,11 +5797,11 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G72" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H72" s="5">
         <f>IF(G72="","",TODAY()-G72)</f>
@@ -5809,11 +5809,11 @@
       </c>
       <c r="I72" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J72" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K72" s="5" t="inlineStr">
         <is>
@@ -5872,11 +5872,11 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G73" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H73" s="5">
         <f>IF(G73="","",TODAY()-G73)</f>
@@ -5884,11 +5884,11 @@
       </c>
       <c r="I73" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J73" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K73" s="5" t="inlineStr">
         <is>
@@ -5947,11 +5947,11 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G74" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H74" s="5">
         <f>IF(G74="","",TODAY()-G74)</f>
@@ -5959,11 +5959,11 @@
       </c>
       <c r="I74" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J74" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K74" s="5" t="inlineStr">
         <is>
@@ -6091,11 +6091,11 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G76" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H76" s="5">
         <f>IF(G76="","",TODAY()-G76)</f>
@@ -6103,11 +6103,11 @@
       </c>
       <c r="I76" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J76" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K76" s="5" t="inlineStr">
         <is>
@@ -6166,11 +6166,11 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G77" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H77" s="5">
         <f>IF(G77="","",TODAY()-G77)</f>
@@ -6178,11 +6178,11 @@
       </c>
       <c r="I77" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J77" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K77" s="5" t="inlineStr">
         <is>
@@ -6310,11 +6310,11 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G79" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H79" s="5">
         <f>IF(G79="","",TODAY()-G79)</f>
@@ -6322,11 +6322,11 @@
       </c>
       <c r="I79" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J79" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K79" s="5" t="inlineStr">
         <is>
@@ -6385,11 +6385,11 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G80" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H80" s="5">
         <f>IF(G80="","",TODAY()-G80)</f>
@@ -6397,11 +6397,11 @@
       </c>
       <c r="I80" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J80" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K80" s="5" t="inlineStr">
         <is>
@@ -6630,10 +6630,12 @@
       <c r="N83" s="6" t="n"/>
       <c r="O83" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="P83" s="6" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P83" s="6" t="n">
+        <v>46267</v>
+      </c>
       <c r="Q83" s="5" t="inlineStr">
         <is>
           <t>India</t>
@@ -6641,7 +6643,7 @@
       </c>
       <c r="R83" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Lead Delivery Consultant role at SplashBI | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Lead Delivery Consultant role at SplashBI | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | Bounced 2026-09-02: Follow-up 1 send failed - "Address not found" (mailer-daemon). Has LinkedIn URL, left Stage/Next Action as-is for manual LinkedIn fallback.</t>
         </is>
       </c>
     </row>
@@ -6742,11 +6744,11 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G85" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H85" s="5">
         <f>IF(G85="","",TODAY()-G85)</f>
@@ -6754,11 +6756,11 @@
       </c>
       <c r="I85" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J85" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K85" s="5" t="inlineStr">
         <is>
@@ -6886,11 +6888,11 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G87" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H87" s="5">
         <f>IF(G87="","",TODAY()-G87)</f>
@@ -6898,11 +6900,11 @@
       </c>
       <c r="I87" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J87" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K87" s="5" t="inlineStr">
         <is>
@@ -6961,11 +6963,11 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G88" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H88" s="5">
         <f>IF(G88="","",TODAY()-G88)</f>
@@ -6973,11 +6975,11 @@
       </c>
       <c r="I88" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J88" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K88" s="5" t="inlineStr">
         <is>
@@ -7036,11 +7038,11 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G89" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H89" s="5">
         <f>IF(G89="","",TODAY()-G89)</f>
@@ -7048,11 +7050,11 @@
       </c>
       <c r="I89" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J89" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K89" s="5" t="inlineStr">
         <is>
@@ -7111,11 +7113,11 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G90" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H90" s="5">
         <f>IF(G90="","",TODAY()-G90)</f>
@@ -7123,11 +7125,11 @@
       </c>
       <c r="I90" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J90" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K90" s="5" t="inlineStr">
         <is>
@@ -7218,10 +7220,12 @@
       <c r="N91" s="6" t="n"/>
       <c r="O91" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="P91" s="6" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P91" s="6" t="n">
+        <v>46267</v>
+      </c>
       <c r="Q91" s="5" t="inlineStr">
         <is>
           <t>India</t>
@@ -7229,7 +7233,7 @@
       </c>
       <c r="R91" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | Bounced 2026-09-02: Follow-up 1 send failed - "Address not found" (mailer-daemon). Has LinkedIn URL, left Stage/Next Action as-is for manual LinkedIn fallback.</t>
         </is>
       </c>
     </row>
@@ -7261,11 +7265,11 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G92" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H92" s="5">
         <f>IF(G92="","",TODAY()-G92)</f>
@@ -7273,11 +7277,11 @@
       </c>
       <c r="I92" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J92" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K92" s="5" t="inlineStr">
         <is>
@@ -7368,10 +7372,12 @@
       <c r="N93" s="6" t="n"/>
       <c r="O93" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="P93" s="6" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P93" s="6" t="n">
+        <v>46267</v>
+      </c>
       <c r="Q93" s="5" t="inlineStr">
         <is>
           <t>India</t>
@@ -7379,7 +7385,7 @@
       </c>
       <c r="R93" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | Bounced 2026-09-02: Follow-up 1 send failed - "Address not found" (mailer-daemon). Has LinkedIn URL, left Stage/Next Action as-is for manual LinkedIn fallback.</t>
         </is>
       </c>
     </row>
@@ -7411,11 +7417,11 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G94" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H94" s="5">
         <f>IF(G94="","",TODAY()-G94)</f>
@@ -7423,11 +7429,11 @@
       </c>
       <c r="I94" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J94" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K94" s="5" t="inlineStr">
         <is>
@@ -7486,11 +7492,11 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G95" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H95" s="5">
         <f>IF(G95="","",TODAY()-G95)</f>
@@ -7498,11 +7504,11 @@
       </c>
       <c r="I95" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J95" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K95" s="5" t="inlineStr">
         <is>
@@ -7561,11 +7567,11 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G96" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H96" s="5">
         <f>IF(G96="","",TODAY()-G96)</f>
@@ -7573,11 +7579,11 @@
       </c>
       <c r="I96" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J96" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K96" s="5" t="inlineStr">
         <is>
@@ -7636,11 +7642,11 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G97" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H97" s="5">
         <f>IF(G97="","",TODAY()-G97)</f>
@@ -7648,11 +7654,11 @@
       </c>
       <c r="I97" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J97" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K97" s="5" t="inlineStr">
         <is>
@@ -7711,11 +7717,11 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G98" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H98" s="5">
         <f>IF(G98="","",TODAY()-G98)</f>
@@ -7723,11 +7729,11 @@
       </c>
       <c r="I98" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J98" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K98" s="5" t="inlineStr">
         <is>
@@ -7786,11 +7792,11 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G99" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H99" s="5">
         <f>IF(G99="","",TODAY()-G99)</f>
@@ -7798,11 +7804,11 @@
       </c>
       <c r="I99" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J99" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K99" s="5" t="inlineStr">
         <is>
@@ -7893,10 +7899,12 @@
       <c r="N100" s="6" t="n"/>
       <c r="O100" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="P100" s="6" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P100" s="6" t="n">
+        <v>46267</v>
+      </c>
       <c r="Q100" s="5" t="inlineStr">
         <is>
           <t>India</t>
@@ -7904,7 +7912,7 @@
       </c>
       <c r="R100" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | Bounced 2026-09-02: Follow-up 1 send failed - "Address not found" (mailer-daemon). Has LinkedIn URL, left Stage/Next Action as-is for manual LinkedIn fallback.</t>
         </is>
       </c>
     </row>
@@ -7936,11 +7944,11 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G101" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H101" s="5">
         <f>IF(G101="","",TODAY()-G101)</f>
@@ -7948,11 +7956,11 @@
       </c>
       <c r="I101" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J101" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K101" s="5" t="inlineStr">
         <is>
@@ -8043,10 +8051,12 @@
       <c r="N102" s="6" t="n"/>
       <c r="O102" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="P102" s="6" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P102" s="6" t="n">
+        <v>46267</v>
+      </c>
       <c r="Q102" s="5" t="inlineStr">
         <is>
           <t>India</t>
@@ -8054,7 +8064,7 @@
       </c>
       <c r="R102" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | Bounced 2026-09-02: Follow-up 1 send failed - "Address not found" (mailer-daemon). Has LinkedIn URL, left Stage/Next Action as-is for manual LinkedIn fallback.</t>
         </is>
       </c>
     </row>
@@ -8118,10 +8128,12 @@
       <c r="N103" s="6" t="n"/>
       <c r="O103" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="P103" s="6" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P103" s="6" t="n">
+        <v>46267</v>
+      </c>
       <c r="Q103" s="5" t="inlineStr">
         <is>
           <t>India</t>
@@ -8129,7 +8141,7 @@
       </c>
       <c r="R103" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Lead Consultant - Project role at Globant | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Lead Consultant - Project role at Globant | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | Bounced 2026-09-02: Follow-up 1 send failed - "Address not found" (mailer-daemon). Has LinkedIn URL, left Stage/Next Action as-is for manual LinkedIn fallback.</t>
         </is>
       </c>
     </row>
@@ -8161,11 +8173,11 @@
       </c>
       <c r="F104" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G104" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H104" s="5">
         <f>IF(G104="","",TODAY()-G104)</f>
@@ -8173,11 +8185,11 @@
       </c>
       <c r="I104" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J104" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K104" s="5" t="inlineStr">
         <is>
@@ -8236,11 +8248,11 @@
       </c>
       <c r="F105" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G105" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H105" s="5">
         <f>IF(G105="","",TODAY()-G105)</f>
@@ -8248,11 +8260,11 @@
       </c>
       <c r="I105" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J105" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K105" s="5" t="inlineStr">
         <is>
@@ -8343,10 +8355,12 @@
       <c r="N106" s="6" t="n"/>
       <c r="O106" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="P106" s="6" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P106" s="6" t="n">
+        <v>46267</v>
+      </c>
       <c r="Q106" s="5" t="inlineStr">
         <is>
           <t>India</t>
@@ -8354,7 +8368,7 @@
       </c>
       <c r="R106" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | Bounced 2026-09-02: Follow-up 1 send failed - "Address not found" (mailer-daemon). Has LinkedIn URL, left Stage/Next Action as-is for manual LinkedIn fallback.</t>
         </is>
       </c>
     </row>
@@ -8418,10 +8432,12 @@
       <c r="N107" s="6" t="n"/>
       <c r="O107" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="P107" s="6" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P107" s="6" t="n">
+        <v>46267</v>
+      </c>
       <c r="Q107" s="5" t="inlineStr">
         <is>
           <t>India</t>
@@ -8429,7 +8445,7 @@
       </c>
       <c r="R107" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | Bounced 2026-09-02: Follow-up 1 send failed - "Address not found" (mailer-daemon). Has LinkedIn URL, left Stage/Next Action as-is for manual LinkedIn fallback.</t>
         </is>
       </c>
     </row>
@@ -8461,11 +8477,11 @@
       </c>
       <c r="F108" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G108" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H108" s="5">
         <f>IF(G108="","",TODAY()-G108)</f>
@@ -8473,11 +8489,11 @@
       </c>
       <c r="I108" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J108" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K108" s="5" t="inlineStr">
         <is>
@@ -8536,11 +8552,11 @@
       </c>
       <c r="F109" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G109" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H109" s="5">
         <f>IF(G109="","",TODAY()-G109)</f>
@@ -8548,11 +8564,11 @@
       </c>
       <c r="I109" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J109" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K109" s="5" t="inlineStr">
         <is>
@@ -8611,11 +8627,11 @@
       </c>
       <c r="F110" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G110" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H110" s="5">
         <f>IF(G110="","",TODAY()-G110)</f>
@@ -8623,11 +8639,11 @@
       </c>
       <c r="I110" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J110" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K110" s="5" t="inlineStr">
         <is>
@@ -8686,11 +8702,11 @@
       </c>
       <c r="F111" s="5" t="inlineStr">
         <is>
-          <t>Email 1 Sent</t>
+          <t>Follow-up 1 Sent</t>
         </is>
       </c>
       <c r="G111" s="6" t="n">
-        <v>46265</v>
+        <v>46267</v>
       </c>
       <c r="H111" s="5">
         <f>IF(G111="","",TODAY()-G111)</f>
@@ -8698,11 +8714,11 @@
       </c>
       <c r="I111" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 1</t>
+          <t>Send Follow-up 2</t>
         </is>
       </c>
       <c r="J111" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="K111" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Friday follow-up run: send Follow-up 2 to 37 due contacts
No bounces, opt-outs, or bookings detected since Wednesday's run.
No rows were due for Follow-up 4 (no Follow-up 3 Sent stage yet).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rq3qqZtZSVYxsKwvtj3Juu
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -4903,11 +4903,11 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G60" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H60" s="5">
         <f>IF(G60="","",TODAY()-G60)</f>
@@ -4915,11 +4915,11 @@
       </c>
       <c r="I60" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J60" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K60" s="5" t="inlineStr">
         <is>
@@ -4978,11 +4978,11 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G61" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H61" s="5">
         <f>IF(G61="","",TODAY()-G61)</f>
@@ -4990,11 +4990,11 @@
       </c>
       <c r="I61" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J61" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K61" s="5" t="inlineStr">
         <is>
@@ -5053,11 +5053,11 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G62" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H62" s="5">
         <f>IF(G62="","",TODAY()-G62)</f>
@@ -5065,11 +5065,11 @@
       </c>
       <c r="I62" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J62" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K62" s="5" t="inlineStr">
         <is>
@@ -5128,11 +5128,11 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G63" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H63" s="5">
         <f>IF(G63="","",TODAY()-G63)</f>
@@ -5140,11 +5140,11 @@
       </c>
       <c r="I63" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J63" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K63" s="5" t="inlineStr">
         <is>
@@ -5203,11 +5203,11 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G64" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H64" s="5">
         <f>IF(G64="","",TODAY()-G64)</f>
@@ -5215,11 +5215,11 @@
       </c>
       <c r="I64" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J64" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K64" s="5" t="inlineStr">
         <is>
@@ -5278,11 +5278,11 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G65" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H65" s="5">
         <f>IF(G65="","",TODAY()-G65)</f>
@@ -5290,11 +5290,11 @@
       </c>
       <c r="I65" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J65" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K65" s="5" t="inlineStr">
         <is>
@@ -5422,11 +5422,11 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G67" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H67" s="5">
         <f>IF(G67="","",TODAY()-G67)</f>
@@ -5434,11 +5434,11 @@
       </c>
       <c r="I67" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J67" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K67" s="5" t="inlineStr">
         <is>
@@ -5497,11 +5497,11 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G68" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H68" s="5">
         <f>IF(G68="","",TODAY()-G68)</f>
@@ -5509,11 +5509,11 @@
       </c>
       <c r="I68" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J68" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K68" s="5" t="inlineStr">
         <is>
@@ -5572,11 +5572,11 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G69" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H69" s="5">
         <f>IF(G69="","",TODAY()-G69)</f>
@@ -5584,11 +5584,11 @@
       </c>
       <c r="I69" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J69" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K69" s="5" t="inlineStr">
         <is>
@@ -5647,11 +5647,11 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G70" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H70" s="5">
         <f>IF(G70="","",TODAY()-G70)</f>
@@ -5659,11 +5659,11 @@
       </c>
       <c r="I70" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J70" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K70" s="5" t="inlineStr">
         <is>
@@ -5722,11 +5722,11 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G71" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H71" s="5">
         <f>IF(G71="","",TODAY()-G71)</f>
@@ -5734,11 +5734,11 @@
       </c>
       <c r="I71" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J71" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K71" s="5" t="inlineStr">
         <is>
@@ -5797,11 +5797,11 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G72" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H72" s="5">
         <f>IF(G72="","",TODAY()-G72)</f>
@@ -5809,11 +5809,11 @@
       </c>
       <c r="I72" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J72" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K72" s="5" t="inlineStr">
         <is>
@@ -5872,11 +5872,11 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G73" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H73" s="5">
         <f>IF(G73="","",TODAY()-G73)</f>
@@ -5884,11 +5884,11 @@
       </c>
       <c r="I73" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J73" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K73" s="5" t="inlineStr">
         <is>
@@ -5947,11 +5947,11 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G74" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H74" s="5">
         <f>IF(G74="","",TODAY()-G74)</f>
@@ -5959,11 +5959,11 @@
       </c>
       <c r="I74" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J74" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K74" s="5" t="inlineStr">
         <is>
@@ -6091,11 +6091,11 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G76" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H76" s="5">
         <f>IF(G76="","",TODAY()-G76)</f>
@@ -6103,11 +6103,11 @@
       </c>
       <c r="I76" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J76" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K76" s="5" t="inlineStr">
         <is>
@@ -6166,11 +6166,11 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G77" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H77" s="5">
         <f>IF(G77="","",TODAY()-G77)</f>
@@ -6178,11 +6178,11 @@
       </c>
       <c r="I77" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J77" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K77" s="5" t="inlineStr">
         <is>
@@ -6310,11 +6310,11 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G79" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H79" s="5">
         <f>IF(G79="","",TODAY()-G79)</f>
@@ -6322,11 +6322,11 @@
       </c>
       <c r="I79" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J79" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K79" s="5" t="inlineStr">
         <is>
@@ -6385,11 +6385,11 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G80" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H80" s="5">
         <f>IF(G80="","",TODAY()-G80)</f>
@@ -6397,11 +6397,11 @@
       </c>
       <c r="I80" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J80" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K80" s="5" t="inlineStr">
         <is>
@@ -6744,11 +6744,11 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G85" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H85" s="5">
         <f>IF(G85="","",TODAY()-G85)</f>
@@ -6756,11 +6756,11 @@
       </c>
       <c r="I85" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J85" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K85" s="5" t="inlineStr">
         <is>
@@ -6888,11 +6888,11 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G87" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H87" s="5">
         <f>IF(G87="","",TODAY()-G87)</f>
@@ -6900,11 +6900,11 @@
       </c>
       <c r="I87" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J87" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K87" s="5" t="inlineStr">
         <is>
@@ -6963,11 +6963,11 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G88" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H88" s="5">
         <f>IF(G88="","",TODAY()-G88)</f>
@@ -6975,11 +6975,11 @@
       </c>
       <c r="I88" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J88" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K88" s="5" t="inlineStr">
         <is>
@@ -7038,11 +7038,11 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G89" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H89" s="5">
         <f>IF(G89="","",TODAY()-G89)</f>
@@ -7050,11 +7050,11 @@
       </c>
       <c r="I89" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J89" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K89" s="5" t="inlineStr">
         <is>
@@ -7113,11 +7113,11 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G90" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H90" s="5">
         <f>IF(G90="","",TODAY()-G90)</f>
@@ -7125,11 +7125,11 @@
       </c>
       <c r="I90" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J90" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K90" s="5" t="inlineStr">
         <is>
@@ -7265,11 +7265,11 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G92" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H92" s="5">
         <f>IF(G92="","",TODAY()-G92)</f>
@@ -7277,11 +7277,11 @@
       </c>
       <c r="I92" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J92" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K92" s="5" t="inlineStr">
         <is>
@@ -7417,11 +7417,11 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G94" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H94" s="5">
         <f>IF(G94="","",TODAY()-G94)</f>
@@ -7429,11 +7429,11 @@
       </c>
       <c r="I94" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J94" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K94" s="5" t="inlineStr">
         <is>
@@ -7492,11 +7492,11 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G95" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H95" s="5">
         <f>IF(G95="","",TODAY()-G95)</f>
@@ -7504,11 +7504,11 @@
       </c>
       <c r="I95" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J95" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K95" s="5" t="inlineStr">
         <is>
@@ -7567,11 +7567,11 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G96" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H96" s="5">
         <f>IF(G96="","",TODAY()-G96)</f>
@@ -7579,11 +7579,11 @@
       </c>
       <c r="I96" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J96" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K96" s="5" t="inlineStr">
         <is>
@@ -7642,11 +7642,11 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G97" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H97" s="5">
         <f>IF(G97="","",TODAY()-G97)</f>
@@ -7654,11 +7654,11 @@
       </c>
       <c r="I97" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J97" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K97" s="5" t="inlineStr">
         <is>
@@ -7717,11 +7717,11 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G98" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H98" s="5">
         <f>IF(G98="","",TODAY()-G98)</f>
@@ -7729,11 +7729,11 @@
       </c>
       <c r="I98" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J98" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K98" s="5" t="inlineStr">
         <is>
@@ -7792,11 +7792,11 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G99" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H99" s="5">
         <f>IF(G99="","",TODAY()-G99)</f>
@@ -7804,11 +7804,11 @@
       </c>
       <c r="I99" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J99" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K99" s="5" t="inlineStr">
         <is>
@@ -7944,11 +7944,11 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G101" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H101" s="5">
         <f>IF(G101="","",TODAY()-G101)</f>
@@ -7956,11 +7956,11 @@
       </c>
       <c r="I101" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J101" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K101" s="5" t="inlineStr">
         <is>
@@ -8173,11 +8173,11 @@
       </c>
       <c r="F104" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G104" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H104" s="5">
         <f>IF(G104="","",TODAY()-G104)</f>
@@ -8185,11 +8185,11 @@
       </c>
       <c r="I104" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J104" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K104" s="5" t="inlineStr">
         <is>
@@ -8248,11 +8248,11 @@
       </c>
       <c r="F105" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G105" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H105" s="5">
         <f>IF(G105="","",TODAY()-G105)</f>
@@ -8260,11 +8260,11 @@
       </c>
       <c r="I105" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J105" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K105" s="5" t="inlineStr">
         <is>
@@ -8477,11 +8477,11 @@
       </c>
       <c r="F108" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G108" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H108" s="5">
         <f>IF(G108="","",TODAY()-G108)</f>
@@ -8489,11 +8489,11 @@
       </c>
       <c r="I108" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J108" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K108" s="5" t="inlineStr">
         <is>
@@ -8552,11 +8552,11 @@
       </c>
       <c r="F109" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G109" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H109" s="5">
         <f>IF(G109="","",TODAY()-G109)</f>
@@ -8564,11 +8564,11 @@
       </c>
       <c r="I109" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J109" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K109" s="5" t="inlineStr">
         <is>
@@ -8627,11 +8627,11 @@
       </c>
       <c r="F110" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G110" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H110" s="5">
         <f>IF(G110="","",TODAY()-G110)</f>
@@ -8639,11 +8639,11 @@
       </c>
       <c r="I110" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J110" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K110" s="5" t="inlineStr">
         <is>
@@ -8702,11 +8702,11 @@
       </c>
       <c r="F111" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 1 Sent</t>
+          <t>Follow-up 2 Sent</t>
         </is>
       </c>
       <c r="G111" s="6" t="n">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="H111" s="5">
         <f>IF(G111="","",TODAY()-G111)</f>
@@ -8714,11 +8714,11 @@
       </c>
       <c r="I111" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 2</t>
+          <t>Send Follow-up 3</t>
         </is>
       </c>
       <c r="J111" s="6" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="K111" s="5" t="inlineStr">
         <is>

</xml_diff>